<commit_message>
COCINA-01 rediseñada como el render: B4 bajo puerta (sin lavavajillas), cornisa, vitrinas, A2 rebatible, tiradores; receptor Ø5 y placa base 37/±16 desde medidas.json; ExportarPiezas ignora cajeados anchos; paquete regenerado (106/106)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,10 +413,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y96"/>
+  <dimension ref="A1:Y107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="4" customWidth="1" min="4" max="4"/>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>9992609290269</t>
+          <t>9992609290269_9992609290269</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>9992609290320</t>
+          <t>9992609290320_9992609290320</t>
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>9992609290382</t>
+          <t>9992609290382_9992609290382</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>9992609290443</t>
+          <t>9992609290443_9992609290443</t>
         </is>
       </c>
       <c r="O45" t="inlineStr"/>
@@ -5035,60 +5035,60 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>COCINA-01_P1 Panel lavavajillas_Panel terminal</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Lateral der</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COCINA-01_P1 Panel lavavajillas_Panel terminal</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Lateral der</t>
         </is>
       </c>
       <c r="D51" t="n">
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>860</v>
+        <v>760</v>
       </c>
       <c r="F51" t="n">
-        <v>598</v>
+        <v>580</v>
       </c>
       <c r="G51" t="n">
-        <v>0.51</v>
+        <v>0.44</v>
       </c>
       <c r="H51" t="n">
         <v>18</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>858</v>
+        <v>760</v>
       </c>
       <c r="K51" t="n">
-        <v>596</v>
+        <v>579</v>
       </c>
       <c r="L51" t="n">
-        <v>0.51</v>
+        <v>0.44</v>
       </c>
       <c r="M51" t="n">
         <v>18</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>9992609290504</t>
+          <t>9992609290504_9992609290504</t>
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S51" t="n">
         <v>1</v>
@@ -5111,7 +5111,7 @@
       <c r="W51" t="inlineStr"/>
       <c r="X51" t="inlineStr">
         <is>
-          <t>COCINA-01_P1 Panel lavavajillas_Panel terminal</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Lateral der</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
@@ -5126,63 +5126,63 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>COCINA-01_P2 Panel cocina_Panel terminal</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Lateral izq</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COCINA-01_P2 Panel cocina_Panel terminal</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Lateral izq</t>
         </is>
       </c>
       <c r="D52" t="n">
         <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>860</v>
+        <v>760</v>
       </c>
       <c r="F52" t="n">
-        <v>598</v>
+        <v>580</v>
       </c>
       <c r="G52" t="n">
-        <v>0.51</v>
+        <v>0.44</v>
       </c>
       <c r="H52" t="n">
         <v>18</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>858</v>
+        <v>760</v>
       </c>
       <c r="K52" t="n">
-        <v>596</v>
+        <v>579</v>
       </c>
       <c r="L52" t="n">
-        <v>0.51</v>
+        <v>0.44</v>
       </c>
       <c r="M52" t="n">
         <v>18</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>9992609290511</t>
+          <t>9992609290511_9992609290511</t>
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R52" t="n">
         <v>1</v>
       </c>
       <c r="S52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T52" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr">
         <is>
-          <t>COCINA-01_P2 Panel cocina_Panel terminal</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Lateral izq</t>
         </is>
       </c>
       <c r="Y52" t="inlineStr">
@@ -5217,25 +5217,25 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Lateral A</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Piso</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Lateral A</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Piso</t>
         </is>
       </c>
       <c r="D53" t="n">
         <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>980</v>
+        <v>580</v>
       </c>
       <c r="F53" t="n">
-        <v>332</v>
+        <v>416</v>
       </c>
       <c r="G53" t="n">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="H53" t="n">
         <v>18</v>
@@ -5246,20 +5246,20 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>980</v>
+        <v>579</v>
       </c>
       <c r="K53" t="n">
-        <v>331</v>
+        <v>416</v>
       </c>
       <c r="L53" t="n">
-        <v>0.32</v>
+        <v>0.24</v>
       </c>
       <c r="M53" t="n">
         <v>18</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>9992609290528_9992609290528</t>
+          <t>9992609290528_9992609290528_9992609290528K</t>
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
@@ -5267,10 +5267,10 @@
         <v>0</v>
       </c>
       <c r="Q53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S53" t="n">
         <v>0</v>
@@ -5293,7 +5293,7 @@
       <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Lateral A</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Piso</t>
         </is>
       </c>
       <c r="Y53" t="inlineStr">
@@ -5308,25 +5308,25 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Lateral B</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Travesano delantero</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Lateral B</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Travesano delantero</t>
         </is>
       </c>
       <c r="D54" t="n">
         <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>980</v>
+        <v>100</v>
       </c>
       <c r="F54" t="n">
-        <v>332</v>
+        <v>416</v>
       </c>
       <c r="G54" t="n">
-        <v>0.33</v>
+        <v>0.04</v>
       </c>
       <c r="H54" t="n">
         <v>18</v>
@@ -5337,13 +5337,13 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>980</v>
+        <v>99</v>
       </c>
       <c r="K54" t="n">
-        <v>331</v>
+        <v>416</v>
       </c>
       <c r="L54" t="n">
-        <v>0.32</v>
+        <v>0.04</v>
       </c>
       <c r="M54" t="n">
         <v>18</v>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q54" t="n">
         <v>0</v>
@@ -5364,7 +5364,7 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="W54" t="inlineStr"/>
       <c r="X54" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Lateral B</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Travesano delantero</t>
         </is>
       </c>
       <c r="Y54" t="inlineStr">
@@ -5399,25 +5399,25 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Piso</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Travesano trasero</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Piso</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Travesano trasero</t>
         </is>
       </c>
       <c r="D55" t="n">
         <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>782</v>
+        <v>100</v>
       </c>
       <c r="F55" t="n">
-        <v>782</v>
+        <v>416</v>
       </c>
       <c r="G55" t="n">
-        <v>0.61</v>
+        <v>0.04</v>
       </c>
       <c r="H55" t="n">
         <v>18</v>
@@ -5428,20 +5428,20 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>782</v>
+        <v>100</v>
       </c>
       <c r="K55" t="n">
-        <v>782</v>
+        <v>416</v>
       </c>
       <c r="L55" t="n">
-        <v>0.61</v>
+        <v>0.04</v>
       </c>
       <c r="M55" t="n">
         <v>18</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>9992609290542_9992609290542_9992609290542K</t>
+          <t>9992609290542_9992609290542</t>
         </is>
       </c>
       <c r="O55" t="inlineStr"/>
@@ -5475,7 +5475,7 @@
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Piso</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Travesano trasero</t>
         </is>
       </c>
       <c r="Y55" t="inlineStr">
@@ -5490,49 +5490,49 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Techo</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Fondo</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Techo</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Fondo</t>
         </is>
       </c>
       <c r="D56" t="n">
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>782</v>
+        <v>746</v>
       </c>
       <c r="F56" t="n">
-        <v>782</v>
+        <v>426</v>
       </c>
       <c r="G56" t="n">
-        <v>0.61</v>
+        <v>0.32</v>
       </c>
       <c r="H56" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>782</v>
+        <v>746</v>
       </c>
       <c r="K56" t="n">
-        <v>782</v>
+        <v>426</v>
       </c>
       <c r="L56" t="n">
-        <v>0.61</v>
+        <v>0.32</v>
       </c>
       <c r="M56" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>9992609290559_9992609290559</t>
+          <t>9992609290559</t>
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
@@ -5566,7 +5566,7 @@
       <c r="W56" t="inlineStr"/>
       <c r="X56" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Techo</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Fondo</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr">
@@ -5581,63 +5581,63 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Fondo A</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Puerta</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Fondo A</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Puerta</t>
         </is>
       </c>
       <c r="D57" t="n">
         <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>954</v>
+        <v>757</v>
       </c>
       <c r="F57" t="n">
+        <v>449</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H57" t="n">
+        <v>18</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
         <v>755</v>
       </c>
-      <c r="G57" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="H57" t="n">
-        <v>5</v>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>5_Melamina_BLANCO 5</t>
-        </is>
-      </c>
-      <c r="J57" t="n">
-        <v>954</v>
-      </c>
       <c r="K57" t="n">
-        <v>755</v>
+        <v>447</v>
       </c>
       <c r="L57" t="n">
-        <v>0.72</v>
+        <v>0.34</v>
       </c>
       <c r="M57" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>9992609290566</t>
+          <t>9992609290566_9992609290566</t>
         </is>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -5657,7 +5657,7 @@
       <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Fondo A</t>
+          <t>COCINA-01_B4 Bajo puerta 452_Puerta</t>
         </is>
       </c>
       <c r="Y57" t="inlineStr">
@@ -5672,45 +5672,45 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Fondo B</t>
+          <t>COCINA-01_P1 Panel terminal_Panel terminal</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Fondo B</t>
+          <t>COCINA-01_P1 Panel terminal_Panel terminal</t>
         </is>
       </c>
       <c r="D58" t="n">
         <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>954</v>
+        <v>860</v>
       </c>
       <c r="F58" t="n">
-        <v>762</v>
+        <v>598</v>
       </c>
       <c r="G58" t="n">
-        <v>0.73</v>
+        <v>0.51</v>
       </c>
       <c r="H58" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>954</v>
+        <v>858</v>
       </c>
       <c r="K58" t="n">
-        <v>762</v>
+        <v>596</v>
       </c>
       <c r="L58" t="n">
-        <v>0.73</v>
+        <v>0.51</v>
       </c>
       <c r="M58" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -5719,16 +5719,16 @@
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
       <c r="W58" t="inlineStr"/>
       <c r="X58" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Fondo B</t>
+          <t>COCINA-01_P1 Panel terminal_Panel terminal</t>
         </is>
       </c>
       <c r="Y58" t="inlineStr">
@@ -5763,63 +5763,63 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Montante A</t>
+          <t>COCINA-01_P2 Panel cocina_Panel terminal</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Montante A</t>
+          <t>COCINA-01_P2 Panel cocina_Panel terminal</t>
         </is>
       </c>
       <c r="D59" t="n">
         <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>944</v>
+        <v>860</v>
       </c>
       <c r="F59" t="n">
-        <v>80</v>
+        <v>598</v>
       </c>
       <c r="G59" t="n">
-        <v>0.08</v>
+        <v>0.51</v>
       </c>
       <c r="H59" t="n">
         <v>18</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>944</v>
+        <v>858</v>
       </c>
       <c r="K59" t="n">
-        <v>79</v>
+        <v>596</v>
       </c>
       <c r="L59" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="M59" t="n">
         <v>18</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>9992609290580_9992609290580</t>
+          <t>9992609290580</t>
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R59" t="n">
         <v>1</v>
       </c>
       <c r="S59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -5839,7 +5839,7 @@
       <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Montante A</t>
+          <t>COCINA-01_P2 Panel cocina_Panel terminal</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
@@ -5854,25 +5854,25 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Montante B</t>
+          <t>COCINA-01_A1 Esquinero alacena_Lateral A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Montante B</t>
+          <t>COCINA-01_A1 Esquinero alacena_Lateral A</t>
         </is>
       </c>
       <c r="D60" t="n">
         <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>944</v>
+        <v>920</v>
       </c>
       <c r="F60" t="n">
-        <v>80</v>
+        <v>332</v>
       </c>
       <c r="G60" t="n">
-        <v>0.08</v>
+        <v>0.31</v>
       </c>
       <c r="H60" t="n">
         <v>18</v>
@@ -5883,13 +5883,13 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>944</v>
+        <v>920</v>
       </c>
       <c r="K60" t="n">
-        <v>79</v>
+        <v>331</v>
       </c>
       <c r="L60" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.3</v>
       </c>
       <c r="M60" t="n">
         <v>18</v>
@@ -5907,10 +5907,10 @@
         <v>0</v>
       </c>
       <c r="R60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T60" t="inlineStr">
         <is>
@@ -5930,7 +5930,7 @@
       <c r="W60" t="inlineStr"/>
       <c r="X60" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Montante B</t>
+          <t>COCINA-01_A1 Esquinero alacena_Lateral A</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
@@ -5945,42 +5945,42 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
+          <t>COCINA-01_A1 Esquinero alacena_Lateral B</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
+          <t>COCINA-01_A1 Esquinero alacena_Lateral B</t>
         </is>
       </c>
       <c r="D61" t="n">
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>977</v>
+        <v>920</v>
       </c>
       <c r="F61" t="n">
-        <v>633.4</v>
+        <v>332</v>
       </c>
       <c r="G61" t="n">
-        <v>0.62</v>
+        <v>0.31</v>
       </c>
       <c r="H61" t="n">
         <v>18</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>975</v>
+        <v>920</v>
       </c>
       <c r="K61" t="n">
-        <v>631.4</v>
+        <v>331</v>
       </c>
       <c r="L61" t="n">
-        <v>0.62</v>
+        <v>0.3</v>
       </c>
       <c r="M61" t="n">
         <v>18</v>
@@ -5992,13 +5992,13 @@
       </c>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S61" t="n">
         <v>1</v>
@@ -6021,7 +6021,7 @@
       <c r="W61" t="inlineStr"/>
       <c r="X61" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
+          <t>COCINA-01_A1 Esquinero alacena_Lateral B</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
@@ -6036,25 +6036,25 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
+          <t>COCINA-01_A1 Esquinero alacena_Piso</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
+          <t>COCINA-01_A1 Esquinero alacena_Piso</t>
         </is>
       </c>
       <c r="D62" t="n">
         <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="F62" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="G62" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="H62" t="n">
         <v>18</v>
@@ -6065,20 +6065,20 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="K62" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="L62" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="M62" t="n">
         <v>18</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>9992609290610</t>
+          <t>9992609290610_9992609290610_9992609290610K</t>
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
@@ -6112,7 +6112,7 @@
       <c r="W62" t="inlineStr"/>
       <c r="X62" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
+          <t>COCINA-01_A1 Esquinero alacena_Piso</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr">
@@ -6127,25 +6127,25 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
+          <t>COCINA-01_A1 Esquinero alacena_Techo</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
+          <t>COCINA-01_A1 Esquinero alacena_Techo</t>
         </is>
       </c>
       <c r="D63" t="n">
         <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="F63" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="G63" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="H63" t="n">
         <v>18</v>
@@ -6156,20 +6156,20 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="K63" t="n">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="L63" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="M63" t="n">
         <v>18</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>9992609290627</t>
+          <t>9992609290627_9992609290627_9992609290627K</t>
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
@@ -6203,7 +6203,7 @@
       <c r="W63" t="inlineStr"/>
       <c r="X63" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
+          <t>COCINA-01_A1 Esquinero alacena_Techo</t>
         </is>
       </c>
       <c r="Y63" t="inlineStr">
@@ -6218,54 +6218,54 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Fondo A</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Fondo A</t>
         </is>
       </c>
       <c r="D64" t="n">
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>60</v>
+        <v>894</v>
       </c>
       <c r="F64" t="n">
-        <v>636.4</v>
+        <v>755</v>
       </c>
       <c r="G64" t="n">
-        <v>0.04</v>
+        <v>0.67</v>
       </c>
       <c r="H64" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>59</v>
+        <v>894</v>
       </c>
       <c r="K64" t="n">
-        <v>636.4</v>
+        <v>755</v>
       </c>
       <c r="L64" t="n">
-        <v>0.04</v>
+        <v>0.67</v>
       </c>
       <c r="M64" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>9992609290634_9992609290634</t>
+          <t>9992609290634</t>
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q64" t="n">
         <v>0</v>
@@ -6294,7 +6294,7 @@
       <c r="W64" t="inlineStr"/>
       <c r="X64" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Fondo A</t>
         </is>
       </c>
       <c r="Y64" t="inlineStr">
@@ -6309,49 +6309,49 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Piso</t>
+          <t>COCINA-01_A1 Esquinero alacena_Fondo B</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Piso</t>
+          <t>COCINA-01_A1 Esquinero alacena_Fondo B</t>
         </is>
       </c>
       <c r="D65" t="n">
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>332</v>
+        <v>894</v>
       </c>
       <c r="F65" t="n">
-        <v>600</v>
+        <v>762</v>
       </c>
       <c r="G65" t="n">
-        <v>0.2</v>
+        <v>0.68</v>
       </c>
       <c r="H65" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>331</v>
+        <v>894</v>
       </c>
       <c r="K65" t="n">
-        <v>600</v>
+        <v>762</v>
       </c>
       <c r="L65" t="n">
-        <v>0.2</v>
+        <v>0.68</v>
       </c>
       <c r="M65" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>9992609290641_9992609290641_9992609290641K</t>
+          <t>9992609290641</t>
         </is>
       </c>
       <c r="O65" t="inlineStr"/>
@@ -6359,7 +6359,7 @@
         <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R65" t="n">
         <v>0</v>
@@ -6385,7 +6385,7 @@
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Piso</t>
+          <t>COCINA-01_A1 Esquinero alacena_Fondo B</t>
         </is>
       </c>
       <c r="Y65" t="inlineStr">
@@ -6400,25 +6400,25 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Techo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Montante A</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Techo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Montante A</t>
         </is>
       </c>
       <c r="D66" t="n">
         <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>332</v>
+        <v>884</v>
       </c>
       <c r="F66" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="G66" t="n">
-        <v>0.2</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H66" t="n">
         <v>18</v>
@@ -6429,13 +6429,13 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>331</v>
+        <v>884</v>
       </c>
       <c r="K66" t="n">
-        <v>600</v>
+        <v>79</v>
       </c>
       <c r="L66" t="n">
-        <v>0.2</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M66" t="n">
         <v>18</v>
@@ -6447,13 +6447,13 @@
       </c>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q66" t="n">
         <v>0</v>
       </c>
       <c r="R66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S66" t="n">
         <v>0</v>
@@ -6476,7 +6476,7 @@
       <c r="W66" t="inlineStr"/>
       <c r="X66" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Techo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Montante A</t>
         </is>
       </c>
       <c r="Y66" t="inlineStr">
@@ -6491,25 +6491,25 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Lateral der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Montante B</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Lateral der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Montante B</t>
         </is>
       </c>
       <c r="D67" t="n">
         <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>944</v>
+        <v>884</v>
       </c>
       <c r="F67" t="n">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="G67" t="n">
-        <v>0.31</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H67" t="n">
         <v>18</v>
@@ -6520,13 +6520,13 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>944</v>
+        <v>884</v>
       </c>
       <c r="K67" t="n">
-        <v>331</v>
+        <v>79</v>
       </c>
       <c r="L67" t="n">
-        <v>0.31</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M67" t="n">
         <v>18</v>
@@ -6567,7 +6567,7 @@
       <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Lateral der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Montante B</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr">
@@ -6582,42 +6582,42 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Lateral izq</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Lateral izq</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
         </is>
       </c>
       <c r="D68" t="n">
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>944</v>
+        <v>917</v>
       </c>
       <c r="F68" t="n">
-        <v>332</v>
+        <v>633.4</v>
       </c>
       <c r="G68" t="n">
-        <v>0.31</v>
+        <v>0.58</v>
       </c>
       <c r="H68" t="n">
         <v>18</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>944</v>
+        <v>915</v>
       </c>
       <c r="K68" t="n">
-        <v>331</v>
+        <v>631.4</v>
       </c>
       <c r="L68" t="n">
-        <v>0.31</v>
+        <v>0.58</v>
       </c>
       <c r="M68" t="n">
         <v>18</v>
@@ -6629,16 +6629,16 @@
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R68" t="n">
         <v>1</v>
       </c>
       <c r="S68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T68" t="inlineStr">
         <is>
@@ -6658,7 +6658,7 @@
       <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Lateral izq</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
         </is>
       </c>
       <c r="Y68" t="inlineStr">
@@ -6673,45 +6673,45 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Fondo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Fondo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>954</v>
+        <v>750</v>
       </c>
       <c r="F69" t="n">
-        <v>574</v>
+        <v>750</v>
       </c>
       <c r="G69" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H69" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>954</v>
+        <v>750</v>
       </c>
       <c r="K69" t="n">
-        <v>574</v>
+        <v>750</v>
       </c>
       <c r="L69" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M69" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -6749,7 +6749,7 @@
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Fondo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr">
@@ -6764,63 +6764,63 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
         </is>
       </c>
       <c r="D70" t="n">
         <v>1</v>
       </c>
       <c r="E70" t="n">
-        <v>60</v>
+        <v>750</v>
       </c>
       <c r="F70" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="G70" t="n">
-        <v>0.04</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H70" t="n">
         <v>18</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>59</v>
+        <v>750</v>
       </c>
       <c r="K70" t="n">
-        <v>598</v>
+        <v>750</v>
       </c>
       <c r="L70" t="n">
-        <v>0.04</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M70" t="n">
         <v>18</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>9992609290696_9992609290696</t>
+          <t>9992609290696</t>
         </is>
       </c>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q70" t="n">
         <v>0</v>
       </c>
       <c r="R70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T70" t="inlineStr">
         <is>
@@ -6840,7 +6840,7 @@
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
         </is>
       </c>
       <c r="Y70" t="inlineStr">
@@ -6855,25 +6855,25 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Puerta der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Puerta der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
         </is>
       </c>
       <c r="D71" t="n">
         <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>977</v>
+        <v>60</v>
       </c>
       <c r="F71" t="n">
-        <v>297</v>
+        <v>636.4</v>
       </c>
       <c r="G71" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="H71" t="n">
         <v>18</v>
@@ -6884,13 +6884,13 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>975</v>
+        <v>59</v>
       </c>
       <c r="K71" t="n">
-        <v>295</v>
+        <v>636.4</v>
       </c>
       <c r="L71" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="M71" t="n">
         <v>18</v>
@@ -6905,13 +6905,13 @@
         <v>1</v>
       </c>
       <c r="Q71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T71" t="inlineStr">
         <is>
@@ -6931,7 +6931,7 @@
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Puerta der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
         </is>
       </c>
       <c r="Y71" t="inlineStr">
@@ -6946,25 +6946,25 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Puerta izq</t>
+          <t>COCINA-01_A1 Esquinero alacena_Cornisa</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Puerta izq</t>
+          <t>COCINA-01_A1 Esquinero alacena_Cornisa</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>977</v>
+        <v>60</v>
       </c>
       <c r="F72" t="n">
-        <v>297</v>
+        <v>636.4</v>
       </c>
       <c r="G72" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="H72" t="n">
         <v>18</v>
@@ -6975,13 +6975,13 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>975</v>
+        <v>59</v>
       </c>
       <c r="K72" t="n">
-        <v>295</v>
+        <v>636.4</v>
       </c>
       <c r="L72" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="M72" t="n">
         <v>18</v>
@@ -6993,16 +6993,16 @@
       </c>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q72" t="n">
         <v>1</v>
       </c>
       <c r="R72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T72" t="inlineStr">
         <is>
@@ -7022,7 +7022,7 @@
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Puerta izq</t>
+          <t>COCINA-01_A1 Esquinero alacena_Cornisa</t>
         </is>
       </c>
       <c r="Y72" t="inlineStr">
@@ -7037,25 +7037,25 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
         </is>
       </c>
       <c r="D73" t="n">
         <v>1</v>
       </c>
       <c r="E73" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F73" t="n">
-        <v>562</v>
+        <v>600</v>
       </c>
       <c r="G73" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="H73" t="n">
         <v>18</v>
@@ -7066,20 +7066,20 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K73" t="n">
-        <v>562</v>
+        <v>600</v>
       </c>
       <c r="L73" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="M73" t="n">
         <v>18</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>9992609290726</t>
+          <t>9992609290726_9992609290726_9992609290726K</t>
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
@@ -7113,7 +7113,7 @@
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
         </is>
       </c>
       <c r="Y73" t="inlineStr">
@@ -7128,25 +7128,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Estante 2</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Estante 2</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
         </is>
       </c>
       <c r="D74" t="n">
         <v>1</v>
       </c>
       <c r="E74" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F74" t="n">
-        <v>562</v>
+        <v>600</v>
       </c>
       <c r="G74" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="H74" t="n">
         <v>18</v>
@@ -7157,28 +7157,28 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K74" t="n">
-        <v>562</v>
+        <v>600</v>
       </c>
       <c r="L74" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="M74" t="n">
         <v>18</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>9992609290733</t>
+          <t>9992609290733_9992609290733_9992609290733K</t>
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R74" t="n">
         <v>0</v>
@@ -7204,7 +7204,7 @@
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600_Estante 2</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
         </is>
       </c>
       <c r="Y74" t="inlineStr">
@@ -7219,25 +7219,25 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
         </is>
       </c>
       <c r="D75" t="n">
         <v>1</v>
       </c>
       <c r="E75" t="n">
+        <v>884</v>
+      </c>
+      <c r="F75" t="n">
         <v>332</v>
       </c>
-      <c r="F75" t="n">
-        <v>800</v>
-      </c>
       <c r="G75" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="H75" t="n">
         <v>18</v>
@@ -7248,20 +7248,20 @@
         </is>
       </c>
       <c r="J75" t="n">
+        <v>884</v>
+      </c>
+      <c r="K75" t="n">
         <v>331</v>
       </c>
-      <c r="K75" t="n">
-        <v>800</v>
-      </c>
       <c r="L75" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="M75" t="n">
         <v>18</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>9992609290740_9992609290740_9992609290740K</t>
+          <t>9992609290740_9992609290740</t>
         </is>
       </c>
       <c r="O75" t="inlineStr"/>
@@ -7269,13 +7269,13 @@
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R75" t="n">
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" t="inlineStr">
         <is>
@@ -7295,7 +7295,7 @@
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
         </is>
       </c>
       <c r="Y75" t="inlineStr">
@@ -7310,25 +7310,25 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Techo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Techo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
         </is>
       </c>
       <c r="D76" t="n">
         <v>1</v>
       </c>
       <c r="E76" t="n">
+        <v>884</v>
+      </c>
+      <c r="F76" t="n">
         <v>332</v>
       </c>
-      <c r="F76" t="n">
-        <v>800</v>
-      </c>
       <c r="G76" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="H76" t="n">
         <v>18</v>
@@ -7339,13 +7339,13 @@
         </is>
       </c>
       <c r="J76" t="n">
+        <v>884</v>
+      </c>
+      <c r="K76" t="n">
         <v>331</v>
       </c>
-      <c r="K76" t="n">
-        <v>800</v>
-      </c>
       <c r="L76" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="M76" t="n">
         <v>18</v>
@@ -7357,13 +7357,13 @@
       </c>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q76" t="n">
         <v>0</v>
       </c>
       <c r="R76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S76" t="n">
         <v>0</v>
@@ -7386,7 +7386,7 @@
       <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Techo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
@@ -7401,49 +7401,49 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Lateral der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Lateral der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
         </is>
       </c>
       <c r="D77" t="n">
         <v>1</v>
       </c>
       <c r="E77" t="n">
-        <v>944</v>
+        <v>894</v>
       </c>
       <c r="F77" t="n">
-        <v>332</v>
+        <v>574</v>
       </c>
       <c r="G77" t="n">
-        <v>0.31</v>
+        <v>0.51</v>
       </c>
       <c r="H77" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>944</v>
+        <v>894</v>
       </c>
       <c r="K77" t="n">
-        <v>331</v>
+        <v>574</v>
       </c>
       <c r="L77" t="n">
-        <v>0.31</v>
+        <v>0.51</v>
       </c>
       <c r="M77" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>9992609290764_9992609290764</t>
+          <t>9992609290764</t>
         </is>
       </c>
       <c r="O77" t="inlineStr"/>
@@ -7457,7 +7457,7 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -7477,7 +7477,7 @@
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Lateral der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
         </is>
       </c>
       <c r="Y77" t="inlineStr">
@@ -7492,42 +7492,42 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Lateral izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Cenefa</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Lateral izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Cenefa</t>
         </is>
       </c>
       <c r="D78" t="n">
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>944</v>
+        <v>60</v>
       </c>
       <c r="F78" t="n">
-        <v>332</v>
+        <v>600</v>
       </c>
       <c r="G78" t="n">
-        <v>0.31</v>
+        <v>0.04</v>
       </c>
       <c r="H78" t="n">
         <v>18</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>944</v>
+        <v>59</v>
       </c>
       <c r="K78" t="n">
-        <v>331</v>
+        <v>598</v>
       </c>
       <c r="L78" t="n">
-        <v>0.31</v>
+        <v>0.04</v>
       </c>
       <c r="M78" t="n">
         <v>18</v>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q78" t="n">
         <v>0</v>
@@ -7548,7 +7548,7 @@
         <v>1</v>
       </c>
       <c r="S78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -7568,7 +7568,7 @@
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Lateral izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Cenefa</t>
         </is>
       </c>
       <c r="Y78" t="inlineStr">
@@ -7583,49 +7583,49 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Fondo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Cornisa</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Fondo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Cornisa</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>954</v>
+        <v>60</v>
       </c>
       <c r="F79" t="n">
-        <v>774</v>
+        <v>600</v>
       </c>
       <c r="G79" t="n">
-        <v>0.74</v>
+        <v>0.04</v>
       </c>
       <c r="H79" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>954</v>
+        <v>59</v>
       </c>
       <c r="K79" t="n">
-        <v>774</v>
+        <v>598</v>
       </c>
       <c r="L79" t="n">
-        <v>0.74</v>
+        <v>0.04</v>
       </c>
       <c r="M79" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>9992609290788</t>
+          <t>9992609290788_9992609290788</t>
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
@@ -7633,13 +7633,13 @@
         <v>0</v>
       </c>
       <c r="Q79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -7659,7 +7659,7 @@
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Fondo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Cornisa</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
@@ -7674,25 +7674,25 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Cenefa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Cenefa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="F80" t="n">
-        <v>800</v>
+        <v>597</v>
       </c>
       <c r="G80" t="n">
-        <v>0.05</v>
+        <v>0.18</v>
       </c>
       <c r="H80" t="n">
         <v>18</v>
@@ -7703,20 +7703,20 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>59</v>
+        <v>298</v>
       </c>
       <c r="K80" t="n">
-        <v>798</v>
+        <v>595</v>
       </c>
       <c r="L80" t="n">
-        <v>0.05</v>
+        <v>0.18</v>
       </c>
       <c r="M80" t="n">
         <v>18</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>9992609290795_9992609290795</t>
+          <t>9992609290795</t>
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
@@ -7724,7 +7724,7 @@
         <v>1</v>
       </c>
       <c r="Q80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R80" t="n">
         <v>1</v>
@@ -7750,7 +7750,7 @@
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Cenefa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -7765,60 +7765,60 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Puerta der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Puerta der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>977</v>
+        <v>564</v>
       </c>
       <c r="F81" t="n">
-        <v>397</v>
+        <v>301</v>
       </c>
       <c r="G81" t="n">
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
       <c r="H81" t="n">
         <v>18</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>975</v>
+        <v>564</v>
       </c>
       <c r="K81" t="n">
-        <v>395</v>
+        <v>300</v>
       </c>
       <c r="L81" t="n">
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
       <c r="M81" t="n">
         <v>18</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>9992609290801_9992609290801</t>
+          <t>9992609290801_9992609290801_9992609290801K</t>
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S81" t="n">
         <v>1</v>
@@ -7841,7 +7841,7 @@
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Puerta der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -7856,25 +7856,25 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Puerta izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Puerta izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>977</v>
+        <v>597</v>
       </c>
       <c r="F82" t="n">
-        <v>397</v>
+        <v>614</v>
       </c>
       <c r="G82" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="H82" t="n">
         <v>18</v>
@@ -7885,13 +7885,13 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>975</v>
+        <v>595</v>
       </c>
       <c r="K82" t="n">
-        <v>395</v>
+        <v>612</v>
       </c>
       <c r="L82" t="n">
-        <v>0.39</v>
+        <v>0.36</v>
       </c>
       <c r="M82" t="n">
         <v>18</v>
@@ -7932,7 +7932,7 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Puerta izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -7947,12 +7947,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -7962,10 +7962,10 @@
         <v>281</v>
       </c>
       <c r="F83" t="n">
-        <v>762</v>
+        <v>562</v>
       </c>
       <c r="G83" t="n">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="H83" t="n">
         <v>18</v>
@@ -7979,10 +7979,10 @@
         <v>280</v>
       </c>
       <c r="K83" t="n">
-        <v>762</v>
+        <v>562</v>
       </c>
       <c r="L83" t="n">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="M83" t="n">
         <v>18</v>
@@ -8023,7 +8023,7 @@
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -8038,25 +8038,25 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>1</v>
       </c>
       <c r="E84" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F84" t="n">
-        <v>762</v>
+        <v>800</v>
       </c>
       <c r="G84" t="n">
-        <v>0.21</v>
+        <v>0.27</v>
       </c>
       <c r="H84" t="n">
         <v>18</v>
@@ -8067,20 +8067,20 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K84" t="n">
-        <v>762</v>
+        <v>800</v>
       </c>
       <c r="L84" t="n">
-        <v>0.21</v>
+        <v>0.26</v>
       </c>
       <c r="M84" t="n">
         <v>18</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>9992609290832</t>
+          <t>9992609290832_9992609290832_9992609290832K</t>
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
@@ -8114,7 +8114,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Alacena 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -8129,12 +8129,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -8144,10 +8144,10 @@
         <v>332</v>
       </c>
       <c r="F85" t="n">
-        <v>570</v>
+        <v>800</v>
       </c>
       <c r="G85" t="n">
-        <v>0.19</v>
+        <v>0.27</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
@@ -8161,10 +8161,10 @@
         <v>331</v>
       </c>
       <c r="K85" t="n">
-        <v>570</v>
+        <v>800</v>
       </c>
       <c r="L85" t="n">
-        <v>0.19</v>
+        <v>0.26</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
@@ -8176,10 +8176,10 @@
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R85" t="n">
         <v>0</v>
@@ -8205,7 +8205,7 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -8220,25 +8220,25 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>1</v>
       </c>
       <c r="E86" t="n">
+        <v>884</v>
+      </c>
+      <c r="F86" t="n">
         <v>332</v>
       </c>
-      <c r="F86" t="n">
-        <v>570</v>
-      </c>
       <c r="G86" t="n">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="H86" t="n">
         <v>18</v>
@@ -8249,13 +8249,13 @@
         </is>
       </c>
       <c r="J86" t="n">
+        <v>884</v>
+      </c>
+      <c r="K86" t="n">
         <v>331</v>
       </c>
-      <c r="K86" t="n">
-        <v>570</v>
-      </c>
       <c r="L86" t="n">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="M86" t="n">
         <v>18</v>
@@ -8267,7 +8267,7 @@
       </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q86" t="n">
         <v>0</v>
@@ -8276,7 +8276,7 @@
         <v>0</v>
       </c>
       <c r="S86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8296,7 +8296,7 @@
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -8311,25 +8311,25 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>944</v>
+        <v>884</v>
       </c>
       <c r="F87" t="n">
         <v>332</v>
       </c>
       <c r="G87" t="n">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
       <c r="H87" t="n">
         <v>18</v>
@@ -8340,13 +8340,13 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>944</v>
+        <v>884</v>
       </c>
       <c r="K87" t="n">
         <v>331</v>
       </c>
       <c r="L87" t="n">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
       <c r="M87" t="n">
         <v>18</v>
@@ -8364,10 +8364,10 @@
         <v>0</v>
       </c>
       <c r="R87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T87" t="inlineStr">
         <is>
@@ -8387,7 +8387,7 @@
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -8402,49 +8402,49 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>944</v>
+        <v>894</v>
       </c>
       <c r="F88" t="n">
-        <v>332</v>
+        <v>774</v>
       </c>
       <c r="G88" t="n">
-        <v>0.31</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H88" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>944</v>
+        <v>894</v>
       </c>
       <c r="K88" t="n">
-        <v>331</v>
+        <v>774</v>
       </c>
       <c r="L88" t="n">
-        <v>0.31</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="M88" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>9992609290870_9992609290870</t>
+          <t>9992609290870</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
@@ -8455,7 +8455,7 @@
         <v>0</v>
       </c>
       <c r="R88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S88" t="n">
         <v>0</v>
@@ -8478,7 +8478,7 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -8493,63 +8493,63 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Cenefa</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Cenefa</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>954</v>
+        <v>60</v>
       </c>
       <c r="F89" t="n">
-        <v>544</v>
+        <v>800</v>
       </c>
       <c r="G89" t="n">
-        <v>0.52</v>
+        <v>0.05</v>
       </c>
       <c r="H89" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>954</v>
+        <v>59</v>
       </c>
       <c r="K89" t="n">
-        <v>544</v>
+        <v>798</v>
       </c>
       <c r="L89" t="n">
-        <v>0.52</v>
+        <v>0.05</v>
       </c>
       <c r="M89" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>9992609290887</t>
+          <t>9992609290887_9992609290887</t>
         </is>
       </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q89" t="n">
         <v>0</v>
       </c>
       <c r="R89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T89" t="inlineStr">
         <is>
@@ -8569,7 +8569,7 @@
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Cenefa</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -8584,12 +8584,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Cenefa</t>
+          <t>COCINA-01_A3 Vitrina 800_Cornisa</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Cenefa</t>
+          <t>COCINA-01_A3 Vitrina 800_Cornisa</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -8599,10 +8599,10 @@
         <v>60</v>
       </c>
       <c r="F90" t="n">
-        <v>570</v>
+        <v>800</v>
       </c>
       <c r="G90" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H90" t="n">
         <v>18</v>
@@ -8616,10 +8616,10 @@
         <v>59</v>
       </c>
       <c r="K90" t="n">
-        <v>568</v>
+        <v>798</v>
       </c>
       <c r="L90" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M90" t="n">
         <v>18</v>
@@ -8631,10 +8631,10 @@
       </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R90" t="n">
         <v>1</v>
@@ -8660,7 +8660,7 @@
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Cenefa</t>
+          <t>COCINA-01_A3 Vitrina 800_Cornisa</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr">
@@ -8675,25 +8675,25 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>977</v>
+        <v>917</v>
       </c>
       <c r="F91" t="n">
-        <v>282</v>
+        <v>397</v>
       </c>
       <c r="G91" t="n">
-        <v>0.28</v>
+        <v>0.36</v>
       </c>
       <c r="H91" t="n">
         <v>18</v>
@@ -8704,13 +8704,13 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>975</v>
+        <v>915</v>
       </c>
       <c r="K91" t="n">
-        <v>280</v>
+        <v>395</v>
       </c>
       <c r="L91" t="n">
-        <v>0.27</v>
+        <v>0.36</v>
       </c>
       <c r="M91" t="n">
         <v>18</v>
@@ -8751,7 +8751,7 @@
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -8766,25 +8766,25 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>977</v>
+        <v>917</v>
       </c>
       <c r="F92" t="n">
-        <v>282</v>
+        <v>397</v>
       </c>
       <c r="G92" t="n">
-        <v>0.28</v>
+        <v>0.36</v>
       </c>
       <c r="H92" t="n">
         <v>18</v>
@@ -8795,13 +8795,13 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>975</v>
+        <v>915</v>
       </c>
       <c r="K92" t="n">
-        <v>280</v>
+        <v>395</v>
       </c>
       <c r="L92" t="n">
-        <v>0.27</v>
+        <v>0.36</v>
       </c>
       <c r="M92" t="n">
         <v>18</v>
@@ -8842,7 +8842,7 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -8857,12 +8857,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -8872,10 +8872,10 @@
         <v>281</v>
       </c>
       <c r="F93" t="n">
-        <v>532</v>
+        <v>762</v>
       </c>
       <c r="G93" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="H93" t="n">
         <v>18</v>
@@ -8889,10 +8889,10 @@
         <v>280</v>
       </c>
       <c r="K93" t="n">
-        <v>532</v>
+        <v>762</v>
       </c>
       <c r="L93" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="M93" t="n">
         <v>18</v>
@@ -8933,7 +8933,7 @@
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -8948,12 +8948,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -8963,10 +8963,10 @@
         <v>281</v>
       </c>
       <c r="F94" t="n">
-        <v>532</v>
+        <v>762</v>
       </c>
       <c r="G94" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="H94" t="n">
         <v>18</v>
@@ -8980,10 +8980,10 @@
         <v>280</v>
       </c>
       <c r="K94" t="n">
-        <v>532</v>
+        <v>762</v>
       </c>
       <c r="L94" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="M94" t="n">
         <v>18</v>
@@ -9024,7 +9024,7 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Alacena 570_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -9039,57 +9039,57 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>99</v>
+        <v>332</v>
       </c>
       <c r="F95" t="n">
-        <v>955</v>
+        <v>570</v>
       </c>
       <c r="G95" t="n">
-        <v>0.09</v>
+        <v>0.19</v>
       </c>
       <c r="H95" t="n">
         <v>18</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>98</v>
+        <v>331</v>
       </c>
       <c r="K95" t="n">
-        <v>955</v>
+        <v>570</v>
       </c>
       <c r="L95" t="n">
-        <v>0.09</v>
+        <v>0.19</v>
       </c>
       <c r="M95" t="n">
         <v>18</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>9992609290948</t>
+          <t>9992609290948_9992609290948_9992609290948K</t>
         </is>
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R95" t="n">
         <v>0</v>
@@ -9115,7 +9115,7 @@
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -9130,49 +9130,49 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>99</v>
+        <v>332</v>
       </c>
       <c r="F96" t="n">
-        <v>367.7</v>
+        <v>570</v>
       </c>
       <c r="G96" t="n">
-        <v>0.04</v>
+        <v>0.19</v>
       </c>
       <c r="H96" t="n">
         <v>18</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>98</v>
+        <v>331</v>
       </c>
       <c r="K96" t="n">
-        <v>367.7</v>
+        <v>570</v>
       </c>
       <c r="L96" t="n">
-        <v>0.04</v>
+        <v>0.19</v>
       </c>
       <c r="M96" t="n">
         <v>18</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>9992609290955</t>
+          <t>9992609290955_9992609290955_9992609290955K</t>
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
@@ -9206,12 +9206,1013 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>9992609290955</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" t="n">
+        <v>884</v>
+      </c>
+      <c r="F97" t="n">
+        <v>332</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H97" t="n">
+        <v>18</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>884</v>
+      </c>
+      <c r="K97" t="n">
+        <v>331</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="M97" t="n">
+        <v>18</v>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>9992609290962_9992609290962</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr"/>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0</v>
+      </c>
+      <c r="R97" t="n">
+        <v>0</v>
+      </c>
+      <c r="S97" t="n">
+        <v>1</v>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr"/>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>9992609290962</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="n">
+        <v>884</v>
+      </c>
+      <c r="F98" t="n">
+        <v>332</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H98" t="n">
+        <v>18</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>884</v>
+      </c>
+      <c r="K98" t="n">
+        <v>331</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="M98" t="n">
+        <v>18</v>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>9992609290979_9992609290979</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr"/>
+      <c r="P98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0</v>
+      </c>
+      <c r="R98" t="n">
+        <v>1</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0</v>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr"/>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>9992609290979</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" t="n">
+        <v>894</v>
+      </c>
+      <c r="F99" t="n">
+        <v>544</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H99" t="n">
+        <v>5</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>5_Melamina_BLANCO 5</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>894</v>
+      </c>
+      <c r="K99" t="n">
+        <v>544</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="M99" t="n">
+        <v>5</v>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>9992609290986</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr"/>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="R99" t="n">
+        <v>0</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0</v>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr"/>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>9992609290986</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Cenefa</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Cenefa</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" t="n">
+        <v>60</v>
+      </c>
+      <c r="F100" t="n">
+        <v>570</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H100" t="n">
+        <v>18</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>59</v>
+      </c>
+      <c r="K100" t="n">
+        <v>568</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M100" t="n">
+        <v>18</v>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>9992609290993_9992609290993</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr"/>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
+        <v>1</v>
+      </c>
+      <c r="S100" t="n">
+        <v>1</v>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr"/>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Cenefa</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>9992609290993</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Cornisa</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Cornisa</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" t="n">
+        <v>60</v>
+      </c>
+      <c r="F101" t="n">
+        <v>570</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H101" t="n">
+        <v>18</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>59</v>
+      </c>
+      <c r="K101" t="n">
+        <v>568</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M101" t="n">
+        <v>18</v>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>9992609291006_9992609291006</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr"/>
+      <c r="P101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>1</v>
+      </c>
+      <c r="R101" t="n">
+        <v>1</v>
+      </c>
+      <c r="S101" t="n">
+        <v>1</v>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr"/>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Cornisa</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>9992609291006</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" t="n">
+        <v>917</v>
+      </c>
+      <c r="F102" t="n">
+        <v>282</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H102" t="n">
+        <v>18</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>915</v>
+      </c>
+      <c r="K102" t="n">
+        <v>280</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="M102" t="n">
+        <v>18</v>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>9992609291013_9992609291013</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr"/>
+      <c r="P102" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>1</v>
+      </c>
+      <c r="R102" t="n">
+        <v>1</v>
+      </c>
+      <c r="S102" t="n">
+        <v>1</v>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr"/>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>9992609291013</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" t="n">
+        <v>917</v>
+      </c>
+      <c r="F103" t="n">
+        <v>282</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H103" t="n">
+        <v>18</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>915</v>
+      </c>
+      <c r="K103" t="n">
+        <v>280</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="M103" t="n">
+        <v>18</v>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>9992609291020_9992609291020</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr"/>
+      <c r="P103" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>1</v>
+      </c>
+      <c r="R103" t="n">
+        <v>1</v>
+      </c>
+      <c r="S103" t="n">
+        <v>1</v>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr"/>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>9992609291020</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" t="n">
+        <v>281</v>
+      </c>
+      <c r="F104" t="n">
+        <v>532</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H104" t="n">
+        <v>18</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>280</v>
+      </c>
+      <c r="K104" t="n">
+        <v>532</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M104" t="n">
+        <v>18</v>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>9992609291037</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr"/>
+      <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>1</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0</v>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr"/>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>9992609291037</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" t="n">
+        <v>281</v>
+      </c>
+      <c r="F105" t="n">
+        <v>532</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H105" t="n">
+        <v>18</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>280</v>
+      </c>
+      <c r="K105" t="n">
+        <v>532</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M105" t="n">
+        <v>18</v>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>9992609291044</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr"/>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>1</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>9992609291044</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" t="n">
+        <v>99</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1407</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H106" t="n">
+        <v>18</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>98</v>
+      </c>
+      <c r="K106" t="n">
+        <v>1407</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="M106" t="n">
+        <v>18</v>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>9992609291051</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>9992609291051</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
           <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
-      <c r="Y96" t="inlineStr">
-        <is>
-          <t>9992609290955</t>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" t="n">
+        <v>99</v>
+      </c>
+      <c r="F107" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H107" t="n">
+        <v>18</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>98</v>
+      </c>
+      <c r="K107" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="L107" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M107" t="n">
+        <v>18</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>9992609291068</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr"/>
+      <c r="P107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr"/>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>9992609291068</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
COCINA-01 alacenas: sin cenefa ni cornisa (LED embutido), travesaño trasero 18x80 para colgar, frente fijo de la rebatible a 1/3; 103/103 receta = sólido; paquete regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,19 +413,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y107"/>
+  <dimension ref="A1:Y104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="4" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="5" customWidth="1" min="13" max="13"/>
@@ -5866,13 +5866,13 @@
         <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>920</v>
+        <v>1040</v>
       </c>
       <c r="F60" t="n">
         <v>332</v>
       </c>
       <c r="G60" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="H60" t="n">
         <v>18</v>
@@ -5883,13 +5883,13 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>920</v>
+        <v>1040</v>
       </c>
       <c r="K60" t="n">
         <v>331</v>
       </c>
       <c r="L60" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="M60" t="n">
         <v>18</v>
@@ -5957,13 +5957,13 @@
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>920</v>
+        <v>1040</v>
       </c>
       <c r="F61" t="n">
         <v>332</v>
       </c>
       <c r="G61" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="H61" t="n">
         <v>18</v>
@@ -5974,13 +5974,13 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>920</v>
+        <v>1040</v>
       </c>
       <c r="K61" t="n">
         <v>331</v>
       </c>
       <c r="L61" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="M61" t="n">
         <v>18</v>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>9992609290627_9992609290627_9992609290627K</t>
+          <t>9992609290627_9992609290627</t>
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
@@ -6230,13 +6230,13 @@
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>894</v>
+        <v>1014</v>
       </c>
       <c r="F64" t="n">
         <v>755</v>
       </c>
       <c r="G64" t="n">
-        <v>0.67</v>
+        <v>0.77</v>
       </c>
       <c r="H64" t="n">
         <v>5</v>
@@ -6247,13 +6247,13 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>894</v>
+        <v>1014</v>
       </c>
       <c r="K64" t="n">
         <v>755</v>
       </c>
       <c r="L64" t="n">
-        <v>0.67</v>
+        <v>0.77</v>
       </c>
       <c r="M64" t="n">
         <v>5</v>
@@ -6321,13 +6321,13 @@
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>894</v>
+        <v>1014</v>
       </c>
       <c r="F65" t="n">
         <v>762</v>
       </c>
       <c r="G65" t="n">
-        <v>0.68</v>
+        <v>0.77</v>
       </c>
       <c r="H65" t="n">
         <v>5</v>
@@ -6338,13 +6338,13 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>894</v>
+        <v>1014</v>
       </c>
       <c r="K65" t="n">
         <v>762</v>
       </c>
       <c r="L65" t="n">
-        <v>0.68</v>
+        <v>0.77</v>
       </c>
       <c r="M65" t="n">
         <v>5</v>
@@ -6412,13 +6412,13 @@
         <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="F66" t="n">
         <v>80</v>
       </c>
       <c r="G66" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="H66" t="n">
         <v>18</v>
@@ -6429,13 +6429,13 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="K66" t="n">
         <v>79</v>
       </c>
       <c r="L66" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="M66" t="n">
         <v>18</v>
@@ -6503,13 +6503,13 @@
         <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="F67" t="n">
         <v>80</v>
       </c>
       <c r="G67" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="H67" t="n">
         <v>18</v>
@@ -6520,13 +6520,13 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="K67" t="n">
         <v>79</v>
       </c>
       <c r="L67" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="M67" t="n">
         <v>18</v>
@@ -6594,13 +6594,13 @@
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>917</v>
+        <v>1037</v>
       </c>
       <c r="F68" t="n">
         <v>633.4</v>
       </c>
       <c r="G68" t="n">
-        <v>0.58</v>
+        <v>0.66</v>
       </c>
       <c r="H68" t="n">
         <v>18</v>
@@ -6611,13 +6611,13 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>915</v>
+        <v>1035</v>
       </c>
       <c r="K68" t="n">
         <v>631.4</v>
       </c>
       <c r="L68" t="n">
-        <v>0.58</v>
+        <v>0.65</v>
       </c>
       <c r="M68" t="n">
         <v>18</v>
@@ -6855,42 +6855,42 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
         </is>
       </c>
       <c r="D71" t="n">
         <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F71" t="n">
-        <v>636.4</v>
+        <v>751</v>
       </c>
       <c r="G71" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="H71" t="n">
         <v>18</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="K71" t="n">
-        <v>636.4</v>
+        <v>751</v>
       </c>
       <c r="L71" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="M71" t="n">
         <v>18</v>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q71" t="n">
         <v>0</v>
@@ -6931,7 +6931,7 @@
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cenefa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
         </is>
       </c>
       <c r="Y71" t="inlineStr">
@@ -6946,42 +6946,42 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cornisa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cornisa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F72" t="n">
-        <v>636.4</v>
+        <v>751</v>
       </c>
       <c r="G72" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="H72" t="n">
         <v>18</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="K72" t="n">
-        <v>636.4</v>
+        <v>751</v>
       </c>
       <c r="L72" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="M72" t="n">
         <v>18</v>
@@ -6996,7 +6996,7 @@
         <v>0</v>
       </c>
       <c r="Q72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R72" t="n">
         <v>0</v>
@@ -7022,7 +7022,7 @@
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Cornisa</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
         </is>
       </c>
       <c r="Y72" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>9992609290733_9992609290733_9992609290733K</t>
+          <t>9992609290733_9992609290733</t>
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
@@ -7231,13 +7231,13 @@
         <v>1</v>
       </c>
       <c r="E75" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="F75" t="n">
         <v>332</v>
       </c>
       <c r="G75" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="H75" t="n">
         <v>18</v>
@@ -7248,13 +7248,13 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="K75" t="n">
         <v>331</v>
       </c>
       <c r="L75" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="M75" t="n">
         <v>18</v>
@@ -7322,13 +7322,13 @@
         <v>1</v>
       </c>
       <c r="E76" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="F76" t="n">
         <v>332</v>
       </c>
       <c r="G76" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="H76" t="n">
         <v>18</v>
@@ -7339,13 +7339,13 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="K76" t="n">
         <v>331</v>
       </c>
       <c r="L76" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="M76" t="n">
         <v>18</v>
@@ -7413,13 +7413,13 @@
         <v>1</v>
       </c>
       <c r="E77" t="n">
-        <v>894</v>
+        <v>1014</v>
       </c>
       <c r="F77" t="n">
         <v>574</v>
       </c>
       <c r="G77" t="n">
-        <v>0.51</v>
+        <v>0.58</v>
       </c>
       <c r="H77" t="n">
         <v>5</v>
@@ -7430,13 +7430,13 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>894</v>
+        <v>1014</v>
       </c>
       <c r="K77" t="n">
         <v>574</v>
       </c>
       <c r="L77" t="n">
-        <v>0.51</v>
+        <v>0.58</v>
       </c>
       <c r="M77" t="n">
         <v>5</v>
@@ -7492,42 +7492,42 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Cenefa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Cenefa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
         </is>
       </c>
       <c r="D78" t="n">
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F78" t="n">
-        <v>600</v>
+        <v>564</v>
       </c>
       <c r="G78" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="H78" t="n">
         <v>18</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="K78" t="n">
-        <v>598</v>
+        <v>564</v>
       </c>
       <c r="L78" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="M78" t="n">
         <v>18</v>
@@ -7539,16 +7539,16 @@
       </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q78" t="n">
         <v>0</v>
       </c>
       <c r="R78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -7568,7 +7568,7 @@
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Cenefa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
         </is>
       </c>
       <c r="Y78" t="inlineStr">
@@ -7583,25 +7583,25 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Cornisa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Cornisa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>60</v>
+        <v>346</v>
       </c>
       <c r="F79" t="n">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="G79" t="n">
-        <v>0.04</v>
+        <v>0.21</v>
       </c>
       <c r="H79" t="n">
         <v>18</v>
@@ -7612,25 +7612,25 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>59</v>
+        <v>344</v>
       </c>
       <c r="K79" t="n">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="L79" t="n">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
       <c r="M79" t="n">
         <v>18</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>9992609290788_9992609290788</t>
+          <t>9992609290788</t>
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q79" t="n">
         <v>1</v>
@@ -7659,7 +7659,7 @@
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Cornisa</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
@@ -7674,60 +7674,60 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>1</v>
       </c>
       <c r="E80" t="n">
+        <v>564</v>
+      </c>
+      <c r="F80" t="n">
+        <v>301</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H80" t="n">
+        <v>18</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>564</v>
+      </c>
+      <c r="K80" t="n">
         <v>300</v>
       </c>
-      <c r="F80" t="n">
-        <v>597</v>
-      </c>
-      <c r="G80" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="H80" t="n">
-        <v>18</v>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>18_Melamina_VERDE 18</t>
-        </is>
-      </c>
-      <c r="J80" t="n">
-        <v>298</v>
-      </c>
-      <c r="K80" t="n">
-        <v>595</v>
-      </c>
       <c r="L80" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="M80" t="n">
         <v>18</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>9992609290795</t>
+          <t>9992609290795_9992609290795_9992609290795K</t>
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S80" t="n">
         <v>1</v>
@@ -7750,7 +7750,7 @@
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -7765,60 +7765,60 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>564</v>
+        <v>597</v>
       </c>
       <c r="F81" t="n">
-        <v>301</v>
+        <v>688</v>
       </c>
       <c r="G81" t="n">
-        <v>0.17</v>
+        <v>0.41</v>
       </c>
       <c r="H81" t="n">
         <v>18</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>564</v>
+        <v>595</v>
       </c>
       <c r="K81" t="n">
-        <v>300</v>
+        <v>686</v>
       </c>
       <c r="L81" t="n">
-        <v>0.17</v>
+        <v>0.41</v>
       </c>
       <c r="M81" t="n">
         <v>18</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>9992609290801_9992609290801_9992609290801K</t>
+          <t>9992609290801_9992609290801</t>
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S81" t="n">
         <v>1</v>
@@ -7841,7 +7841,7 @@
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -7856,63 +7856,63 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>597</v>
+        <v>281</v>
       </c>
       <c r="F82" t="n">
-        <v>614</v>
+        <v>562</v>
       </c>
       <c r="G82" t="n">
-        <v>0.37</v>
+        <v>0.16</v>
       </c>
       <c r="H82" t="n">
         <v>18</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>595</v>
+        <v>280</v>
       </c>
       <c r="K82" t="n">
-        <v>612</v>
+        <v>562</v>
       </c>
       <c r="L82" t="n">
-        <v>0.36</v>
+        <v>0.16</v>
       </c>
       <c r="M82" t="n">
         <v>18</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>9992609290818_9992609290818</t>
+          <t>9992609290818</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q82" t="n">
         <v>1</v>
       </c>
       <c r="R82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T82" t="inlineStr">
         <is>
@@ -7932,7 +7932,7 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -7947,25 +7947,25 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F83" t="n">
-        <v>562</v>
+        <v>800</v>
       </c>
       <c r="G83" t="n">
-        <v>0.16</v>
+        <v>0.27</v>
       </c>
       <c r="H83" t="n">
         <v>18</v>
@@ -7976,20 +7976,20 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K83" t="n">
-        <v>562</v>
+        <v>800</v>
       </c>
       <c r="L83" t="n">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="M83" t="n">
         <v>18</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>9992609290825</t>
+          <t>9992609290825_9992609290825_9992609290825K</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
@@ -8023,7 +8023,7 @@
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -8038,12 +8038,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -8080,15 +8080,15 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>9992609290832_9992609290832_9992609290832K</t>
+          <t>9992609290832_9992609290832</t>
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R84" t="n">
         <v>0</v>
@@ -8114,7 +8114,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -8129,25 +8129,25 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F85" t="n">
         <v>332</v>
       </c>
-      <c r="F85" t="n">
-        <v>800</v>
-      </c>
       <c r="G85" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
@@ -8158,25 +8158,25 @@
         </is>
       </c>
       <c r="J85" t="n">
+        <v>1004</v>
+      </c>
+      <c r="K85" t="n">
         <v>331</v>
       </c>
-      <c r="K85" t="n">
-        <v>800</v>
-      </c>
       <c r="L85" t="n">
-        <v>0.26</v>
+        <v>0.33</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>9992609290849_9992609290849_9992609290849K</t>
+          <t>9992609290849_9992609290849</t>
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q85" t="n">
         <v>0</v>
@@ -8185,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="S85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -8205,7 +8205,7 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -8220,25 +8220,25 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="F86" t="n">
         <v>332</v>
       </c>
       <c r="G86" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="H86" t="n">
         <v>18</v>
@@ -8249,13 +8249,13 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>884</v>
+        <v>1004</v>
       </c>
       <c r="K86" t="n">
         <v>331</v>
       </c>
       <c r="L86" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="M86" t="n">
         <v>18</v>
@@ -8273,10 +8273,10 @@
         <v>0</v>
       </c>
       <c r="R86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8296,7 +8296,7 @@
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -8311,49 +8311,49 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>884</v>
+        <v>1014</v>
       </c>
       <c r="F87" t="n">
-        <v>332</v>
+        <v>774</v>
       </c>
       <c r="G87" t="n">
-        <v>0.29</v>
+        <v>0.78</v>
       </c>
       <c r="H87" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>884</v>
+        <v>1014</v>
       </c>
       <c r="K87" t="n">
-        <v>331</v>
+        <v>774</v>
       </c>
       <c r="L87" t="n">
-        <v>0.29</v>
+        <v>0.78</v>
       </c>
       <c r="M87" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>9992609290863_9992609290863</t>
+          <t>9992609290863</t>
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
@@ -8364,7 +8364,7 @@
         <v>0</v>
       </c>
       <c r="R87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S87" t="n">
         <v>0</v>
@@ -8387,7 +8387,7 @@
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -8402,49 +8402,49 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>894</v>
+        <v>80</v>
       </c>
       <c r="F88" t="n">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="G88" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="H88" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>894</v>
+        <v>80</v>
       </c>
       <c r="K88" t="n">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="L88" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="M88" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>9992609290870</t>
+          <t>9992609290870_9992609290870</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -8493,25 +8493,25 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Cenefa</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Cenefa</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>60</v>
+        <v>1037</v>
       </c>
       <c r="F89" t="n">
-        <v>800</v>
+        <v>397</v>
       </c>
       <c r="G89" t="n">
-        <v>0.05</v>
+        <v>0.41</v>
       </c>
       <c r="H89" t="n">
         <v>18</v>
@@ -8522,13 +8522,13 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>59</v>
+        <v>1035</v>
       </c>
       <c r="K89" t="n">
-        <v>798</v>
+        <v>395</v>
       </c>
       <c r="L89" t="n">
-        <v>0.05</v>
+        <v>0.41</v>
       </c>
       <c r="M89" t="n">
         <v>18</v>
@@ -8543,7 +8543,7 @@
         <v>1</v>
       </c>
       <c r="Q89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R89" t="n">
         <v>1</v>
@@ -8569,7 +8569,7 @@
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Cenefa</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -8584,25 +8584,25 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Cornisa</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Cornisa</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="D90" t="n">
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>60</v>
+        <v>1037</v>
       </c>
       <c r="F90" t="n">
-        <v>800</v>
+        <v>397</v>
       </c>
       <c r="G90" t="n">
-        <v>0.05</v>
+        <v>0.41</v>
       </c>
       <c r="H90" t="n">
         <v>18</v>
@@ -8613,13 +8613,13 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>59</v>
+        <v>1035</v>
       </c>
       <c r="K90" t="n">
-        <v>798</v>
+        <v>395</v>
       </c>
       <c r="L90" t="n">
-        <v>0.05</v>
+        <v>0.41</v>
       </c>
       <c r="M90" t="n">
         <v>18</v>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q90" t="n">
         <v>1</v>
@@ -8660,7 +8660,7 @@
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Cornisa</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr">
@@ -8675,63 +8675,63 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>917</v>
+        <v>281</v>
       </c>
       <c r="F91" t="n">
-        <v>397</v>
+        <v>762</v>
       </c>
       <c r="G91" t="n">
-        <v>0.36</v>
+        <v>0.21</v>
       </c>
       <c r="H91" t="n">
         <v>18</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>915</v>
+        <v>280</v>
       </c>
       <c r="K91" t="n">
-        <v>395</v>
+        <v>762</v>
       </c>
       <c r="L91" t="n">
-        <v>0.36</v>
+        <v>0.21</v>
       </c>
       <c r="M91" t="n">
         <v>18</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>9992609290900_9992609290900</t>
+          <t>9992609290900</t>
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q91" t="n">
         <v>1</v>
       </c>
       <c r="R91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T91" t="inlineStr">
         <is>
@@ -8751,7 +8751,7 @@
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -8766,63 +8766,63 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>917</v>
+        <v>281</v>
       </c>
       <c r="F92" t="n">
-        <v>397</v>
+        <v>762</v>
       </c>
       <c r="G92" t="n">
-        <v>0.36</v>
+        <v>0.21</v>
       </c>
       <c r="H92" t="n">
         <v>18</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>915</v>
+        <v>280</v>
       </c>
       <c r="K92" t="n">
-        <v>395</v>
+        <v>762</v>
       </c>
       <c r="L92" t="n">
-        <v>0.36</v>
+        <v>0.21</v>
       </c>
       <c r="M92" t="n">
         <v>18</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>9992609290917_9992609290917</t>
+          <t>9992609290917</t>
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q92" t="n">
         <v>1</v>
       </c>
       <c r="R92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T92" t="inlineStr">
         <is>
@@ -8842,7 +8842,7 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -8857,25 +8857,25 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F93" t="n">
-        <v>762</v>
+        <v>570</v>
       </c>
       <c r="G93" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="H93" t="n">
         <v>18</v>
@@ -8886,20 +8886,20 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K93" t="n">
-        <v>762</v>
+        <v>570</v>
       </c>
       <c r="L93" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="M93" t="n">
         <v>18</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>9992609290924</t>
+          <t>9992609290924_9992609290924_9992609290924K</t>
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -8948,25 +8948,25 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F94" t="n">
-        <v>762</v>
+        <v>570</v>
       </c>
       <c r="G94" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="H94" t="n">
         <v>18</v>
@@ -8977,28 +8977,28 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K94" t="n">
-        <v>762</v>
+        <v>570</v>
       </c>
       <c r="L94" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="M94" t="n">
         <v>18</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>9992609290931</t>
+          <t>9992609290931_9992609290931</t>
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R94" t="n">
         <v>0</v>
@@ -9024,7 +9024,7 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -9039,25 +9039,25 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F95" t="n">
         <v>332</v>
       </c>
-      <c r="F95" t="n">
-        <v>570</v>
-      </c>
       <c r="G95" t="n">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="H95" t="n">
         <v>18</v>
@@ -9068,20 +9068,20 @@
         </is>
       </c>
       <c r="J95" t="n">
+        <v>1004</v>
+      </c>
+      <c r="K95" t="n">
         <v>331</v>
       </c>
-      <c r="K95" t="n">
-        <v>570</v>
-      </c>
       <c r="L95" t="n">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="M95" t="n">
         <v>18</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>9992609290948_9992609290948_9992609290948K</t>
+          <t>9992609290948_9992609290948</t>
         </is>
       </c>
       <c r="O95" t="inlineStr"/>
@@ -9089,13 +9089,13 @@
         <v>0</v>
       </c>
       <c r="Q95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R95" t="n">
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T95" t="inlineStr">
         <is>
@@ -9115,7 +9115,7 @@
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -9130,25 +9130,25 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F96" t="n">
         <v>332</v>
       </c>
-      <c r="F96" t="n">
-        <v>570</v>
-      </c>
       <c r="G96" t="n">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="H96" t="n">
         <v>18</v>
@@ -9159,31 +9159,31 @@
         </is>
       </c>
       <c r="J96" t="n">
+        <v>1004</v>
+      </c>
+      <c r="K96" t="n">
         <v>331</v>
       </c>
-      <c r="K96" t="n">
-        <v>570</v>
-      </c>
       <c r="L96" t="n">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="M96" t="n">
         <v>18</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>9992609290955_9992609290955_9992609290955K</t>
+          <t>9992609290955_9992609290955</t>
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q96" t="n">
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S96" t="n">
         <v>0</v>
@@ -9206,7 +9206,7 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -9221,49 +9221,49 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>884</v>
+        <v>1014</v>
       </c>
       <c r="F97" t="n">
-        <v>332</v>
+        <v>544</v>
       </c>
       <c r="G97" t="n">
-        <v>0.29</v>
+        <v>0.55</v>
       </c>
       <c r="H97" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>884</v>
+        <v>1014</v>
       </c>
       <c r="K97" t="n">
-        <v>331</v>
+        <v>544</v>
       </c>
       <c r="L97" t="n">
-        <v>0.29</v>
+        <v>0.55</v>
       </c>
       <c r="M97" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>9992609290962_9992609290962</t>
+          <t>9992609290962</t>
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
@@ -9277,7 +9277,7 @@
         <v>0</v>
       </c>
       <c r="S97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T97" t="inlineStr">
         <is>
@@ -9297,7 +9297,7 @@
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -9312,25 +9312,25 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>884</v>
+        <v>80</v>
       </c>
       <c r="F98" t="n">
-        <v>332</v>
+        <v>534</v>
       </c>
       <c r="G98" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="H98" t="n">
         <v>18</v>
@@ -9341,13 +9341,13 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>884</v>
+        <v>80</v>
       </c>
       <c r="K98" t="n">
-        <v>331</v>
+        <v>534</v>
       </c>
       <c r="L98" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="M98" t="n">
         <v>18</v>
@@ -9365,7 +9365,7 @@
         <v>0</v>
       </c>
       <c r="R98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S98" t="n">
         <v>0</v>
@@ -9388,7 +9388,7 @@
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -9403,63 +9403,63 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>894</v>
+        <v>1037</v>
       </c>
       <c r="F99" t="n">
-        <v>544</v>
+        <v>282</v>
       </c>
       <c r="G99" t="n">
-        <v>0.49</v>
+        <v>0.29</v>
       </c>
       <c r="H99" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>894</v>
+        <v>1035</v>
       </c>
       <c r="K99" t="n">
-        <v>544</v>
+        <v>280</v>
       </c>
       <c r="L99" t="n">
-        <v>0.49</v>
+        <v>0.29</v>
       </c>
       <c r="M99" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>9992609290986</t>
+          <t>9992609290986_9992609290986</t>
         </is>
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
@@ -9479,7 +9479,7 @@
       <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -9494,25 +9494,25 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Cenefa</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Cenefa</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>60</v>
+        <v>1037</v>
       </c>
       <c r="F100" t="n">
-        <v>570</v>
+        <v>282</v>
       </c>
       <c r="G100" t="n">
-        <v>0.03</v>
+        <v>0.29</v>
       </c>
       <c r="H100" t="n">
         <v>18</v>
@@ -9523,13 +9523,13 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>59</v>
+        <v>1035</v>
       </c>
       <c r="K100" t="n">
-        <v>568</v>
+        <v>280</v>
       </c>
       <c r="L100" t="n">
-        <v>0.03</v>
+        <v>0.29</v>
       </c>
       <c r="M100" t="n">
         <v>18</v>
@@ -9544,7 +9544,7 @@
         <v>1</v>
       </c>
       <c r="Q100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R100" t="n">
         <v>1</v>
@@ -9570,7 +9570,7 @@
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Cenefa</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -9585,49 +9585,49 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Cornisa</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Cornisa</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>60</v>
+        <v>281</v>
       </c>
       <c r="F101" t="n">
-        <v>570</v>
+        <v>532</v>
       </c>
       <c r="G101" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="H101" t="n">
         <v>18</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>59</v>
+        <v>280</v>
       </c>
       <c r="K101" t="n">
-        <v>568</v>
+        <v>532</v>
       </c>
       <c r="L101" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="M101" t="n">
         <v>18</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>9992609291006_9992609291006</t>
+          <t>9992609291006</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
@@ -9638,10 +9638,10 @@
         <v>1</v>
       </c>
       <c r="R101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T101" t="inlineStr">
         <is>
@@ -9661,7 +9661,7 @@
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Cornisa</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -9676,63 +9676,63 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>917</v>
+        <v>281</v>
       </c>
       <c r="F102" t="n">
-        <v>282</v>
+        <v>532</v>
       </c>
       <c r="G102" t="n">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="H102" t="n">
         <v>18</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>915</v>
+        <v>280</v>
       </c>
       <c r="K102" t="n">
-        <v>280</v>
+        <v>532</v>
       </c>
       <c r="L102" t="n">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="M102" t="n">
         <v>18</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>9992609291013_9992609291013</t>
+          <t>9992609291013</t>
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q102" t="n">
         <v>1</v>
       </c>
       <c r="R102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T102" t="inlineStr">
         <is>
@@ -9752,7 +9752,7 @@
       <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -9767,25 +9767,25 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>917</v>
+        <v>99</v>
       </c>
       <c r="F103" t="n">
-        <v>282</v>
+        <v>1407</v>
       </c>
       <c r="G103" t="n">
-        <v>0.26</v>
+        <v>0.14</v>
       </c>
       <c r="H103" t="n">
         <v>18</v>
@@ -9796,20 +9796,20 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>915</v>
+        <v>98</v>
       </c>
       <c r="K103" t="n">
-        <v>280</v>
+        <v>1407</v>
       </c>
       <c r="L103" t="n">
-        <v>0.26</v>
+        <v>0.14</v>
       </c>
       <c r="M103" t="n">
         <v>18</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>9992609291020_9992609291020</t>
+          <t>9992609291020</t>
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
@@ -9817,13 +9817,13 @@
         <v>1</v>
       </c>
       <c r="Q103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T103" t="inlineStr">
         <is>
@@ -9843,7 +9843,7 @@
       <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -9858,42 +9858,42 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>281</v>
+        <v>99</v>
       </c>
       <c r="F104" t="n">
-        <v>532</v>
+        <v>367.7</v>
       </c>
       <c r="G104" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="H104" t="n">
         <v>18</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>280</v>
+        <v>98</v>
       </c>
       <c r="K104" t="n">
-        <v>532</v>
+        <v>367.7</v>
       </c>
       <c r="L104" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="M104" t="n">
         <v>18</v>
@@ -9905,10 +9905,10 @@
       </c>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R104" t="n">
         <v>0</v>
@@ -9934,285 +9934,12 @@
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="Y104" t="inlineStr">
         <is>
           <t>9992609291037</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>104</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
-        </is>
-      </c>
-      <c r="D105" t="n">
-        <v>1</v>
-      </c>
-      <c r="E105" t="n">
-        <v>281</v>
-      </c>
-      <c r="F105" t="n">
-        <v>532</v>
-      </c>
-      <c r="G105" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H105" t="n">
-        <v>18</v>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>18_Melamina_BLANCO 18</t>
-        </is>
-      </c>
-      <c r="J105" t="n">
-        <v>280</v>
-      </c>
-      <c r="K105" t="n">
-        <v>532</v>
-      </c>
-      <c r="L105" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M105" t="n">
-        <v>18</v>
-      </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>9992609291044</t>
-        </is>
-      </c>
-      <c r="O105" t="inlineStr"/>
-      <c r="P105" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q105" t="n">
-        <v>1</v>
-      </c>
-      <c r="R105" t="n">
-        <v>0</v>
-      </c>
-      <c r="S105" t="n">
-        <v>0</v>
-      </c>
-      <c r="T105" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U105" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V105" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W105" t="inlineStr"/>
-      <c r="X105" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
-        </is>
-      </c>
-      <c r="Y105" t="inlineStr">
-        <is>
-          <t>9992609291044</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>105</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
-        </is>
-      </c>
-      <c r="D106" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" t="n">
-        <v>99</v>
-      </c>
-      <c r="F106" t="n">
-        <v>1407</v>
-      </c>
-      <c r="G106" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="H106" t="n">
-        <v>18</v>
-      </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>18_Melamina_VERDE 18</t>
-        </is>
-      </c>
-      <c r="J106" t="n">
-        <v>98</v>
-      </c>
-      <c r="K106" t="n">
-        <v>1407</v>
-      </c>
-      <c r="L106" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="M106" t="n">
-        <v>18</v>
-      </c>
-      <c r="N106" t="inlineStr">
-        <is>
-          <t>9992609291051</t>
-        </is>
-      </c>
-      <c r="O106" t="inlineStr"/>
-      <c r="P106" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q106" t="n">
-        <v>0</v>
-      </c>
-      <c r="R106" t="n">
-        <v>0</v>
-      </c>
-      <c r="S106" t="n">
-        <v>0</v>
-      </c>
-      <c r="T106" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U106" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V106" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W106" t="inlineStr"/>
-      <c r="X106" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
-        </is>
-      </c>
-      <c r="Y106" t="inlineStr">
-        <is>
-          <t>9992609291051</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="D107" t="n">
-        <v>1</v>
-      </c>
-      <c r="E107" t="n">
-        <v>99</v>
-      </c>
-      <c r="F107" t="n">
-        <v>367.7</v>
-      </c>
-      <c r="G107" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H107" t="n">
-        <v>18</v>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>18_Melamina_VERDE 18</t>
-        </is>
-      </c>
-      <c r="J107" t="n">
-        <v>98</v>
-      </c>
-      <c r="K107" t="n">
-        <v>367.7</v>
-      </c>
-      <c r="L107" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M107" t="n">
-        <v>18</v>
-      </c>
-      <c r="N107" t="inlineStr">
-        <is>
-          <t>9992609291068</t>
-        </is>
-      </c>
-      <c r="O107" t="inlineStr"/>
-      <c r="P107" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q107" t="n">
-        <v>0</v>
-      </c>
-      <c r="R107" t="n">
-        <v>0</v>
-      </c>
-      <c r="S107" t="n">
-        <v>0</v>
-      </c>
-      <c r="T107" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U107" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V107" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W107" t="inlineStr"/>
-      <c r="X107" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="Y107" t="inlineStr">
-        <is>
-          <t>9992609291068</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A2: hoja rebatible arriba (como la Spar) + 2 puertas abajo; 104/104 receta = sólido; paquete regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y104"/>
+  <dimension ref="A1:Y105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7140,10 +7140,10 @@
         <v>1</v>
       </c>
       <c r="E74" t="n">
+        <v>600</v>
+      </c>
+      <c r="F74" t="n">
         <v>332</v>
-      </c>
-      <c r="F74" t="n">
-        <v>600</v>
       </c>
       <c r="G74" t="n">
         <v>0.2</v>
@@ -7157,10 +7157,10 @@
         </is>
       </c>
       <c r="J74" t="n">
+        <v>600</v>
+      </c>
+      <c r="K74" t="n">
         <v>331</v>
-      </c>
-      <c r="K74" t="n">
-        <v>600</v>
       </c>
       <c r="L74" t="n">
         <v>0.2</v>
@@ -7175,7 +7175,7 @@
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q74" t="n">
         <v>0</v>
@@ -7184,7 +7184,7 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -7583,49 +7583,49 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>346</v>
+        <v>301</v>
       </c>
       <c r="F79" t="n">
-        <v>597</v>
+        <v>564</v>
       </c>
       <c r="G79" t="n">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="H79" t="n">
         <v>18</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>344</v>
+        <v>300</v>
       </c>
       <c r="K79" t="n">
-        <v>595</v>
+        <v>564</v>
       </c>
       <c r="L79" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="M79" t="n">
         <v>18</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>9992609290788</t>
+          <t>9992609290788_9992609290788</t>
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
@@ -7633,13 +7633,13 @@
         <v>1</v>
       </c>
       <c r="Q79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -7659,7 +7659,7 @@
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Frente fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
@@ -7674,60 +7674,60 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>564</v>
+        <v>597</v>
       </c>
       <c r="F80" t="n">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="G80" t="n">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="H80" t="n">
         <v>18</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>564</v>
+        <v>595</v>
       </c>
       <c r="K80" t="n">
-        <v>300</v>
+        <v>344</v>
       </c>
       <c r="L80" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="M80" t="n">
         <v>18</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>9992609290795_9992609290795_9992609290795K</t>
+          <t>9992609290795_9992609290795</t>
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S80" t="n">
         <v>1</v>
@@ -7750,7 +7750,7 @@
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -7765,25 +7765,25 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta der</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta der</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>597</v>
+        <v>688</v>
       </c>
       <c r="F81" t="n">
-        <v>688</v>
+        <v>297</v>
       </c>
       <c r="G81" t="n">
-        <v>0.41</v>
+        <v>0.2</v>
       </c>
       <c r="H81" t="n">
         <v>18</v>
@@ -7794,13 +7794,13 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>595</v>
+        <v>686</v>
       </c>
       <c r="K81" t="n">
-        <v>686</v>
+        <v>295</v>
       </c>
       <c r="L81" t="n">
-        <v>0.41</v>
+        <v>0.2</v>
       </c>
       <c r="M81" t="n">
         <v>18</v>
@@ -7841,7 +7841,7 @@
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta der</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -7856,63 +7856,63 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta izq</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta izq</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>281</v>
+        <v>688</v>
       </c>
       <c r="F82" t="n">
-        <v>562</v>
+        <v>297</v>
       </c>
       <c r="G82" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="H82" t="n">
         <v>18</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>280</v>
+        <v>686</v>
       </c>
       <c r="K82" t="n">
-        <v>562</v>
+        <v>295</v>
       </c>
       <c r="L82" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="M82" t="n">
         <v>18</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>9992609290818</t>
+          <t>9992609290818_9992609290818</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q82" t="n">
         <v>1</v>
       </c>
       <c r="R82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T82" t="inlineStr">
         <is>
@@ -7932,7 +7932,7 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta izq</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -7947,25 +7947,25 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>332</v>
+        <v>281</v>
       </c>
       <c r="F83" t="n">
-        <v>800</v>
+        <v>562</v>
       </c>
       <c r="G83" t="n">
-        <v>0.27</v>
+        <v>0.16</v>
       </c>
       <c r="H83" t="n">
         <v>18</v>
@@ -7976,20 +7976,20 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>331</v>
+        <v>280</v>
       </c>
       <c r="K83" t="n">
-        <v>800</v>
+        <v>562</v>
       </c>
       <c r="L83" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="M83" t="n">
         <v>18</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>9992609290825_9992609290825_9992609290825K</t>
+          <t>9992609290825</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
@@ -8023,7 +8023,7 @@
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -8038,12 +8038,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -8080,15 +8080,15 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>9992609290832_9992609290832</t>
+          <t>9992609290832_9992609290832_9992609290832K</t>
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R84" t="n">
         <v>0</v>
@@ -8114,7 +8114,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -8129,25 +8129,25 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
-        <v>1004</v>
+        <v>332</v>
       </c>
       <c r="F85" t="n">
-        <v>332</v>
+        <v>800</v>
       </c>
       <c r="G85" t="n">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
@@ -8158,13 +8158,13 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>1004</v>
+        <v>331</v>
       </c>
       <c r="K85" t="n">
-        <v>331</v>
+        <v>800</v>
       </c>
       <c r="L85" t="n">
-        <v>0.33</v>
+        <v>0.26</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
@@ -8176,7 +8176,7 @@
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q85" t="n">
         <v>0</v>
@@ -8185,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="S85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -8205,7 +8205,7 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -8220,12 +8220,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -8273,10 +8273,10 @@
         <v>0</v>
       </c>
       <c r="R86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8296,7 +8296,7 @@
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -8311,49 +8311,49 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>1014</v>
+        <v>1004</v>
       </c>
       <c r="F87" t="n">
-        <v>774</v>
+        <v>332</v>
       </c>
       <c r="G87" t="n">
-        <v>0.78</v>
+        <v>0.33</v>
       </c>
       <c r="H87" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>1014</v>
+        <v>1004</v>
       </c>
       <c r="K87" t="n">
-        <v>774</v>
+        <v>331</v>
       </c>
       <c r="L87" t="n">
-        <v>0.78</v>
+        <v>0.33</v>
       </c>
       <c r="M87" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>9992609290863</t>
+          <t>9992609290863_9992609290863</t>
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
@@ -8364,7 +8364,7 @@
         <v>0</v>
       </c>
       <c r="R87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S87" t="n">
         <v>0</v>
@@ -8387,7 +8387,7 @@
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -8402,49 +8402,49 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>80</v>
+        <v>1014</v>
       </c>
       <c r="F88" t="n">
-        <v>764</v>
+        <v>774</v>
       </c>
       <c r="G88" t="n">
-        <v>0.06</v>
+        <v>0.78</v>
       </c>
       <c r="H88" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>80</v>
+        <v>1014</v>
       </c>
       <c r="K88" t="n">
-        <v>764</v>
+        <v>774</v>
       </c>
       <c r="L88" t="n">
-        <v>0.06</v>
+        <v>0.78</v>
       </c>
       <c r="M88" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>9992609290870_9992609290870</t>
+          <t>9992609290870</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -8493,42 +8493,42 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>1037</v>
+        <v>80</v>
       </c>
       <c r="F89" t="n">
-        <v>397</v>
+        <v>764</v>
       </c>
       <c r="G89" t="n">
-        <v>0.41</v>
+        <v>0.06</v>
       </c>
       <c r="H89" t="n">
         <v>18</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>1035</v>
+        <v>80</v>
       </c>
       <c r="K89" t="n">
-        <v>395</v>
+        <v>764</v>
       </c>
       <c r="L89" t="n">
-        <v>0.41</v>
+        <v>0.06</v>
       </c>
       <c r="M89" t="n">
         <v>18</v>
@@ -8540,16 +8540,16 @@
       </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T89" t="inlineStr">
         <is>
@@ -8569,7 +8569,7 @@
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -8584,12 +8584,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -8660,7 +8660,7 @@
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr">
@@ -8675,63 +8675,63 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>281</v>
+        <v>1037</v>
       </c>
       <c r="F91" t="n">
-        <v>762</v>
+        <v>397</v>
       </c>
       <c r="G91" t="n">
-        <v>0.21</v>
+        <v>0.41</v>
       </c>
       <c r="H91" t="n">
         <v>18</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>280</v>
+        <v>1035</v>
       </c>
       <c r="K91" t="n">
-        <v>762</v>
+        <v>395</v>
       </c>
       <c r="L91" t="n">
-        <v>0.21</v>
+        <v>0.41</v>
       </c>
       <c r="M91" t="n">
         <v>18</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>9992609290900</t>
+          <t>9992609290900_9992609290900</t>
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q91" t="n">
         <v>1</v>
       </c>
       <c r="R91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T91" t="inlineStr">
         <is>
@@ -8751,7 +8751,7 @@
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -8766,12 +8766,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -8842,7 +8842,7 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -8857,25 +8857,25 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>332</v>
+        <v>281</v>
       </c>
       <c r="F93" t="n">
-        <v>570</v>
+        <v>762</v>
       </c>
       <c r="G93" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="H93" t="n">
         <v>18</v>
@@ -8886,20 +8886,20 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>331</v>
+        <v>280</v>
       </c>
       <c r="K93" t="n">
-        <v>570</v>
+        <v>762</v>
       </c>
       <c r="L93" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="M93" t="n">
         <v>18</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>9992609290924_9992609290924_9992609290924K</t>
+          <t>9992609290924</t>
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -8948,12 +8948,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -8990,15 +8990,15 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>9992609290931_9992609290931</t>
+          <t>9992609290931_9992609290931_9992609290931K</t>
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R94" t="n">
         <v>0</v>
@@ -9024,7 +9024,7 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -9039,25 +9039,25 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>1004</v>
+        <v>332</v>
       </c>
       <c r="F95" t="n">
-        <v>332</v>
+        <v>570</v>
       </c>
       <c r="G95" t="n">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="H95" t="n">
         <v>18</v>
@@ -9068,13 +9068,13 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>1004</v>
+        <v>331</v>
       </c>
       <c r="K95" t="n">
-        <v>331</v>
+        <v>570</v>
       </c>
       <c r="L95" t="n">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="M95" t="n">
         <v>18</v>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q95" t="n">
         <v>0</v>
@@ -9095,7 +9095,7 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T95" t="inlineStr">
         <is>
@@ -9115,7 +9115,7 @@
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -9130,12 +9130,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -9183,10 +9183,10 @@
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T96" t="inlineStr">
         <is>
@@ -9206,7 +9206,7 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -9221,49 +9221,49 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>1014</v>
+        <v>1004</v>
       </c>
       <c r="F97" t="n">
-        <v>544</v>
+        <v>332</v>
       </c>
       <c r="G97" t="n">
-        <v>0.55</v>
+        <v>0.33</v>
       </c>
       <c r="H97" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>1014</v>
+        <v>1004</v>
       </c>
       <c r="K97" t="n">
-        <v>544</v>
+        <v>331</v>
       </c>
       <c r="L97" t="n">
-        <v>0.55</v>
+        <v>0.33</v>
       </c>
       <c r="M97" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>9992609290962</t>
+          <t>9992609290962_9992609290962</t>
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
@@ -9274,7 +9274,7 @@
         <v>0</v>
       </c>
       <c r="R97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S97" t="n">
         <v>0</v>
@@ -9297,7 +9297,7 @@
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -9312,49 +9312,49 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>80</v>
+        <v>1014</v>
       </c>
       <c r="F98" t="n">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="G98" t="n">
-        <v>0.04</v>
+        <v>0.55</v>
       </c>
       <c r="H98" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>80</v>
+        <v>1014</v>
       </c>
       <c r="K98" t="n">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="L98" t="n">
-        <v>0.04</v>
+        <v>0.55</v>
       </c>
       <c r="M98" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>9992609290979_9992609290979</t>
+          <t>9992609290979</t>
         </is>
       </c>
       <c r="O98" t="inlineStr"/>
@@ -9388,7 +9388,7 @@
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -9403,42 +9403,42 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>1037</v>
+        <v>80</v>
       </c>
       <c r="F99" t="n">
-        <v>282</v>
+        <v>534</v>
       </c>
       <c r="G99" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="H99" t="n">
         <v>18</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>1035</v>
+        <v>80</v>
       </c>
       <c r="K99" t="n">
-        <v>280</v>
+        <v>534</v>
       </c>
       <c r="L99" t="n">
-        <v>0.29</v>
+        <v>0.04</v>
       </c>
       <c r="M99" t="n">
         <v>18</v>
@@ -9450,16 +9450,16 @@
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
@@ -9479,7 +9479,7 @@
       <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -9494,12 +9494,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -9570,7 +9570,7 @@
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -9585,63 +9585,63 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>281</v>
+        <v>1037</v>
       </c>
       <c r="F101" t="n">
-        <v>532</v>
+        <v>282</v>
       </c>
       <c r="G101" t="n">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="H101" t="n">
         <v>18</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J101" t="n">
+        <v>1035</v>
+      </c>
+      <c r="K101" t="n">
         <v>280</v>
       </c>
-      <c r="K101" t="n">
-        <v>532</v>
-      </c>
       <c r="L101" t="n">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="M101" t="n">
         <v>18</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>9992609291006</t>
+          <t>9992609291006_9992609291006</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q101" t="n">
         <v>1</v>
       </c>
       <c r="R101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T101" t="inlineStr">
         <is>
@@ -9661,7 +9661,7 @@
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -9676,12 +9676,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -9752,7 +9752,7 @@
       <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -9767,42 +9767,42 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>99</v>
+        <v>281</v>
       </c>
       <c r="F103" t="n">
-        <v>1407</v>
+        <v>532</v>
       </c>
       <c r="G103" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="H103" t="n">
         <v>18</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>98</v>
+        <v>280</v>
       </c>
       <c r="K103" t="n">
-        <v>1407</v>
+        <v>532</v>
       </c>
       <c r="L103" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="M103" t="n">
         <v>18</v>
@@ -9814,10 +9814,10 @@
       </c>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R103" t="n">
         <v>0</v>
@@ -9843,7 +9843,7 @@
       <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -9858,12 +9858,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -9873,10 +9873,10 @@
         <v>99</v>
       </c>
       <c r="F104" t="n">
-        <v>367.7</v>
+        <v>1407</v>
       </c>
       <c r="G104" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="H104" t="n">
         <v>18</v>
@@ -9890,10 +9890,10 @@
         <v>98</v>
       </c>
       <c r="K104" t="n">
-        <v>367.7</v>
+        <v>1407</v>
       </c>
       <c r="L104" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="M104" t="n">
         <v>18</v>
@@ -9934,12 +9934,103 @@
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr">
         <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>9992609291037</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
-      <c r="Y104" t="inlineStr">
-        <is>
-          <t>9992609291037</t>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" t="n">
+        <v>99</v>
+      </c>
+      <c r="F105" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H105" t="n">
+        <v>18</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>98</v>
+      </c>
+      <c r="K105" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M105" t="n">
+        <v>18</v>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>9992609291044</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr"/>
+      <c r="P105" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>9992609291044</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A2: dos hojas rebatibles hacia arriba (sin puertas dobles); 103/103 receta = sólido; paquete regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y105"/>
+  <dimension ref="A1:Y104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7595,10 +7595,10 @@
         <v>1</v>
       </c>
       <c r="E79" t="n">
+        <v>564</v>
+      </c>
+      <c r="F79" t="n">
         <v>301</v>
-      </c>
-      <c r="F79" t="n">
-        <v>564</v>
       </c>
       <c r="G79" t="n">
         <v>0.17</v>
@@ -7612,10 +7612,10 @@
         </is>
       </c>
       <c r="J79" t="n">
+        <v>564</v>
+      </c>
+      <c r="K79" t="n">
         <v>300</v>
-      </c>
-      <c r="K79" t="n">
-        <v>564</v>
       </c>
       <c r="L79" t="n">
         <v>0.17</v>
@@ -7625,12 +7625,12 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>9992609290788_9992609290788</t>
+          <t>9992609290788_9992609290788_9992609290788K</t>
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q79" t="n">
         <v>0</v>
@@ -7639,7 +7639,7 @@
         <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -7674,12 +7674,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -7750,7 +7750,7 @@
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -7765,25 +7765,25 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
+        <v>597</v>
+      </c>
+      <c r="F81" t="n">
         <v>688</v>
       </c>
-      <c r="F81" t="n">
-        <v>297</v>
-      </c>
       <c r="G81" t="n">
-        <v>0.2</v>
+        <v>0.41</v>
       </c>
       <c r="H81" t="n">
         <v>18</v>
@@ -7794,13 +7794,13 @@
         </is>
       </c>
       <c r="J81" t="n">
+        <v>595</v>
+      </c>
+      <c r="K81" t="n">
         <v>686</v>
       </c>
-      <c r="K81" t="n">
-        <v>295</v>
-      </c>
       <c r="L81" t="n">
-        <v>0.2</v>
+        <v>0.41</v>
       </c>
       <c r="M81" t="n">
         <v>18</v>
@@ -7841,7 +7841,7 @@
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -7856,63 +7856,63 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>688</v>
+        <v>281</v>
       </c>
       <c r="F82" t="n">
-        <v>297</v>
+        <v>562</v>
       </c>
       <c r="G82" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="H82" t="n">
         <v>18</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>686</v>
+        <v>280</v>
       </c>
       <c r="K82" t="n">
-        <v>295</v>
+        <v>562</v>
       </c>
       <c r="L82" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="M82" t="n">
         <v>18</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>9992609290818_9992609290818</t>
+          <t>9992609290818</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q82" t="n">
         <v>1</v>
       </c>
       <c r="R82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T82" t="inlineStr">
         <is>
@@ -7932,7 +7932,7 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -7947,25 +7947,25 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F83" t="n">
-        <v>562</v>
+        <v>800</v>
       </c>
       <c r="G83" t="n">
-        <v>0.16</v>
+        <v>0.27</v>
       </c>
       <c r="H83" t="n">
         <v>18</v>
@@ -7976,20 +7976,20 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K83" t="n">
-        <v>562</v>
+        <v>800</v>
       </c>
       <c r="L83" t="n">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="M83" t="n">
         <v>18</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>9992609290825</t>
+          <t>9992609290825_9992609290825_9992609290825K</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
@@ -8023,7 +8023,7 @@
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -8038,12 +8038,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -8080,15 +8080,15 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>9992609290832_9992609290832_9992609290832K</t>
+          <t>9992609290832_9992609290832</t>
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R84" t="n">
         <v>0</v>
@@ -8114,7 +8114,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -8129,25 +8129,25 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F85" t="n">
         <v>332</v>
       </c>
-      <c r="F85" t="n">
-        <v>800</v>
-      </c>
       <c r="G85" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
@@ -8158,13 +8158,13 @@
         </is>
       </c>
       <c r="J85" t="n">
+        <v>1004</v>
+      </c>
+      <c r="K85" t="n">
         <v>331</v>
       </c>
-      <c r="K85" t="n">
-        <v>800</v>
-      </c>
       <c r="L85" t="n">
-        <v>0.26</v>
+        <v>0.33</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
@@ -8176,7 +8176,7 @@
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q85" t="n">
         <v>0</v>
@@ -8185,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="S85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -8205,7 +8205,7 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -8220,12 +8220,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -8273,10 +8273,10 @@
         <v>0</v>
       </c>
       <c r="R86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8296,7 +8296,7 @@
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -8311,49 +8311,49 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>1004</v>
+        <v>1014</v>
       </c>
       <c r="F87" t="n">
-        <v>332</v>
+        <v>774</v>
       </c>
       <c r="G87" t="n">
-        <v>0.33</v>
+        <v>0.78</v>
       </c>
       <c r="H87" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>1004</v>
+        <v>1014</v>
       </c>
       <c r="K87" t="n">
-        <v>331</v>
+        <v>774</v>
       </c>
       <c r="L87" t="n">
-        <v>0.33</v>
+        <v>0.78</v>
       </c>
       <c r="M87" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>9992609290863_9992609290863</t>
+          <t>9992609290863</t>
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
@@ -8364,7 +8364,7 @@
         <v>0</v>
       </c>
       <c r="R87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S87" t="n">
         <v>0</v>
@@ -8387,7 +8387,7 @@
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -8402,49 +8402,49 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>1014</v>
+        <v>80</v>
       </c>
       <c r="F88" t="n">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="G88" t="n">
-        <v>0.78</v>
+        <v>0.06</v>
       </c>
       <c r="H88" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>1014</v>
+        <v>80</v>
       </c>
       <c r="K88" t="n">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="L88" t="n">
-        <v>0.78</v>
+        <v>0.06</v>
       </c>
       <c r="M88" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>9992609290870</t>
+          <t>9992609290870_9992609290870</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -8493,42 +8493,42 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>80</v>
+        <v>1037</v>
       </c>
       <c r="F89" t="n">
-        <v>764</v>
+        <v>397</v>
       </c>
       <c r="G89" t="n">
-        <v>0.06</v>
+        <v>0.41</v>
       </c>
       <c r="H89" t="n">
         <v>18</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>80</v>
+        <v>1035</v>
       </c>
       <c r="K89" t="n">
-        <v>764</v>
+        <v>395</v>
       </c>
       <c r="L89" t="n">
-        <v>0.06</v>
+        <v>0.41</v>
       </c>
       <c r="M89" t="n">
         <v>18</v>
@@ -8540,16 +8540,16 @@
       </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T89" t="inlineStr">
         <is>
@@ -8569,7 +8569,7 @@
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -8584,12 +8584,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -8660,7 +8660,7 @@
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr">
@@ -8675,63 +8675,63 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>1037</v>
+        <v>281</v>
       </c>
       <c r="F91" t="n">
-        <v>397</v>
+        <v>762</v>
       </c>
       <c r="G91" t="n">
-        <v>0.41</v>
+        <v>0.21</v>
       </c>
       <c r="H91" t="n">
         <v>18</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>1035</v>
+        <v>280</v>
       </c>
       <c r="K91" t="n">
-        <v>395</v>
+        <v>762</v>
       </c>
       <c r="L91" t="n">
-        <v>0.41</v>
+        <v>0.21</v>
       </c>
       <c r="M91" t="n">
         <v>18</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>9992609290900_9992609290900</t>
+          <t>9992609290900</t>
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q91" t="n">
         <v>1</v>
       </c>
       <c r="R91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T91" t="inlineStr">
         <is>
@@ -8751,7 +8751,7 @@
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -8766,12 +8766,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -8842,7 +8842,7 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -8857,25 +8857,25 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F93" t="n">
-        <v>762</v>
+        <v>570</v>
       </c>
       <c r="G93" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="H93" t="n">
         <v>18</v>
@@ -8886,20 +8886,20 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K93" t="n">
-        <v>762</v>
+        <v>570</v>
       </c>
       <c r="L93" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="M93" t="n">
         <v>18</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>9992609290924</t>
+          <t>9992609290924_9992609290924_9992609290924K</t>
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -8948,12 +8948,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -8990,15 +8990,15 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>9992609290931_9992609290931_9992609290931K</t>
+          <t>9992609290931_9992609290931</t>
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R94" t="n">
         <v>0</v>
@@ -9024,7 +9024,7 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -9039,25 +9039,25 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F95" t="n">
         <v>332</v>
       </c>
-      <c r="F95" t="n">
-        <v>570</v>
-      </c>
       <c r="G95" t="n">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="H95" t="n">
         <v>18</v>
@@ -9068,13 +9068,13 @@
         </is>
       </c>
       <c r="J95" t="n">
+        <v>1004</v>
+      </c>
+      <c r="K95" t="n">
         <v>331</v>
       </c>
-      <c r="K95" t="n">
-        <v>570</v>
-      </c>
       <c r="L95" t="n">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="M95" t="n">
         <v>18</v>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q95" t="n">
         <v>0</v>
@@ -9095,7 +9095,7 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T95" t="inlineStr">
         <is>
@@ -9115,7 +9115,7 @@
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -9130,12 +9130,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -9183,10 +9183,10 @@
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T96" t="inlineStr">
         <is>
@@ -9206,7 +9206,7 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -9221,49 +9221,49 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>1004</v>
+        <v>1014</v>
       </c>
       <c r="F97" t="n">
-        <v>332</v>
+        <v>544</v>
       </c>
       <c r="G97" t="n">
-        <v>0.33</v>
+        <v>0.55</v>
       </c>
       <c r="H97" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>1004</v>
+        <v>1014</v>
       </c>
       <c r="K97" t="n">
-        <v>331</v>
+        <v>544</v>
       </c>
       <c r="L97" t="n">
-        <v>0.33</v>
+        <v>0.55</v>
       </c>
       <c r="M97" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>9992609290962_9992609290962</t>
+          <t>9992609290962</t>
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
@@ -9274,7 +9274,7 @@
         <v>0</v>
       </c>
       <c r="R97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S97" t="n">
         <v>0</v>
@@ -9297,7 +9297,7 @@
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -9312,49 +9312,49 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>1014</v>
+        <v>80</v>
       </c>
       <c r="F98" t="n">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="G98" t="n">
-        <v>0.55</v>
+        <v>0.04</v>
       </c>
       <c r="H98" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>1014</v>
+        <v>80</v>
       </c>
       <c r="K98" t="n">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="L98" t="n">
-        <v>0.55</v>
+        <v>0.04</v>
       </c>
       <c r="M98" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>9992609290979</t>
+          <t>9992609290979_9992609290979</t>
         </is>
       </c>
       <c r="O98" t="inlineStr"/>
@@ -9388,7 +9388,7 @@
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -9403,42 +9403,42 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>80</v>
+        <v>1037</v>
       </c>
       <c r="F99" t="n">
-        <v>534</v>
+        <v>282</v>
       </c>
       <c r="G99" t="n">
-        <v>0.04</v>
+        <v>0.29</v>
       </c>
       <c r="H99" t="n">
         <v>18</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>80</v>
+        <v>1035</v>
       </c>
       <c r="K99" t="n">
-        <v>534</v>
+        <v>280</v>
       </c>
       <c r="L99" t="n">
-        <v>0.04</v>
+        <v>0.29</v>
       </c>
       <c r="M99" t="n">
         <v>18</v>
@@ -9450,16 +9450,16 @@
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
@@ -9479,7 +9479,7 @@
       <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -9494,12 +9494,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -9570,7 +9570,7 @@
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -9585,63 +9585,63 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>1037</v>
+        <v>281</v>
       </c>
       <c r="F101" t="n">
-        <v>282</v>
+        <v>532</v>
       </c>
       <c r="G101" t="n">
-        <v>0.29</v>
+        <v>0.15</v>
       </c>
       <c r="H101" t="n">
         <v>18</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>1035</v>
+        <v>280</v>
       </c>
       <c r="K101" t="n">
-        <v>280</v>
+        <v>532</v>
       </c>
       <c r="L101" t="n">
-        <v>0.29</v>
+        <v>0.15</v>
       </c>
       <c r="M101" t="n">
         <v>18</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>9992609291006_9992609291006</t>
+          <t>9992609291006</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q101" t="n">
         <v>1</v>
       </c>
       <c r="R101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T101" t="inlineStr">
         <is>
@@ -9661,7 +9661,7 @@
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -9676,12 +9676,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -9752,7 +9752,7 @@
       <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -9767,42 +9767,42 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>281</v>
+        <v>99</v>
       </c>
       <c r="F103" t="n">
-        <v>532</v>
+        <v>1407</v>
       </c>
       <c r="G103" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="H103" t="n">
         <v>18</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>280</v>
+        <v>98</v>
       </c>
       <c r="K103" t="n">
-        <v>532</v>
+        <v>1407</v>
       </c>
       <c r="L103" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="M103" t="n">
         <v>18</v>
@@ -9814,10 +9814,10 @@
       </c>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R103" t="n">
         <v>0</v>
@@ -9843,7 +9843,7 @@
       <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -9858,12 +9858,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -9873,10 +9873,10 @@
         <v>99</v>
       </c>
       <c r="F104" t="n">
-        <v>1407</v>
+        <v>367.7</v>
       </c>
       <c r="G104" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="H104" t="n">
         <v>18</v>
@@ -9890,10 +9890,10 @@
         <v>98</v>
       </c>
       <c r="K104" t="n">
-        <v>1407</v>
+        <v>367.7</v>
       </c>
       <c r="L104" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="M104" t="n">
         <v>18</v>
@@ -9934,103 +9934,12 @@
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="Y104" t="inlineStr">
         <is>
           <t>9992609291037</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>104</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="D105" t="n">
-        <v>1</v>
-      </c>
-      <c r="E105" t="n">
-        <v>99</v>
-      </c>
-      <c r="F105" t="n">
-        <v>367.7</v>
-      </c>
-      <c r="G105" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H105" t="n">
-        <v>18</v>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>18_Melamina_VERDE 18</t>
-        </is>
-      </c>
-      <c r="J105" t="n">
-        <v>98</v>
-      </c>
-      <c r="K105" t="n">
-        <v>367.7</v>
-      </c>
-      <c r="L105" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M105" t="n">
-        <v>18</v>
-      </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>9992609291044</t>
-        </is>
-      </c>
-      <c r="O105" t="inlineStr"/>
-      <c r="P105" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q105" t="n">
-        <v>0</v>
-      </c>
-      <c r="R105" t="n">
-        <v>0</v>
-      </c>
-      <c r="S105" t="n">
-        <v>0</v>
-      </c>
-      <c r="T105" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U105" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V105" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W105" t="inlineStr"/>
-      <c r="X105" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="Y105" t="inlineStr">
-        <is>
-          <t>9992609291044</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vitrinas de madera maciza (marco de 4 piezas con Minifix + tarugo, vidrio en ranura, cruz de listones), A4 una puerta, A2 45/55; ExportarPiezas: el O8 de canto solo se estira a 33 si desemboca en la excentrica; 114/114 receta = solido; paquete regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,19 +413,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y104"/>
+  <dimension ref="A1:Y115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="4" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="5" customWidth="1" min="13" max="13"/>
@@ -6582,12 +6582,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta montante izq</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta montante izq</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -6597,27 +6597,27 @@
         <v>1037</v>
       </c>
       <c r="F68" t="n">
-        <v>633.4</v>
+        <v>60</v>
       </c>
       <c r="G68" t="n">
-        <v>0.66</v>
+        <v>0.06</v>
       </c>
       <c r="H68" t="n">
         <v>18</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="K68" t="n">
-        <v>631.4</v>
+        <v>60</v>
       </c>
       <c r="L68" t="n">
-        <v>0.65</v>
+        <v>0.06</v>
       </c>
       <c r="M68" t="n">
         <v>18</v>
@@ -6629,16 +6629,16 @@
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T68" t="inlineStr">
         <is>
@@ -6658,7 +6658,7 @@
       <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Puerta</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta montante izq</t>
         </is>
       </c>
       <c r="Y68" t="inlineStr">
@@ -6673,49 +6673,49 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta montante der</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta montante der</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>750</v>
+        <v>1037</v>
       </c>
       <c r="F69" t="n">
-        <v>750</v>
+        <v>60</v>
       </c>
       <c r="G69" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="H69" t="n">
         <v>18</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>750</v>
+        <v>1037</v>
       </c>
       <c r="K69" t="n">
-        <v>750</v>
+        <v>60</v>
       </c>
       <c r="L69" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="M69" t="n">
         <v>18</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>9992609290689</t>
+          <t>9992609290689_9992609290689</t>
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
@@ -6749,7 +6749,7 @@
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta montante der</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr">
@@ -6764,49 +6764,49 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta travesano abajo</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta travesano abajo</t>
         </is>
       </c>
       <c r="D70" t="n">
         <v>1</v>
       </c>
       <c r="E70" t="n">
-        <v>750</v>
+        <v>513.4</v>
       </c>
       <c r="F70" t="n">
-        <v>750</v>
+        <v>70</v>
       </c>
       <c r="G70" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="H70" t="n">
         <v>18</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>750</v>
+        <v>513.4</v>
       </c>
       <c r="K70" t="n">
-        <v>750</v>
+        <v>70</v>
       </c>
       <c r="L70" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="M70" t="n">
         <v>18</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>9992609290696</t>
+          <t>9992609290696_9992609290696</t>
         </is>
       </c>
       <c r="O70" t="inlineStr"/>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="T70" t="inlineStr">
         <is>
-          <t>竖纹</t>
+          <t>横纹</t>
         </is>
       </c>
       <c r="U70" t="inlineStr">
@@ -6840,7 +6840,7 @@
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta travesano abajo</t>
         </is>
       </c>
       <c r="Y70" t="inlineStr">
@@ -6855,42 +6855,42 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta travesano arriba</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta travesano arriba</t>
         </is>
       </c>
       <c r="D71" t="n">
         <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>80</v>
+        <v>513.4</v>
       </c>
       <c r="F71" t="n">
-        <v>751</v>
+        <v>70</v>
       </c>
       <c r="G71" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H71" t="n">
         <v>18</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>80</v>
+        <v>513.4</v>
       </c>
       <c r="K71" t="n">
-        <v>751</v>
+        <v>70</v>
       </c>
       <c r="L71" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="M71" t="n">
         <v>18</v>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="T71" t="inlineStr">
         <is>
-          <t>竖纹</t>
+          <t>横纹</t>
         </is>
       </c>
       <c r="U71" t="inlineStr">
@@ -6931,7 +6931,7 @@
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
+          <t>COCINA-01_A1 Esquinero alacena_Puerta travesano arriba</t>
         </is>
       </c>
       <c r="Y71" t="inlineStr">
@@ -6946,25 +6946,25 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>80</v>
+        <v>750</v>
       </c>
       <c r="F72" t="n">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G72" t="n">
-        <v>0.06</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H72" t="n">
         <v>18</v>
@@ -6975,20 +6975,20 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>80</v>
+        <v>750</v>
       </c>
       <c r="K72" t="n">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="L72" t="n">
-        <v>0.06</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M72" t="n">
         <v>18</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>9992609290719_9992609290719</t>
+          <t>9992609290719</t>
         </is>
       </c>
       <c r="O72" t="inlineStr"/>
@@ -7022,7 +7022,7 @@
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr">
         <is>
-          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 1</t>
         </is>
       </c>
       <c r="Y72" t="inlineStr">
@@ -7037,25 +7037,25 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
         </is>
       </c>
       <c r="D73" t="n">
         <v>1</v>
       </c>
       <c r="E73" t="n">
-        <v>332</v>
+        <v>750</v>
       </c>
       <c r="F73" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="G73" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H73" t="n">
         <v>18</v>
@@ -7066,20 +7066,20 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>331</v>
+        <v>750</v>
       </c>
       <c r="K73" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="L73" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M73" t="n">
         <v>18</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>9992609290726_9992609290726_9992609290726K</t>
+          <t>9992609290726</t>
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
@@ -7087,7 +7087,7 @@
         <v>0</v>
       </c>
       <c r="Q73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R73" t="n">
         <v>0</v>
@@ -7113,7 +7113,7 @@
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
+          <t>COCINA-01_A1 Esquinero alacena_Estante 2</t>
         </is>
       </c>
       <c r="Y73" t="inlineStr">
@@ -7128,25 +7128,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
         </is>
       </c>
       <c r="D74" t="n">
         <v>1</v>
       </c>
       <c r="E74" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="F74" t="n">
-        <v>332</v>
+        <v>751</v>
       </c>
       <c r="G74" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="H74" t="n">
         <v>18</v>
@@ -7157,13 +7157,13 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="K74" t="n">
-        <v>331</v>
+        <v>751</v>
       </c>
       <c r="L74" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="M74" t="n">
         <v>18</v>
@@ -7184,7 +7184,7 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -7204,7 +7204,7 @@
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano A</t>
         </is>
       </c>
       <c r="Y74" t="inlineStr">
@@ -7219,25 +7219,25 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
         </is>
       </c>
       <c r="D75" t="n">
         <v>1</v>
       </c>
       <c r="E75" t="n">
-        <v>1004</v>
+        <v>80</v>
       </c>
       <c r="F75" t="n">
-        <v>332</v>
+        <v>751</v>
       </c>
       <c r="G75" t="n">
-        <v>0.33</v>
+        <v>0.06</v>
       </c>
       <c r="H75" t="n">
         <v>18</v>
@@ -7248,13 +7248,13 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>1004</v>
+        <v>80</v>
       </c>
       <c r="K75" t="n">
-        <v>331</v>
+        <v>751</v>
       </c>
       <c r="L75" t="n">
-        <v>0.33</v>
+        <v>0.06</v>
       </c>
       <c r="M75" t="n">
         <v>18</v>
@@ -7275,7 +7275,7 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T75" t="inlineStr">
         <is>
@@ -7295,7 +7295,7 @@
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
+          <t>COCINA-01_A1 Esquinero alacena_Travesano B</t>
         </is>
       </c>
       <c r="Y75" t="inlineStr">
@@ -7310,25 +7310,25 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
         </is>
       </c>
       <c r="D76" t="n">
         <v>1</v>
       </c>
       <c r="E76" t="n">
-        <v>1004</v>
+        <v>332</v>
       </c>
       <c r="F76" t="n">
-        <v>332</v>
+        <v>600</v>
       </c>
       <c r="G76" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="H76" t="n">
         <v>18</v>
@@ -7339,20 +7339,20 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>1004</v>
+        <v>331</v>
       </c>
       <c r="K76" t="n">
-        <v>331</v>
+        <v>600</v>
       </c>
       <c r="L76" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="M76" t="n">
         <v>18</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>9992609290757_9992609290757</t>
+          <t>9992609290757_9992609290757_9992609290757K</t>
         </is>
       </c>
       <c r="O76" t="inlineStr"/>
@@ -7360,10 +7360,10 @@
         <v>0</v>
       </c>
       <c r="Q76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S76" t="n">
         <v>0</v>
@@ -7386,7 +7386,7 @@
       <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
@@ -7401,49 +7401,49 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
         </is>
       </c>
       <c r="D77" t="n">
         <v>1</v>
       </c>
       <c r="E77" t="n">
-        <v>1014</v>
+        <v>600</v>
       </c>
       <c r="F77" t="n">
-        <v>574</v>
+        <v>332</v>
       </c>
       <c r="G77" t="n">
-        <v>0.58</v>
+        <v>0.2</v>
       </c>
       <c r="H77" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>1014</v>
+        <v>600</v>
       </c>
       <c r="K77" t="n">
-        <v>574</v>
+        <v>331</v>
       </c>
       <c r="L77" t="n">
-        <v>0.58</v>
+        <v>0.2</v>
       </c>
       <c r="M77" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>9992609290764</t>
+          <t>9992609290764_9992609290764</t>
         </is>
       </c>
       <c r="O77" t="inlineStr"/>
@@ -7457,7 +7457,7 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -7477,7 +7477,7 @@
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Techo</t>
         </is>
       </c>
       <c r="Y77" t="inlineStr">
@@ -7492,25 +7492,25 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
         </is>
       </c>
       <c r="D78" t="n">
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>80</v>
+        <v>1004</v>
       </c>
       <c r="F78" t="n">
-        <v>564</v>
+        <v>332</v>
       </c>
       <c r="G78" t="n">
-        <v>0.05</v>
+        <v>0.33</v>
       </c>
       <c r="H78" t="n">
         <v>18</v>
@@ -7521,13 +7521,13 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>80</v>
+        <v>1004</v>
       </c>
       <c r="K78" t="n">
-        <v>564</v>
+        <v>331</v>
       </c>
       <c r="L78" t="n">
-        <v>0.05</v>
+        <v>0.33</v>
       </c>
       <c r="M78" t="n">
         <v>18</v>
@@ -7548,7 +7548,7 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -7568,7 +7568,7 @@
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral der</t>
         </is>
       </c>
       <c r="Y78" t="inlineStr">
@@ -7583,25 +7583,25 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>564</v>
+        <v>1004</v>
       </c>
       <c r="F79" t="n">
-        <v>301</v>
+        <v>332</v>
       </c>
       <c r="G79" t="n">
-        <v>0.17</v>
+        <v>0.33</v>
       </c>
       <c r="H79" t="n">
         <v>18</v>
@@ -7612,20 +7612,20 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>564</v>
+        <v>1004</v>
       </c>
       <c r="K79" t="n">
-        <v>300</v>
+        <v>331</v>
       </c>
       <c r="L79" t="n">
-        <v>0.17</v>
+        <v>0.33</v>
       </c>
       <c r="M79" t="n">
         <v>18</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>9992609290788_9992609290788_9992609290788K</t>
+          <t>9992609290788_9992609290788</t>
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
@@ -7636,10 +7636,10 @@
         <v>0</v>
       </c>
       <c r="R79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -7659,7 +7659,7 @@
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Lateral izq</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
@@ -7674,63 +7674,63 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>597</v>
+        <v>1014</v>
       </c>
       <c r="F80" t="n">
-        <v>346</v>
+        <v>574</v>
       </c>
       <c r="G80" t="n">
-        <v>0.21</v>
+        <v>0.58</v>
       </c>
       <c r="H80" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>595</v>
+        <v>1014</v>
       </c>
       <c r="K80" t="n">
-        <v>344</v>
+        <v>574</v>
       </c>
       <c r="L80" t="n">
-        <v>0.2</v>
+        <v>0.58</v>
       </c>
       <c r="M80" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>9992609290795_9992609290795</t>
+          <t>9992609290795</t>
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T80" t="inlineStr">
         <is>
@@ -7750,7 +7750,7 @@
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Fondo</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -7765,42 +7765,42 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>597</v>
+        <v>80</v>
       </c>
       <c r="F81" t="n">
-        <v>688</v>
+        <v>564</v>
       </c>
       <c r="G81" t="n">
-        <v>0.41</v>
+        <v>0.05</v>
       </c>
       <c r="H81" t="n">
         <v>18</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>595</v>
+        <v>80</v>
       </c>
       <c r="K81" t="n">
-        <v>686</v>
+        <v>564</v>
       </c>
       <c r="L81" t="n">
-        <v>0.41</v>
+        <v>0.05</v>
       </c>
       <c r="M81" t="n">
         <v>18</v>
@@ -7812,16 +7812,16 @@
       </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -7841,7 +7841,7 @@
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -7856,25 +7856,25 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>281</v>
+        <v>564</v>
       </c>
       <c r="F82" t="n">
-        <v>562</v>
+        <v>301</v>
       </c>
       <c r="G82" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="H82" t="n">
         <v>18</v>
@@ -7885,20 +7885,20 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>280</v>
+        <v>564</v>
       </c>
       <c r="K82" t="n">
-        <v>562</v>
+        <v>300</v>
       </c>
       <c r="L82" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="M82" t="n">
         <v>18</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>9992609290818</t>
+          <t>9992609290818_9992609290818_9992609290818K</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
@@ -7906,13 +7906,13 @@
         <v>0</v>
       </c>
       <c r="Q82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R82" t="n">
         <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T82" t="inlineStr">
         <is>
@@ -7932,7 +7932,7 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -7947,63 +7947,63 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>332</v>
+        <v>597</v>
       </c>
       <c r="F83" t="n">
-        <v>800</v>
+        <v>467</v>
       </c>
       <c r="G83" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="H83" t="n">
         <v>18</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>331</v>
+        <v>595</v>
       </c>
       <c r="K83" t="n">
-        <v>800</v>
+        <v>465</v>
       </c>
       <c r="L83" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="M83" t="n">
         <v>18</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>9992609290825_9992609290825_9992609290825K</t>
+          <t>9992609290825_9992609290825</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q83" t="n">
         <v>1</v>
       </c>
       <c r="R83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T83" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -8038,42 +8038,42 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>1</v>
       </c>
       <c r="E84" t="n">
-        <v>332</v>
+        <v>597</v>
       </c>
       <c r="F84" t="n">
-        <v>800</v>
+        <v>567</v>
       </c>
       <c r="G84" t="n">
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
       <c r="H84" t="n">
         <v>18</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>331</v>
+        <v>595</v>
       </c>
       <c r="K84" t="n">
-        <v>800</v>
+        <v>565</v>
       </c>
       <c r="L84" t="n">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="M84" t="n">
         <v>18</v>
@@ -8088,13 +8088,13 @@
         <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T84" t="inlineStr">
         <is>
@@ -8114,7 +8114,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Techo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -8129,25 +8129,25 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
-        <v>1004</v>
+        <v>281</v>
       </c>
       <c r="F85" t="n">
-        <v>332</v>
+        <v>562</v>
       </c>
       <c r="G85" t="n">
-        <v>0.33</v>
+        <v>0.16</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
@@ -8158,20 +8158,20 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>1004</v>
+        <v>280</v>
       </c>
       <c r="K85" t="n">
-        <v>331</v>
+        <v>562</v>
       </c>
       <c r="L85" t="n">
-        <v>0.33</v>
+        <v>0.16</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>9992609290849_9992609290849</t>
+          <t>9992609290849</t>
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
@@ -8179,13 +8179,13 @@
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R85" t="n">
         <v>0</v>
       </c>
       <c r="S85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -8205,7 +8205,7 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -8220,25 +8220,25 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>1004</v>
+        <v>332</v>
       </c>
       <c r="F86" t="n">
-        <v>332</v>
+        <v>800</v>
       </c>
       <c r="G86" t="n">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="H86" t="n">
         <v>18</v>
@@ -8249,20 +8249,20 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>1004</v>
+        <v>331</v>
       </c>
       <c r="K86" t="n">
-        <v>331</v>
+        <v>800</v>
       </c>
       <c r="L86" t="n">
-        <v>0.33</v>
+        <v>0.26</v>
       </c>
       <c r="M86" t="n">
         <v>18</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>9992609290856_9992609290856</t>
+          <t>9992609290856_9992609290856_9992609290856K</t>
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
@@ -8270,10 +8270,10 @@
         <v>0</v>
       </c>
       <c r="Q86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S86" t="n">
         <v>0</v>
@@ -8296,7 +8296,7 @@
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Piso</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -8311,54 +8311,54 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>1014</v>
+        <v>332</v>
       </c>
       <c r="F87" t="n">
-        <v>774</v>
+        <v>800</v>
       </c>
       <c r="G87" t="n">
-        <v>0.78</v>
+        <v>0.27</v>
       </c>
       <c r="H87" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>1014</v>
+        <v>331</v>
       </c>
       <c r="K87" t="n">
-        <v>774</v>
+        <v>800</v>
       </c>
       <c r="L87" t="n">
-        <v>0.78</v>
+        <v>0.26</v>
       </c>
       <c r="M87" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>9992609290863</t>
+          <t>9992609290863_9992609290863</t>
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q87" t="n">
         <v>0</v>
@@ -8387,7 +8387,7 @@
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Techo</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -8402,25 +8402,25 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>80</v>
+        <v>1004</v>
       </c>
       <c r="F88" t="n">
-        <v>764</v>
+        <v>332</v>
       </c>
       <c r="G88" t="n">
-        <v>0.06</v>
+        <v>0.33</v>
       </c>
       <c r="H88" t="n">
         <v>18</v>
@@ -8431,13 +8431,13 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>80</v>
+        <v>1004</v>
       </c>
       <c r="K88" t="n">
-        <v>764</v>
+        <v>331</v>
       </c>
       <c r="L88" t="n">
-        <v>0.06</v>
+        <v>0.33</v>
       </c>
       <c r="M88" t="n">
         <v>18</v>
@@ -8458,7 +8458,7 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T88" t="inlineStr">
         <is>
@@ -8478,7 +8478,7 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral der</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -8493,42 +8493,42 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>1037</v>
+        <v>1004</v>
       </c>
       <c r="F89" t="n">
-        <v>397</v>
+        <v>332</v>
       </c>
       <c r="G89" t="n">
-        <v>0.41</v>
+        <v>0.33</v>
       </c>
       <c r="H89" t="n">
         <v>18</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>1035</v>
+        <v>1004</v>
       </c>
       <c r="K89" t="n">
-        <v>395</v>
+        <v>331</v>
       </c>
       <c r="L89" t="n">
-        <v>0.41</v>
+        <v>0.33</v>
       </c>
       <c r="M89" t="n">
         <v>18</v>
@@ -8540,16 +8540,16 @@
       </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R89" t="n">
         <v>1</v>
       </c>
       <c r="S89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T89" t="inlineStr">
         <is>
@@ -8569,7 +8569,7 @@
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Lateral izq</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -8584,63 +8584,63 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="D90" t="n">
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>1037</v>
+        <v>1014</v>
       </c>
       <c r="F90" t="n">
-        <v>397</v>
+        <v>774</v>
       </c>
       <c r="G90" t="n">
-        <v>0.41</v>
+        <v>0.78</v>
       </c>
       <c r="H90" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>1035</v>
+        <v>1014</v>
       </c>
       <c r="K90" t="n">
-        <v>395</v>
+        <v>774</v>
       </c>
       <c r="L90" t="n">
-        <v>0.41</v>
+        <v>0.78</v>
       </c>
       <c r="M90" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>9992609290894_9992609290894</t>
+          <t>9992609290894</t>
         </is>
       </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T90" t="inlineStr">
         <is>
@@ -8660,7 +8660,7 @@
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Fondo</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr">
@@ -8675,25 +8675,25 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>281</v>
+        <v>80</v>
       </c>
       <c r="F91" t="n">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="G91" t="n">
-        <v>0.21</v>
+        <v>0.06</v>
       </c>
       <c r="H91" t="n">
         <v>18</v>
@@ -8704,20 +8704,20 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>280</v>
+        <v>80</v>
       </c>
       <c r="K91" t="n">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="L91" t="n">
-        <v>0.21</v>
+        <v>0.06</v>
       </c>
       <c r="M91" t="n">
         <v>18</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>9992609290900</t>
+          <t>9992609290900_9992609290900</t>
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
@@ -8725,7 +8725,7 @@
         <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R91" t="n">
         <v>0</v>
@@ -8751,7 +8751,7 @@
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Travesano trasero</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -8766,49 +8766,49 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der montante izq</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der montante izq</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>281</v>
+        <v>1037</v>
       </c>
       <c r="F92" t="n">
-        <v>762</v>
+        <v>60</v>
       </c>
       <c r="G92" t="n">
-        <v>0.21</v>
+        <v>0.06</v>
       </c>
       <c r="H92" t="n">
         <v>18</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>280</v>
+        <v>1037</v>
       </c>
       <c r="K92" t="n">
-        <v>762</v>
+        <v>60</v>
       </c>
       <c r="L92" t="n">
-        <v>0.21</v>
+        <v>0.06</v>
       </c>
       <c r="M92" t="n">
         <v>18</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>9992609290917</t>
+          <t>9992609290917_9992609290917</t>
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
@@ -8816,7 +8816,7 @@
         <v>0</v>
       </c>
       <c r="Q92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R92" t="n">
         <v>0</v>
@@ -8842,7 +8842,7 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der montante izq</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -8857,49 +8857,49 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der montante der</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der montante der</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>332</v>
+        <v>1037</v>
       </c>
       <c r="F93" t="n">
-        <v>570</v>
+        <v>60</v>
       </c>
       <c r="G93" t="n">
-        <v>0.19</v>
+        <v>0.06</v>
       </c>
       <c r="H93" t="n">
         <v>18</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>331</v>
+        <v>1037</v>
       </c>
       <c r="K93" t="n">
-        <v>570</v>
+        <v>60</v>
       </c>
       <c r="L93" t="n">
-        <v>0.19</v>
+        <v>0.06</v>
       </c>
       <c r="M93" t="n">
         <v>18</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>9992609290924_9992609290924_9992609290924K</t>
+          <t>9992609290924_9992609290924</t>
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
@@ -8907,7 +8907,7 @@
         <v>0</v>
       </c>
       <c r="Q93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R93" t="n">
         <v>0</v>
@@ -8933,7 +8933,7 @@
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der montante der</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -8948,42 +8948,42 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano abajo</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano abajo</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>332</v>
+        <v>277</v>
       </c>
       <c r="F94" t="n">
-        <v>570</v>
+        <v>70</v>
       </c>
       <c r="G94" t="n">
-        <v>0.19</v>
+        <v>0.02</v>
       </c>
       <c r="H94" t="n">
         <v>18</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>331</v>
+        <v>277</v>
       </c>
       <c r="K94" t="n">
-        <v>570</v>
+        <v>70</v>
       </c>
       <c r="L94" t="n">
-        <v>0.19</v>
+        <v>0.02</v>
       </c>
       <c r="M94" t="n">
         <v>18</v>
@@ -8995,7 +8995,7 @@
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q94" t="n">
         <v>0</v>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="T94" t="inlineStr">
         <is>
-          <t>竖纹</t>
+          <t>横纹</t>
         </is>
       </c>
       <c r="U94" t="inlineStr">
@@ -9024,7 +9024,7 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano abajo</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -9039,42 +9039,42 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano arriba</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano arriba</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>1004</v>
+        <v>277</v>
       </c>
       <c r="F95" t="n">
-        <v>332</v>
+        <v>70</v>
       </c>
       <c r="G95" t="n">
-        <v>0.33</v>
+        <v>0.02</v>
       </c>
       <c r="H95" t="n">
         <v>18</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>1004</v>
+        <v>277</v>
       </c>
       <c r="K95" t="n">
-        <v>331</v>
+        <v>70</v>
       </c>
       <c r="L95" t="n">
-        <v>0.33</v>
+        <v>0.02</v>
       </c>
       <c r="M95" t="n">
         <v>18</v>
@@ -9095,11 +9095,11 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T95" t="inlineStr">
         <is>
-          <t>竖纹</t>
+          <t>横纹</t>
         </is>
       </c>
       <c r="U95" t="inlineStr">
@@ -9115,7 +9115,7 @@
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano arriba</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -9130,42 +9130,42 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante izq</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante izq</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>1004</v>
+        <v>1037</v>
       </c>
       <c r="F96" t="n">
-        <v>332</v>
+        <v>60</v>
       </c>
       <c r="G96" t="n">
-        <v>0.33</v>
+        <v>0.06</v>
       </c>
       <c r="H96" t="n">
         <v>18</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>1004</v>
+        <v>1037</v>
       </c>
       <c r="K96" t="n">
-        <v>331</v>
+        <v>60</v>
       </c>
       <c r="L96" t="n">
-        <v>0.33</v>
+        <v>0.06</v>
       </c>
       <c r="M96" t="n">
         <v>18</v>
@@ -9183,7 +9183,7 @@
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S96" t="n">
         <v>0</v>
@@ -9206,7 +9206,7 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante izq</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -9221,49 +9221,49 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante der</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante der</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>1014</v>
+        <v>1037</v>
       </c>
       <c r="F97" t="n">
-        <v>544</v>
+        <v>60</v>
       </c>
       <c r="G97" t="n">
-        <v>0.55</v>
+        <v>0.06</v>
       </c>
       <c r="H97" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>1014</v>
+        <v>1037</v>
       </c>
       <c r="K97" t="n">
-        <v>544</v>
+        <v>60</v>
       </c>
       <c r="L97" t="n">
-        <v>0.55</v>
+        <v>0.06</v>
       </c>
       <c r="M97" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>9992609290962</t>
+          <t>9992609290962_9992609290962</t>
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
@@ -9297,7 +9297,7 @@
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante der</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -9312,42 +9312,42 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano abajo</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano abajo</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>80</v>
+        <v>277</v>
       </c>
       <c r="F98" t="n">
-        <v>534</v>
+        <v>70</v>
       </c>
       <c r="G98" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="H98" t="n">
         <v>18</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>80</v>
+        <v>277</v>
       </c>
       <c r="K98" t="n">
-        <v>534</v>
+        <v>70</v>
       </c>
       <c r="L98" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="M98" t="n">
         <v>18</v>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>竖纹</t>
+          <t>横纹</t>
         </is>
       </c>
       <c r="U98" t="inlineStr">
@@ -9388,7 +9388,7 @@
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano abajo</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -9403,42 +9403,42 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano arriba</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano arriba</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>1037</v>
+        <v>277</v>
       </c>
       <c r="F99" t="n">
-        <v>282</v>
+        <v>70</v>
       </c>
       <c r="G99" t="n">
-        <v>0.29</v>
+        <v>0.02</v>
       </c>
       <c r="H99" t="n">
         <v>18</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>1035</v>
+        <v>277</v>
       </c>
       <c r="K99" t="n">
-        <v>280</v>
+        <v>70</v>
       </c>
       <c r="L99" t="n">
-        <v>0.29</v>
+        <v>0.02</v>
       </c>
       <c r="M99" t="n">
         <v>18</v>
@@ -9450,20 +9450,20 @@
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
-          <t>竖纹</t>
+          <t>横纹</t>
         </is>
       </c>
       <c r="U99" t="inlineStr">
@@ -9479,7 +9479,7 @@
       <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano arriba</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -9494,63 +9494,63 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>1037</v>
+        <v>281</v>
       </c>
       <c r="F100" t="n">
-        <v>282</v>
+        <v>762</v>
       </c>
       <c r="G100" t="n">
-        <v>0.29</v>
+        <v>0.21</v>
       </c>
       <c r="H100" t="n">
         <v>18</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>1035</v>
+        <v>280</v>
       </c>
       <c r="K100" t="n">
-        <v>280</v>
+        <v>762</v>
       </c>
       <c r="L100" t="n">
-        <v>0.29</v>
+        <v>0.21</v>
       </c>
       <c r="M100" t="n">
         <v>18</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>9992609290993_9992609290993</t>
+          <t>9992609290993</t>
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q100" t="n">
         <v>1</v>
       </c>
       <c r="R100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T100" t="inlineStr">
         <is>
@@ -9570,7 +9570,7 @@
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -9585,12 +9585,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -9600,10 +9600,10 @@
         <v>281</v>
       </c>
       <c r="F101" t="n">
-        <v>532</v>
+        <v>762</v>
       </c>
       <c r="G101" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="H101" t="n">
         <v>18</v>
@@ -9617,10 +9617,10 @@
         <v>280</v>
       </c>
       <c r="K101" t="n">
-        <v>532</v>
+        <v>762</v>
       </c>
       <c r="L101" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="M101" t="n">
         <v>18</v>
@@ -9661,7 +9661,7 @@
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -9676,25 +9676,25 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="F102" t="n">
-        <v>532</v>
+        <v>570</v>
       </c>
       <c r="G102" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="H102" t="n">
         <v>18</v>
@@ -9705,20 +9705,20 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="K102" t="n">
-        <v>532</v>
+        <v>570</v>
       </c>
       <c r="L102" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="M102" t="n">
         <v>18</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>9992609291013</t>
+          <t>9992609291013_9992609291013_9992609291013K</t>
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
@@ -9752,7 +9752,7 @@
       <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+          <t>COCINA-01_A4 Vitrina 570_Piso</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -9767,49 +9767,49 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>99</v>
+        <v>332</v>
       </c>
       <c r="F103" t="n">
-        <v>1407</v>
+        <v>570</v>
       </c>
       <c r="G103" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="H103" t="n">
         <v>18</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>98</v>
+        <v>331</v>
       </c>
       <c r="K103" t="n">
-        <v>1407</v>
+        <v>570</v>
       </c>
       <c r="L103" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="M103" t="n">
         <v>18</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>9992609291020</t>
+          <t>9992609291020_9992609291020</t>
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
@@ -9843,7 +9843,7 @@
       <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Vitrina 570_Techo</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -9858,54 +9858,54 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>99</v>
+        <v>1004</v>
       </c>
       <c r="F104" t="n">
-        <v>367.7</v>
+        <v>332</v>
       </c>
       <c r="G104" t="n">
-        <v>0.04</v>
+        <v>0.33</v>
       </c>
       <c r="H104" t="n">
         <v>18</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>98</v>
+        <v>1004</v>
       </c>
       <c r="K104" t="n">
-        <v>367.7</v>
+        <v>331</v>
       </c>
       <c r="L104" t="n">
-        <v>0.04</v>
+        <v>0.33</v>
       </c>
       <c r="M104" t="n">
         <v>18</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>9992609291037</t>
+          <t>9992609291037_9992609291037</t>
         </is>
       </c>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q104" t="n">
         <v>0</v>
@@ -9914,7 +9914,7 @@
         <v>0</v>
       </c>
       <c r="S104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T104" t="inlineStr">
         <is>
@@ -9934,12 +9934,1013 @@
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr">
         <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>9992609291037</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" t="n">
+        <v>1004</v>
+      </c>
+      <c r="F105" t="n">
+        <v>332</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H105" t="n">
+        <v>18</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>1004</v>
+      </c>
+      <c r="K105" t="n">
+        <v>331</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="M105" t="n">
+        <v>18</v>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>9992609291044_9992609291044</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr"/>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0</v>
+      </c>
+      <c r="R105" t="n">
+        <v>1</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>9992609291044</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" t="n">
+        <v>1014</v>
+      </c>
+      <c r="F106" t="n">
+        <v>544</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H106" t="n">
+        <v>5</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>5_Melamina_BLANCO 5</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>1014</v>
+      </c>
+      <c r="K106" t="n">
+        <v>544</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M106" t="n">
+        <v>5</v>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>9992609291051</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>9992609291051</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" t="n">
+        <v>80</v>
+      </c>
+      <c r="F107" t="n">
+        <v>534</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H107" t="n">
+        <v>18</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>80</v>
+      </c>
+      <c r="K107" t="n">
+        <v>534</v>
+      </c>
+      <c r="L107" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M107" t="n">
+        <v>18</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>9992609291068_9992609291068</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr"/>
+      <c r="P107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr"/>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>9992609291068</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta montante izq</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta montante izq</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" t="n">
+        <v>1037</v>
+      </c>
+      <c r="F108" t="n">
+        <v>60</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H108" t="n">
+        <v>18</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>1037</v>
+      </c>
+      <c r="K108" t="n">
+        <v>60</v>
+      </c>
+      <c r="L108" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M108" t="n">
+        <v>18</v>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>9992609291075_9992609291075</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr"/>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0</v>
+      </c>
+      <c r="S108" t="n">
+        <v>0</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr"/>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta montante izq</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>9992609291075</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta montante der</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta montante der</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" t="n">
+        <v>1037</v>
+      </c>
+      <c r="F109" t="n">
+        <v>60</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H109" t="n">
+        <v>18</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>1037</v>
+      </c>
+      <c r="K109" t="n">
+        <v>60</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M109" t="n">
+        <v>18</v>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>9992609291082_9992609291082</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr"/>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
+        <v>0</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta montante der</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>9992609291082</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta travesano abajo</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta travesano abajo</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" t="n">
+        <v>447</v>
+      </c>
+      <c r="F110" t="n">
+        <v>70</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H110" t="n">
+        <v>18</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>447</v>
+      </c>
+      <c r="K110" t="n">
+        <v>70</v>
+      </c>
+      <c r="L110" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M110" t="n">
+        <v>18</v>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>9992609291099_9992609291099</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr"/>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="n">
+        <v>0</v>
+      </c>
+      <c r="S110" t="n">
+        <v>0</v>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>横纹</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W110" t="inlineStr"/>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta travesano abajo</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>9992609291099</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta travesano arriba</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta travesano arriba</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" t="n">
+        <v>447</v>
+      </c>
+      <c r="F111" t="n">
+        <v>70</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H111" t="n">
+        <v>18</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>18_Madera maciza_MADERA VERDE 18</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>447</v>
+      </c>
+      <c r="K111" t="n">
+        <v>70</v>
+      </c>
+      <c r="L111" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M111" t="n">
+        <v>18</v>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>9992609291105_9992609291105</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr"/>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="n">
+        <v>0</v>
+      </c>
+      <c r="S111" t="n">
+        <v>0</v>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>横纹</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr"/>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Puerta travesano arriba</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>9992609291105</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" t="n">
+        <v>281</v>
+      </c>
+      <c r="F112" t="n">
+        <v>532</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H112" t="n">
+        <v>18</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>280</v>
+      </c>
+      <c r="K112" t="n">
+        <v>532</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M112" t="n">
+        <v>18</v>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>9992609291112</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr"/>
+      <c r="P112" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>1</v>
+      </c>
+      <c r="R112" t="n">
+        <v>0</v>
+      </c>
+      <c r="S112" t="n">
+        <v>0</v>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr"/>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>9992609291112</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>1</v>
+      </c>
+      <c r="E113" t="n">
+        <v>281</v>
+      </c>
+      <c r="F113" t="n">
+        <v>532</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H113" t="n">
+        <v>18</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>18_Melamina_BLANCO 18</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>280</v>
+      </c>
+      <c r="K113" t="n">
+        <v>532</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M113" t="n">
+        <v>18</v>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>9992609291129</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr"/>
+      <c r="P113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>1</v>
+      </c>
+      <c r="R113" t="n">
+        <v>0</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr"/>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>9992609291129</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" t="n">
+        <v>99</v>
+      </c>
+      <c r="F114" t="n">
+        <v>1407</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H114" t="n">
+        <v>18</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>98</v>
+      </c>
+      <c r="K114" t="n">
+        <v>1407</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="M114" t="n">
+        <v>18</v>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>9992609291136</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr"/>
+      <c r="P114" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" t="n">
+        <v>0</v>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr"/>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>9992609291136</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
           <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
-      <c r="Y104" t="inlineStr">
-        <is>
-          <t>9992609291037</t>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" t="n">
+        <v>99</v>
+      </c>
+      <c r="F115" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H115" t="n">
+        <v>18</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>98</v>
+      </c>
+      <c r="K115" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="L115" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M115" t="n">
+        <v>18</v>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>9992609291143</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr"/>
+      <c r="P115" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0</v>
+      </c>
+      <c r="R115" t="n">
+        <v>0</v>
+      </c>
+      <c r="S115" t="n">
+        <v>0</v>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W115" t="inlineStr"/>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>9992609291143</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A2 escurreplatos: sin piso sobre la bacha, listón frente + travesaño inferior, junta 38/62, Bronzen LC-560 + cubiertero como herrajes; 114/114
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -7310,25 +7310,25 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Liston frente</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Liston frente</t>
         </is>
       </c>
       <c r="D76" t="n">
         <v>1</v>
       </c>
       <c r="E76" t="n">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="F76" t="n">
-        <v>600</v>
+        <v>564</v>
       </c>
       <c r="G76" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="H76" t="n">
         <v>18</v>
@@ -7339,13 +7339,13 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>331</v>
+        <v>79</v>
       </c>
       <c r="K76" t="n">
-        <v>600</v>
+        <v>564</v>
       </c>
       <c r="L76" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="M76" t="n">
         <v>18</v>
@@ -7386,7 +7386,7 @@
       <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Piso</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Liston frente</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
@@ -7504,13 +7504,13 @@
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>1004</v>
+        <v>1022</v>
       </c>
       <c r="F78" t="n">
         <v>332</v>
       </c>
       <c r="G78" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="H78" t="n">
         <v>18</v>
@@ -7521,13 +7521,13 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>1004</v>
+        <v>1021</v>
       </c>
       <c r="K78" t="n">
         <v>331</v>
       </c>
       <c r="L78" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="M78" t="n">
         <v>18</v>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q78" t="n">
         <v>0</v>
@@ -7595,13 +7595,13 @@
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>1004</v>
+        <v>1022</v>
       </c>
       <c r="F79" t="n">
         <v>332</v>
       </c>
       <c r="G79" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="H79" t="n">
         <v>18</v>
@@ -7612,13 +7612,13 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>1004</v>
+        <v>1021</v>
       </c>
       <c r="K79" t="n">
         <v>331</v>
       </c>
       <c r="L79" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="M79" t="n">
         <v>18</v>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q79" t="n">
         <v>0</v>
@@ -7856,25 +7856,25 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero inferior</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero inferior</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>1</v>
       </c>
       <c r="E82" t="n">
+        <v>80</v>
+      </c>
+      <c r="F82" t="n">
         <v>564</v>
       </c>
-      <c r="F82" t="n">
-        <v>301</v>
-      </c>
       <c r="G82" t="n">
-        <v>0.17</v>
+        <v>0.05</v>
       </c>
       <c r="H82" t="n">
         <v>18</v>
@@ -7885,25 +7885,25 @@
         </is>
       </c>
       <c r="J82" t="n">
+        <v>79</v>
+      </c>
+      <c r="K82" t="n">
         <v>564</v>
       </c>
-      <c r="K82" t="n">
-        <v>300</v>
-      </c>
       <c r="L82" t="n">
-        <v>0.17</v>
+        <v>0.04</v>
       </c>
       <c r="M82" t="n">
         <v>18</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>9992609290818_9992609290818_9992609290818K</t>
+          <t>9992609290818_9992609290818</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q82" t="n">
         <v>0</v>
@@ -7912,7 +7912,7 @@
         <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T82" t="inlineStr">
         <is>
@@ -7932,7 +7932,7 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Travesano trasero inferior</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -7947,60 +7947,60 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>597</v>
+        <v>564</v>
       </c>
       <c r="F83" t="n">
-        <v>467</v>
+        <v>301</v>
       </c>
       <c r="G83" t="n">
-        <v>0.28</v>
+        <v>0.17</v>
       </c>
       <c r="H83" t="n">
         <v>18</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>595</v>
+        <v>564</v>
       </c>
       <c r="K83" t="n">
-        <v>465</v>
+        <v>300</v>
       </c>
       <c r="L83" t="n">
-        <v>0.28</v>
+        <v>0.17</v>
       </c>
       <c r="M83" t="n">
         <v>18</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>9992609290825_9992609290825</t>
+          <t>9992609290825_9992609290825_9992609290825K</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S83" t="n">
         <v>1</v>
@@ -8023,7 +8023,7 @@
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Estante fijo</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -8038,12 +8038,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -8053,10 +8053,10 @@
         <v>597</v>
       </c>
       <c r="F84" t="n">
-        <v>567</v>
+        <v>394</v>
       </c>
       <c r="G84" t="n">
-        <v>0.34</v>
+        <v>0.24</v>
       </c>
       <c r="H84" t="n">
         <v>18</v>
@@ -8070,10 +8070,10 @@
         <v>595</v>
       </c>
       <c r="K84" t="n">
-        <v>565</v>
+        <v>392</v>
       </c>
       <c r="L84" t="n">
-        <v>0.34</v>
+        <v>0.23</v>
       </c>
       <c r="M84" t="n">
         <v>18</v>
@@ -8114,7 +8114,7 @@
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible arriba</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -8129,63 +8129,63 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>1</v>
       </c>
       <c r="E85" t="n">
-        <v>281</v>
+        <v>597</v>
       </c>
       <c r="F85" t="n">
-        <v>562</v>
+        <v>640</v>
       </c>
       <c r="G85" t="n">
-        <v>0.16</v>
+        <v>0.38</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>280</v>
+        <v>595</v>
       </c>
       <c r="K85" t="n">
-        <v>562</v>
+        <v>638</v>
       </c>
       <c r="L85" t="n">
-        <v>0.16</v>
+        <v>0.38</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>9992609290849</t>
+          <t>9992609290849_9992609290849</t>
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q85" t="n">
         <v>1</v>
       </c>
       <c r="R85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -8205,7 +8205,7 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>COCINA-01_A2 Alacena 600 rebatible_Estante 1</t>
+          <t>COCINA-01_A2 Alacena 600 rebatible_Puerta rebatible abajo</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">

</xml_diff>

<commit_message>
Alacenas hasta 2450 (techo a 2470, 20 de aire); 114/114; paquete regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -5866,13 +5866,13 @@
         <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>1040</v>
+        <v>1000</v>
       </c>
       <c r="F60" t="n">
         <v>332</v>
       </c>
       <c r="G60" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="H60" t="n">
         <v>18</v>
@@ -5883,13 +5883,13 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>1040</v>
+        <v>1000</v>
       </c>
       <c r="K60" t="n">
         <v>331</v>
       </c>
       <c r="L60" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="M60" t="n">
         <v>18</v>
@@ -5957,13 +5957,13 @@
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>1040</v>
+        <v>1000</v>
       </c>
       <c r="F61" t="n">
         <v>332</v>
       </c>
       <c r="G61" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="H61" t="n">
         <v>18</v>
@@ -5974,13 +5974,13 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>1040</v>
+        <v>1000</v>
       </c>
       <c r="K61" t="n">
         <v>331</v>
       </c>
       <c r="L61" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="M61" t="n">
         <v>18</v>
@@ -6230,13 +6230,13 @@
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="F64" t="n">
         <v>755</v>
       </c>
       <c r="G64" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="H64" t="n">
         <v>5</v>
@@ -6247,13 +6247,13 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="K64" t="n">
         <v>755</v>
       </c>
       <c r="L64" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="M64" t="n">
         <v>5</v>
@@ -6321,13 +6321,13 @@
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="F65" t="n">
         <v>762</v>
       </c>
       <c r="G65" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="H65" t="n">
         <v>5</v>
@@ -6338,13 +6338,13 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="K65" t="n">
         <v>762</v>
       </c>
       <c r="L65" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="M65" t="n">
         <v>5</v>
@@ -6412,7 +6412,7 @@
         <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="F66" t="n">
         <v>80</v>
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="K66" t="n">
         <v>79</v>
@@ -6503,7 +6503,7 @@
         <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="F67" t="n">
         <v>80</v>
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="K67" t="n">
         <v>79</v>
@@ -6594,7 +6594,7 @@
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F68" t="n">
         <v>60</v>
@@ -6611,7 +6611,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K68" t="n">
         <v>60</v>
@@ -6685,7 +6685,7 @@
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F69" t="n">
         <v>60</v>
@@ -6702,7 +6702,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K69" t="n">
         <v>60</v>
@@ -7504,13 +7504,13 @@
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>1022</v>
+        <v>982</v>
       </c>
       <c r="F78" t="n">
         <v>332</v>
       </c>
       <c r="G78" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="H78" t="n">
         <v>18</v>
@@ -7521,13 +7521,13 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>1021</v>
+        <v>981</v>
       </c>
       <c r="K78" t="n">
         <v>331</v>
       </c>
       <c r="L78" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="M78" t="n">
         <v>18</v>
@@ -7595,13 +7595,13 @@
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>1022</v>
+        <v>982</v>
       </c>
       <c r="F79" t="n">
         <v>332</v>
       </c>
       <c r="G79" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="H79" t="n">
         <v>18</v>
@@ -7612,13 +7612,13 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>1021</v>
+        <v>981</v>
       </c>
       <c r="K79" t="n">
         <v>331</v>
       </c>
       <c r="L79" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="M79" t="n">
         <v>18</v>
@@ -7686,13 +7686,13 @@
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="F80" t="n">
         <v>574</v>
       </c>
       <c r="G80" t="n">
-        <v>0.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H80" t="n">
         <v>5</v>
@@ -7703,13 +7703,13 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="K80" t="n">
         <v>574</v>
       </c>
       <c r="L80" t="n">
-        <v>0.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M80" t="n">
         <v>5</v>
@@ -8053,10 +8053,10 @@
         <v>597</v>
       </c>
       <c r="F84" t="n">
-        <v>394</v>
+        <v>379</v>
       </c>
       <c r="G84" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="H84" t="n">
         <v>18</v>
@@ -8070,10 +8070,10 @@
         <v>595</v>
       </c>
       <c r="K84" t="n">
-        <v>392</v>
+        <v>377</v>
       </c>
       <c r="L84" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="M84" t="n">
         <v>18</v>
@@ -8144,10 +8144,10 @@
         <v>597</v>
       </c>
       <c r="F85" t="n">
-        <v>640</v>
+        <v>615</v>
       </c>
       <c r="G85" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="H85" t="n">
         <v>18</v>
@@ -8161,10 +8161,10 @@
         <v>595</v>
       </c>
       <c r="K85" t="n">
-        <v>638</v>
+        <v>613</v>
       </c>
       <c r="L85" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="M85" t="n">
         <v>18</v>
@@ -8414,13 +8414,13 @@
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="F88" t="n">
         <v>332</v>
       </c>
       <c r="G88" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="H88" t="n">
         <v>18</v>
@@ -8431,13 +8431,13 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="K88" t="n">
         <v>331</v>
       </c>
       <c r="L88" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="M88" t="n">
         <v>18</v>
@@ -8505,13 +8505,13 @@
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="F89" t="n">
         <v>332</v>
       </c>
       <c r="G89" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="H89" t="n">
         <v>18</v>
@@ -8522,13 +8522,13 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="K89" t="n">
         <v>331</v>
       </c>
       <c r="L89" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="M89" t="n">
         <v>18</v>
@@ -8596,13 +8596,13 @@
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="F90" t="n">
         <v>774</v>
       </c>
       <c r="G90" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="H90" t="n">
         <v>5</v>
@@ -8613,13 +8613,13 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="K90" t="n">
         <v>774</v>
       </c>
       <c r="L90" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="M90" t="n">
         <v>5</v>
@@ -8778,7 +8778,7 @@
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F92" t="n">
         <v>60</v>
@@ -8795,7 +8795,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K92" t="n">
         <v>60</v>
@@ -8869,7 +8869,7 @@
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F93" t="n">
         <v>60</v>
@@ -8886,7 +8886,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K93" t="n">
         <v>60</v>
@@ -9142,7 +9142,7 @@
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F96" t="n">
         <v>60</v>
@@ -9159,7 +9159,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K96" t="n">
         <v>60</v>
@@ -9233,7 +9233,7 @@
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F97" t="n">
         <v>60</v>
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K97" t="n">
         <v>60</v>
@@ -9870,13 +9870,13 @@
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="F104" t="n">
         <v>332</v>
       </c>
       <c r="G104" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="H104" t="n">
         <v>18</v>
@@ -9887,13 +9887,13 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="K104" t="n">
         <v>331</v>
       </c>
       <c r="L104" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="M104" t="n">
         <v>18</v>
@@ -9961,13 +9961,13 @@
         <v>1</v>
       </c>
       <c r="E105" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="F105" t="n">
         <v>332</v>
       </c>
       <c r="G105" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="H105" t="n">
         <v>18</v>
@@ -9978,13 +9978,13 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1004</v>
+        <v>964</v>
       </c>
       <c r="K105" t="n">
         <v>331</v>
       </c>
       <c r="L105" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="M105" t="n">
         <v>18</v>
@@ -10052,13 +10052,13 @@
         <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="F106" t="n">
         <v>544</v>
       </c>
       <c r="G106" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="H106" t="n">
         <v>5</v>
@@ -10069,13 +10069,13 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>1014</v>
+        <v>974</v>
       </c>
       <c r="K106" t="n">
         <v>544</v>
       </c>
       <c r="L106" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="M106" t="n">
         <v>5</v>
@@ -10234,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="E108" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F108" t="n">
         <v>60</v>
@@ -10251,7 +10251,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K108" t="n">
         <v>60</v>
@@ -10325,7 +10325,7 @@
         <v>1</v>
       </c>
       <c r="E109" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="F109" t="n">
         <v>60</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>1037</v>
+        <v>997</v>
       </c>
       <c r="K109" t="n">
         <v>60</v>

</xml_diff>

<commit_message>
Viga pared larga: escotaduras en alacenas A1/A2/A3, techos recortados, travesaños contra la viga; Placa.escotadura + dentro() no convexo; 114/114
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -6139,13 +6139,13 @@
         <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>782</v>
+        <v>657</v>
       </c>
       <c r="F63" t="n">
         <v>782</v>
       </c>
       <c r="G63" t="n">
-        <v>0.61</v>
+        <v>0.51</v>
       </c>
       <c r="H63" t="n">
         <v>18</v>
@@ -6156,13 +6156,13 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>782</v>
+        <v>657</v>
       </c>
       <c r="K63" t="n">
         <v>782</v>
       </c>
       <c r="L63" t="n">
-        <v>0.61</v>
+        <v>0.51</v>
       </c>
       <c r="M63" t="n">
         <v>18</v>
@@ -6230,13 +6230,13 @@
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>974</v>
+        <v>689</v>
       </c>
       <c r="F64" t="n">
         <v>755</v>
       </c>
       <c r="G64" t="n">
-        <v>0.74</v>
+        <v>0.52</v>
       </c>
       <c r="H64" t="n">
         <v>5</v>
@@ -6247,13 +6247,13 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>974</v>
+        <v>689</v>
       </c>
       <c r="K64" t="n">
         <v>755</v>
       </c>
       <c r="L64" t="n">
-        <v>0.74</v>
+        <v>0.52</v>
       </c>
       <c r="M64" t="n">
         <v>5</v>
@@ -7234,10 +7234,10 @@
         <v>80</v>
       </c>
       <c r="F75" t="n">
-        <v>751</v>
+        <v>638</v>
       </c>
       <c r="G75" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="H75" t="n">
         <v>18</v>
@@ -7251,10 +7251,10 @@
         <v>80</v>
       </c>
       <c r="K75" t="n">
-        <v>751</v>
+        <v>638</v>
       </c>
       <c r="L75" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="M75" t="n">
         <v>18</v>
@@ -7416,10 +7416,10 @@
         <v>600</v>
       </c>
       <c r="F77" t="n">
-        <v>332</v>
+        <v>207</v>
       </c>
       <c r="G77" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="H77" t="n">
         <v>18</v>
@@ -7433,10 +7433,10 @@
         <v>600</v>
       </c>
       <c r="K77" t="n">
-        <v>331</v>
+        <v>206</v>
       </c>
       <c r="L77" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="M77" t="n">
         <v>18</v>
@@ -7686,13 +7686,13 @@
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>974</v>
+        <v>689</v>
       </c>
       <c r="F80" t="n">
         <v>574</v>
       </c>
       <c r="G80" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="H80" t="n">
         <v>5</v>
@@ -7703,13 +7703,13 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>974</v>
+        <v>689</v>
       </c>
       <c r="K80" t="n">
         <v>574</v>
       </c>
       <c r="L80" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="M80" t="n">
         <v>5</v>
@@ -8323,13 +8323,13 @@
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>332</v>
+        <v>207</v>
       </c>
       <c r="F87" t="n">
         <v>800</v>
       </c>
       <c r="G87" t="n">
-        <v>0.27</v>
+        <v>0.17</v>
       </c>
       <c r="H87" t="n">
         <v>18</v>
@@ -8340,13 +8340,13 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>331</v>
+        <v>206</v>
       </c>
       <c r="K87" t="n">
         <v>800</v>
       </c>
       <c r="L87" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="M87" t="n">
         <v>18</v>
@@ -8596,13 +8596,13 @@
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>974</v>
+        <v>689</v>
       </c>
       <c r="F90" t="n">
         <v>774</v>
       </c>
       <c r="G90" t="n">
-        <v>0.75</v>
+        <v>0.53</v>
       </c>
       <c r="H90" t="n">
         <v>5</v>
@@ -8613,13 +8613,13 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>974</v>
+        <v>689</v>
       </c>
       <c r="K90" t="n">
         <v>774</v>
       </c>
       <c r="L90" t="n">
-        <v>0.75</v>
+        <v>0.53</v>
       </c>
       <c r="M90" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
A4 mueble campana 1794-2450 con SDC-100 colgada debajo, puerta ciega, ducto O150 a la salida de aire (Y1120/Z2120); alacena() con z_piso; 106/106
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y115"/>
+  <dimension ref="A1:Y107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8766,12 +8766,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der montante izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta montante izq</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der montante izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta montante izq</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -8842,7 +8842,7 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der montante izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta montante izq</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -8857,12 +8857,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der montante der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta montante der</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der montante der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta montante der</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -8933,7 +8933,7 @@
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der montante der</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta montante der</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -8948,25 +8948,25 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano abajo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta travesano abajo</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano abajo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta travesano abajo</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>277</v>
+        <v>677</v>
       </c>
       <c r="F94" t="n">
         <v>70</v>
       </c>
       <c r="G94" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="H94" t="n">
         <v>18</v>
@@ -8977,13 +8977,13 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>277</v>
+        <v>677</v>
       </c>
       <c r="K94" t="n">
         <v>70</v>
       </c>
       <c r="L94" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="M94" t="n">
         <v>18</v>
@@ -9024,7 +9024,7 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano abajo</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta travesano abajo</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -9039,25 +9039,25 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano arriba</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta travesano arriba</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano arriba</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta travesano arriba</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>277</v>
+        <v>677</v>
       </c>
       <c r="F95" t="n">
         <v>70</v>
       </c>
       <c r="G95" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="H95" t="n">
         <v>18</v>
@@ -9068,13 +9068,13 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>277</v>
+        <v>677</v>
       </c>
       <c r="K95" t="n">
         <v>70</v>
       </c>
       <c r="L95" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="M95" t="n">
         <v>18</v>
@@ -9115,7 +9115,7 @@
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta der travesano arriba</t>
+          <t>COCINA-01_A3 Vitrina 800_Puerta travesano arriba</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -9130,49 +9130,49 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>997</v>
+        <v>281</v>
       </c>
       <c r="F96" t="n">
-        <v>60</v>
+        <v>762</v>
       </c>
       <c r="G96" t="n">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="H96" t="n">
         <v>18</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>997</v>
+        <v>280</v>
       </c>
       <c r="K96" t="n">
-        <v>60</v>
+        <v>762</v>
       </c>
       <c r="L96" t="n">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="M96" t="n">
         <v>18</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>9992609290955_9992609290955</t>
+          <t>9992609290955</t>
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
@@ -9180,7 +9180,7 @@
         <v>0</v>
       </c>
       <c r="Q96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R96" t="n">
         <v>0</v>
@@ -9206,7 +9206,7 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante izq</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -9221,49 +9221,49 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante der</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante der</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>997</v>
+        <v>281</v>
       </c>
       <c r="F97" t="n">
-        <v>60</v>
+        <v>762</v>
       </c>
       <c r="G97" t="n">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="H97" t="n">
         <v>18</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>997</v>
+        <v>280</v>
       </c>
       <c r="K97" t="n">
-        <v>60</v>
+        <v>762</v>
       </c>
       <c r="L97" t="n">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="M97" t="n">
         <v>18</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>9992609290962_9992609290962</t>
+          <t>9992609290962</t>
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
@@ -9271,7 +9271,7 @@
         <v>0</v>
       </c>
       <c r="Q97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R97" t="n">
         <v>0</v>
@@ -9297,7 +9297,7 @@
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq montante der</t>
+          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -9312,42 +9312,42 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano abajo</t>
+          <t>COCINA-01_A4 Campana 570_Piso</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano abajo</t>
+          <t>COCINA-01_A4 Campana 570_Piso</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>277</v>
+        <v>332</v>
       </c>
       <c r="F98" t="n">
-        <v>70</v>
+        <v>570</v>
       </c>
       <c r="G98" t="n">
-        <v>0.02</v>
+        <v>0.19</v>
       </c>
       <c r="H98" t="n">
         <v>18</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>277</v>
+        <v>331</v>
       </c>
       <c r="K98" t="n">
-        <v>70</v>
+        <v>570</v>
       </c>
       <c r="L98" t="n">
-        <v>0.02</v>
+        <v>0.19</v>
       </c>
       <c r="M98" t="n">
         <v>18</v>
@@ -9362,7 +9362,7 @@
         <v>0</v>
       </c>
       <c r="Q98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R98" t="n">
         <v>0</v>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>横纹</t>
+          <t>竖纹</t>
         </is>
       </c>
       <c r="U98" t="inlineStr">
@@ -9388,7 +9388,7 @@
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano abajo</t>
+          <t>COCINA-01_A4 Campana 570_Piso</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -9403,42 +9403,42 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano arriba</t>
+          <t>COCINA-01_A4 Campana 570_Techo</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano arriba</t>
+          <t>COCINA-01_A4 Campana 570_Techo</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>277</v>
+        <v>332</v>
       </c>
       <c r="F99" t="n">
-        <v>70</v>
+        <v>570</v>
       </c>
       <c r="G99" t="n">
-        <v>0.02</v>
+        <v>0.19</v>
       </c>
       <c r="H99" t="n">
         <v>18</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>277</v>
+        <v>331</v>
       </c>
       <c r="K99" t="n">
-        <v>70</v>
+        <v>570</v>
       </c>
       <c r="L99" t="n">
-        <v>0.02</v>
+        <v>0.19</v>
       </c>
       <c r="M99" t="n">
         <v>18</v>
@@ -9450,7 +9450,7 @@
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q99" t="n">
         <v>0</v>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="T99" t="inlineStr">
         <is>
-          <t>横纹</t>
+          <t>竖纹</t>
         </is>
       </c>
       <c r="U99" t="inlineStr">
@@ -9479,7 +9479,7 @@
       <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Puerta izq travesano arriba</t>
+          <t>COCINA-01_A4 Campana 570_Techo</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -9494,22 +9494,22 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A4 Campana 570_Lateral der</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A4 Campana 570_Lateral der</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>281</v>
+        <v>620</v>
       </c>
       <c r="F100" t="n">
-        <v>762</v>
+        <v>332</v>
       </c>
       <c r="G100" t="n">
         <v>0.21</v>
@@ -9523,10 +9523,10 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>280</v>
+        <v>620</v>
       </c>
       <c r="K100" t="n">
-        <v>762</v>
+        <v>331</v>
       </c>
       <c r="L100" t="n">
         <v>0.21</v>
@@ -9536,7 +9536,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>9992609290993</t>
+          <t>9992609290993_9992609290993</t>
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
@@ -9544,13 +9544,13 @@
         <v>0</v>
       </c>
       <c r="Q100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R100" t="n">
         <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T100" t="inlineStr">
         <is>
@@ -9570,7 +9570,7 @@
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 1</t>
+          <t>COCINA-01_A4 Campana 570_Lateral der</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -9585,22 +9585,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Campana 570_Lateral izq</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Campana 570_Lateral izq</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>281</v>
+        <v>620</v>
       </c>
       <c r="F101" t="n">
-        <v>762</v>
+        <v>332</v>
       </c>
       <c r="G101" t="n">
         <v>0.21</v>
@@ -9614,10 +9614,10 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>280</v>
+        <v>620</v>
       </c>
       <c r="K101" t="n">
-        <v>762</v>
+        <v>331</v>
       </c>
       <c r="L101" t="n">
         <v>0.21</v>
@@ -9627,7 +9627,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>9992609291006</t>
+          <t>9992609291006_9992609291006</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
@@ -9635,10 +9635,10 @@
         <v>0</v>
       </c>
       <c r="Q101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S101" t="n">
         <v>0</v>
@@ -9661,7 +9661,7 @@
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>COCINA-01_A3 Vitrina 800_Estante 2</t>
+          <t>COCINA-01_A4 Campana 570_Lateral izq</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -9676,49 +9676,49 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Campana 570_Fondo</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Campana 570_Fondo</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>332</v>
+        <v>630</v>
       </c>
       <c r="F102" t="n">
-        <v>570</v>
+        <v>544</v>
       </c>
       <c r="G102" t="n">
-        <v>0.19</v>
+        <v>0.34</v>
       </c>
       <c r="H102" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>5_Melamina_BLANCO 5</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>331</v>
+        <v>630</v>
       </c>
       <c r="K102" t="n">
-        <v>570</v>
+        <v>544</v>
       </c>
       <c r="L102" t="n">
-        <v>0.19</v>
+        <v>0.34</v>
       </c>
       <c r="M102" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>9992609291013_9992609291013_9992609291013K</t>
+          <t>9992609291013</t>
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
@@ -9726,7 +9726,7 @@
         <v>0</v>
       </c>
       <c r="Q102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R102" t="n">
         <v>0</v>
@@ -9752,7 +9752,7 @@
       <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Piso</t>
+          <t>COCINA-01_A4 Campana 570_Fondo</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -9767,25 +9767,25 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Campana 570_Travesano trasero</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Campana 570_Travesano trasero</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>332</v>
+        <v>80</v>
       </c>
       <c r="F103" t="n">
-        <v>570</v>
+        <v>534</v>
       </c>
       <c r="G103" t="n">
-        <v>0.19</v>
+        <v>0.04</v>
       </c>
       <c r="H103" t="n">
         <v>18</v>
@@ -9796,13 +9796,13 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>331</v>
+        <v>80</v>
       </c>
       <c r="K103" t="n">
-        <v>570</v>
+        <v>534</v>
       </c>
       <c r="L103" t="n">
-        <v>0.19</v>
+        <v>0.04</v>
       </c>
       <c r="M103" t="n">
         <v>18</v>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q103" t="n">
         <v>0</v>
@@ -9843,7 +9843,7 @@
       <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Techo</t>
+          <t>COCINA-01_A4 Campana 570_Travesano trasero</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -9858,42 +9858,42 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Campana 570_Puerta</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Campana 570_Puerta</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>964</v>
+        <v>653</v>
       </c>
       <c r="F104" t="n">
-        <v>332</v>
+        <v>567</v>
       </c>
       <c r="G104" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="H104" t="n">
         <v>18</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>964</v>
+        <v>651</v>
       </c>
       <c r="K104" t="n">
-        <v>331</v>
+        <v>565</v>
       </c>
       <c r="L104" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="M104" t="n">
         <v>18</v>
@@ -9905,13 +9905,13 @@
       </c>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S104" t="n">
         <v>1</v>
@@ -9934,7 +9934,7 @@
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral der</t>
+          <t>COCINA-01_A4 Campana 570_Puerta</t>
         </is>
       </c>
       <c r="Y104" t="inlineStr">
@@ -9949,25 +9949,25 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Campana 570_Estante 1</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Campana 570_Estante 1</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>1</v>
       </c>
       <c r="E105" t="n">
-        <v>964</v>
+        <v>281</v>
       </c>
       <c r="F105" t="n">
-        <v>332</v>
+        <v>532</v>
       </c>
       <c r="G105" t="n">
-        <v>0.32</v>
+        <v>0.15</v>
       </c>
       <c r="H105" t="n">
         <v>18</v>
@@ -9978,20 +9978,20 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>964</v>
+        <v>280</v>
       </c>
       <c r="K105" t="n">
-        <v>331</v>
+        <v>532</v>
       </c>
       <c r="L105" t="n">
-        <v>0.32</v>
+        <v>0.15</v>
       </c>
       <c r="M105" t="n">
         <v>18</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>9992609291044_9992609291044</t>
+          <t>9992609291044</t>
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
@@ -9999,10 +9999,10 @@
         <v>0</v>
       </c>
       <c r="Q105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S105" t="n">
         <v>0</v>
@@ -10025,7 +10025,7 @@
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Lateral izq</t>
+          <t>COCINA-01_A4 Campana 570_Estante 1</t>
         </is>
       </c>
       <c r="Y105" t="inlineStr">
@@ -10040,45 +10040,45 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="D106" t="n">
         <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>974</v>
+        <v>99</v>
       </c>
       <c r="F106" t="n">
-        <v>544</v>
+        <v>1407</v>
       </c>
       <c r="G106" t="n">
-        <v>0.53</v>
+        <v>0.14</v>
       </c>
       <c r="H106" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>5_Melamina_BLANCO 5</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>974</v>
+        <v>98</v>
       </c>
       <c r="K106" t="n">
-        <v>544</v>
+        <v>1407</v>
       </c>
       <c r="L106" t="n">
-        <v>0.53</v>
+        <v>0.14</v>
       </c>
       <c r="M106" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -10087,7 +10087,7 @@
       </c>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q106" t="n">
         <v>0</v>
@@ -10116,7 +10116,7 @@
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Fondo</t>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
         </is>
       </c>
       <c r="Y106" t="inlineStr">
@@ -10131,22 +10131,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="D107" t="n">
         <v>1</v>
       </c>
       <c r="E107" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="F107" t="n">
-        <v>534</v>
+        <v>367.7</v>
       </c>
       <c r="G107" t="n">
         <v>0.04</v>
@@ -10156,14 +10156,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="K107" t="n">
-        <v>534</v>
+        <v>367.7</v>
       </c>
       <c r="L107" t="n">
         <v>0.04</v>
@@ -10173,12 +10173,12 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>9992609291068_9992609291068</t>
+          <t>9992609291068</t>
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q107" t="n">
         <v>0</v>
@@ -10207,740 +10207,12 @@
       <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Vitrina 570_Travesano trasero</t>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
       <c r="Y107" t="inlineStr">
         <is>
           <t>9992609291068</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>107</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta montante izq</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta montante izq</t>
-        </is>
-      </c>
-      <c r="D108" t="n">
-        <v>1</v>
-      </c>
-      <c r="E108" t="n">
-        <v>997</v>
-      </c>
-      <c r="F108" t="n">
-        <v>60</v>
-      </c>
-      <c r="G108" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="H108" t="n">
-        <v>18</v>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
-        </is>
-      </c>
-      <c r="J108" t="n">
-        <v>997</v>
-      </c>
-      <c r="K108" t="n">
-        <v>60</v>
-      </c>
-      <c r="L108" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="M108" t="n">
-        <v>18</v>
-      </c>
-      <c r="N108" t="inlineStr">
-        <is>
-          <t>9992609291075_9992609291075</t>
-        </is>
-      </c>
-      <c r="O108" t="inlineStr"/>
-      <c r="P108" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q108" t="n">
-        <v>0</v>
-      </c>
-      <c r="R108" t="n">
-        <v>0</v>
-      </c>
-      <c r="S108" t="n">
-        <v>0</v>
-      </c>
-      <c r="T108" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U108" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V108" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W108" t="inlineStr"/>
-      <c r="X108" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta montante izq</t>
-        </is>
-      </c>
-      <c r="Y108" t="inlineStr">
-        <is>
-          <t>9992609291075</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>108</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta montante der</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta montante der</t>
-        </is>
-      </c>
-      <c r="D109" t="n">
-        <v>1</v>
-      </c>
-      <c r="E109" t="n">
-        <v>997</v>
-      </c>
-      <c r="F109" t="n">
-        <v>60</v>
-      </c>
-      <c r="G109" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="H109" t="n">
-        <v>18</v>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
-        </is>
-      </c>
-      <c r="J109" t="n">
-        <v>997</v>
-      </c>
-      <c r="K109" t="n">
-        <v>60</v>
-      </c>
-      <c r="L109" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="M109" t="n">
-        <v>18</v>
-      </c>
-      <c r="N109" t="inlineStr">
-        <is>
-          <t>9992609291082_9992609291082</t>
-        </is>
-      </c>
-      <c r="O109" t="inlineStr"/>
-      <c r="P109" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q109" t="n">
-        <v>0</v>
-      </c>
-      <c r="R109" t="n">
-        <v>0</v>
-      </c>
-      <c r="S109" t="n">
-        <v>0</v>
-      </c>
-      <c r="T109" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U109" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V109" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W109" t="inlineStr"/>
-      <c r="X109" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta montante der</t>
-        </is>
-      </c>
-      <c r="Y109" t="inlineStr">
-        <is>
-          <t>9992609291082</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>109</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta travesano abajo</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta travesano abajo</t>
-        </is>
-      </c>
-      <c r="D110" t="n">
-        <v>1</v>
-      </c>
-      <c r="E110" t="n">
-        <v>447</v>
-      </c>
-      <c r="F110" t="n">
-        <v>70</v>
-      </c>
-      <c r="G110" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="H110" t="n">
-        <v>18</v>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
-        </is>
-      </c>
-      <c r="J110" t="n">
-        <v>447</v>
-      </c>
-      <c r="K110" t="n">
-        <v>70</v>
-      </c>
-      <c r="L110" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="M110" t="n">
-        <v>18</v>
-      </c>
-      <c r="N110" t="inlineStr">
-        <is>
-          <t>9992609291099_9992609291099</t>
-        </is>
-      </c>
-      <c r="O110" t="inlineStr"/>
-      <c r="P110" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q110" t="n">
-        <v>0</v>
-      </c>
-      <c r="R110" t="n">
-        <v>0</v>
-      </c>
-      <c r="S110" t="n">
-        <v>0</v>
-      </c>
-      <c r="T110" t="inlineStr">
-        <is>
-          <t>横纹</t>
-        </is>
-      </c>
-      <c r="U110" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V110" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W110" t="inlineStr"/>
-      <c r="X110" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta travesano abajo</t>
-        </is>
-      </c>
-      <c r="Y110" t="inlineStr">
-        <is>
-          <t>9992609291099</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>110</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta travesano arriba</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta travesano arriba</t>
-        </is>
-      </c>
-      <c r="D111" t="n">
-        <v>1</v>
-      </c>
-      <c r="E111" t="n">
-        <v>447</v>
-      </c>
-      <c r="F111" t="n">
-        <v>70</v>
-      </c>
-      <c r="G111" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="H111" t="n">
-        <v>18</v>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>18_Madera maciza_MADERA VERDE 18</t>
-        </is>
-      </c>
-      <c r="J111" t="n">
-        <v>447</v>
-      </c>
-      <c r="K111" t="n">
-        <v>70</v>
-      </c>
-      <c r="L111" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="M111" t="n">
-        <v>18</v>
-      </c>
-      <c r="N111" t="inlineStr">
-        <is>
-          <t>9992609291105_9992609291105</t>
-        </is>
-      </c>
-      <c r="O111" t="inlineStr"/>
-      <c r="P111" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q111" t="n">
-        <v>0</v>
-      </c>
-      <c r="R111" t="n">
-        <v>0</v>
-      </c>
-      <c r="S111" t="n">
-        <v>0</v>
-      </c>
-      <c r="T111" t="inlineStr">
-        <is>
-          <t>横纹</t>
-        </is>
-      </c>
-      <c r="U111" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V111" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W111" t="inlineStr"/>
-      <c r="X111" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Puerta travesano arriba</t>
-        </is>
-      </c>
-      <c r="Y111" t="inlineStr">
-        <is>
-          <t>9992609291105</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>111</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
-        </is>
-      </c>
-      <c r="D112" t="n">
-        <v>1</v>
-      </c>
-      <c r="E112" t="n">
-        <v>281</v>
-      </c>
-      <c r="F112" t="n">
-        <v>532</v>
-      </c>
-      <c r="G112" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H112" t="n">
-        <v>18</v>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>18_Melamina_BLANCO 18</t>
-        </is>
-      </c>
-      <c r="J112" t="n">
-        <v>280</v>
-      </c>
-      <c r="K112" t="n">
-        <v>532</v>
-      </c>
-      <c r="L112" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M112" t="n">
-        <v>18</v>
-      </c>
-      <c r="N112" t="inlineStr">
-        <is>
-          <t>9992609291112</t>
-        </is>
-      </c>
-      <c r="O112" t="inlineStr"/>
-      <c r="P112" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q112" t="n">
-        <v>1</v>
-      </c>
-      <c r="R112" t="n">
-        <v>0</v>
-      </c>
-      <c r="S112" t="n">
-        <v>0</v>
-      </c>
-      <c r="T112" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U112" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V112" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W112" t="inlineStr"/>
-      <c r="X112" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 1</t>
-        </is>
-      </c>
-      <c r="Y112" t="inlineStr">
-        <is>
-          <t>9992609291112</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>112</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
-        </is>
-      </c>
-      <c r="D113" t="n">
-        <v>1</v>
-      </c>
-      <c r="E113" t="n">
-        <v>281</v>
-      </c>
-      <c r="F113" t="n">
-        <v>532</v>
-      </c>
-      <c r="G113" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H113" t="n">
-        <v>18</v>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>18_Melamina_BLANCO 18</t>
-        </is>
-      </c>
-      <c r="J113" t="n">
-        <v>280</v>
-      </c>
-      <c r="K113" t="n">
-        <v>532</v>
-      </c>
-      <c r="L113" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M113" t="n">
-        <v>18</v>
-      </c>
-      <c r="N113" t="inlineStr">
-        <is>
-          <t>9992609291129</t>
-        </is>
-      </c>
-      <c r="O113" t="inlineStr"/>
-      <c r="P113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q113" t="n">
-        <v>1</v>
-      </c>
-      <c r="R113" t="n">
-        <v>0</v>
-      </c>
-      <c r="S113" t="n">
-        <v>0</v>
-      </c>
-      <c r="T113" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U113" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V113" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W113" t="inlineStr"/>
-      <c r="X113" t="inlineStr">
-        <is>
-          <t>COCINA-01_A4 Vitrina 570_Estante 2</t>
-        </is>
-      </c>
-      <c r="Y113" t="inlineStr">
-        <is>
-          <t>9992609291129</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>113</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
-        </is>
-      </c>
-      <c r="D114" t="n">
-        <v>1</v>
-      </c>
-      <c r="E114" t="n">
-        <v>99</v>
-      </c>
-      <c r="F114" t="n">
-        <v>1407</v>
-      </c>
-      <c r="G114" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="H114" t="n">
-        <v>18</v>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>18_Melamina_VERDE 18</t>
-        </is>
-      </c>
-      <c r="J114" t="n">
-        <v>98</v>
-      </c>
-      <c r="K114" t="n">
-        <v>1407</v>
-      </c>
-      <c r="L114" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="M114" t="n">
-        <v>18</v>
-      </c>
-      <c r="N114" t="inlineStr">
-        <is>
-          <t>9992609291136</t>
-        </is>
-      </c>
-      <c r="O114" t="inlineStr"/>
-      <c r="P114" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q114" t="n">
-        <v>0</v>
-      </c>
-      <c r="R114" t="n">
-        <v>0</v>
-      </c>
-      <c r="S114" t="n">
-        <v>0</v>
-      </c>
-      <c r="T114" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U114" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V114" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W114" t="inlineStr"/>
-      <c r="X114" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
-        </is>
-      </c>
-      <c r="Y114" t="inlineStr">
-        <is>
-          <t>9992609291136</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>114</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
-        <v>1</v>
-      </c>
-      <c r="E115" t="n">
-        <v>99</v>
-      </c>
-      <c r="F115" t="n">
-        <v>367.7</v>
-      </c>
-      <c r="G115" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H115" t="n">
-        <v>18</v>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>18_Melamina_VERDE 18</t>
-        </is>
-      </c>
-      <c r="J115" t="n">
-        <v>98</v>
-      </c>
-      <c r="K115" t="n">
-        <v>367.7</v>
-      </c>
-      <c r="L115" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M115" t="n">
-        <v>18</v>
-      </c>
-      <c r="N115" t="inlineStr">
-        <is>
-          <t>9992609291143</t>
-        </is>
-      </c>
-      <c r="O115" t="inlineStr"/>
-      <c r="P115" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q115" t="n">
-        <v>0</v>
-      </c>
-      <c r="R115" t="n">
-        <v>0</v>
-      </c>
-      <c r="S115" t="n">
-        <v>0</v>
-      </c>
-      <c r="T115" t="inlineStr">
-        <is>
-          <t>竖纹</t>
-        </is>
-      </c>
-      <c r="U115" t="inlineStr">
-        <is>
-          <t>COCINA-01</t>
-        </is>
-      </c>
-      <c r="V115" t="inlineStr">
-        <is>
-          <t>PRUEBA</t>
-        </is>
-      </c>
-      <c r="W115" t="inlineStr"/>
-      <c r="X115" t="inlineStr">
-        <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
-        </is>
-      </c>
-      <c r="Y115" t="inlineStr">
-        <is>
-          <t>9992609291143</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A4 campana oculta: frente fijo + frente movil sobre el visor, linea pareja a 1450; 108/108
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y107"/>
+  <dimension ref="A1:Y109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9949,42 +9949,42 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Campana 570_Estante 1</t>
+          <t>COCINA-01_A4 Campana 570_Frente campana fijo</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Campana 570_Estante 1</t>
+          <t>COCINA-01_A4 Campana 570_Frente campana fijo</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>1</v>
       </c>
       <c r="E105" t="n">
-        <v>281</v>
+        <v>149.5</v>
       </c>
       <c r="F105" t="n">
-        <v>532</v>
+        <v>567</v>
       </c>
       <c r="G105" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="H105" t="n">
         <v>18</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>18_Melamina_BLANCO 18</t>
+          <t>18_Melamina_VERDE 18</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>280</v>
+        <v>147.5</v>
       </c>
       <c r="K105" t="n">
-        <v>532</v>
+        <v>565</v>
       </c>
       <c r="L105" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="M105" t="n">
         <v>18</v>
@@ -9996,16 +9996,16 @@
       </c>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q105" t="n">
         <v>1</v>
       </c>
       <c r="R105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T105" t="inlineStr">
         <is>
@@ -10025,7 +10025,7 @@
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr">
         <is>
-          <t>COCINA-01_A4 Campana 570_Estante 1</t>
+          <t>COCINA-01_A4 Campana 570_Frente campana fijo</t>
         </is>
       </c>
       <c r="Y105" t="inlineStr">
@@ -10040,25 +10040,25 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Campana 570_Frente campana visor</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Campana 570_Frente campana visor</t>
         </is>
       </c>
       <c r="D106" t="n">
         <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>99</v>
+        <v>188.5</v>
       </c>
       <c r="F106" t="n">
-        <v>1407</v>
+        <v>567</v>
       </c>
       <c r="G106" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="H106" t="n">
         <v>18</v>
@@ -10069,13 +10069,13 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>98</v>
+        <v>186.5</v>
       </c>
       <c r="K106" t="n">
-        <v>1407</v>
+        <v>565</v>
       </c>
       <c r="L106" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="M106" t="n">
         <v>18</v>
@@ -10090,13 +10090,13 @@
         <v>1</v>
       </c>
       <c r="Q106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T106" t="inlineStr">
         <is>
@@ -10116,7 +10116,7 @@
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+          <t>COCINA-01_A4 Campana 570_Frente campana visor</t>
         </is>
       </c>
       <c r="Y106" t="inlineStr">
@@ -10131,42 +10131,42 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_A4 Campana 570_Estante 1</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+          <t>COCINA-01_A4 Campana 570_Estante 1</t>
         </is>
       </c>
       <c r="D107" t="n">
         <v>1</v>
       </c>
       <c r="E107" t="n">
-        <v>99</v>
+        <v>281</v>
       </c>
       <c r="F107" t="n">
-        <v>367.7</v>
+        <v>532</v>
       </c>
       <c r="G107" t="n">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="H107" t="n">
         <v>18</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>18_Melamina_VERDE 18</t>
+          <t>18_Melamina_BLANCO 18</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>98</v>
+        <v>280</v>
       </c>
       <c r="K107" t="n">
-        <v>367.7</v>
+        <v>532</v>
       </c>
       <c r="L107" t="n">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="M107" t="n">
         <v>18</v>
@@ -10178,10 +10178,10 @@
       </c>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R107" t="n">
         <v>0</v>
@@ -10207,12 +10207,194 @@
       <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr">
         <is>
+          <t>COCINA-01_A4 Campana 570_Estante 1</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>9992609291068</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" t="n">
+        <v>99</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1407</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H108" t="n">
+        <v>18</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>98</v>
+      </c>
+      <c r="K108" t="n">
+        <v>1407</v>
+      </c>
+      <c r="L108" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="M108" t="n">
+        <v>18</v>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>9992609291075</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr"/>
+      <c r="P108" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0</v>
+      </c>
+      <c r="S108" t="n">
+        <v>0</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr"/>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo largo</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>9992609291075</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
           <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
         </is>
       </c>
-      <c r="Y107" t="inlineStr">
-        <is>
-          <t>9992609291068</t>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" t="n">
+        <v>99</v>
+      </c>
+      <c r="F109" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H109" t="n">
+        <v>18</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>18_Melamina_VERDE 18</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>98</v>
+      </c>
+      <c r="K109" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M109" t="n">
+        <v>18</v>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>9992609291082</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr"/>
+      <c r="P109" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
+        <v>0</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>竖纹</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>COCINA-01</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>PRUEBA</t>
+        </is>
+      </c>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>COCINA-01_Z Zocalos_Zocalo diagonal</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>9992609291082</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Columna del rincón 60x180: esquineros con el rincón recortado, fondos/travesaños después de la columna, mesada recortada; ArmarReceta chanfle + escotadura; 108/108
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -955,10 +955,10 @@
         <v>734</v>
       </c>
       <c r="F6" t="n">
-        <v>755</v>
+        <v>722</v>
       </c>
       <c r="G6" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="H6" t="n">
         <v>5</v>
@@ -972,10 +972,10 @@
         <v>734</v>
       </c>
       <c r="K6" t="n">
-        <v>755</v>
+        <v>722</v>
       </c>
       <c r="L6" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="M6" t="n">
         <v>5</v>
@@ -1046,10 +1046,10 @@
         <v>734</v>
       </c>
       <c r="F7" t="n">
-        <v>762</v>
+        <v>602</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.44</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
@@ -1063,10 +1063,10 @@
         <v>734</v>
       </c>
       <c r="K7" t="n">
-        <v>762</v>
+        <v>602</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.44</v>
       </c>
       <c r="M7" t="n">
         <v>5</v>
@@ -6233,10 +6233,10 @@
         <v>689</v>
       </c>
       <c r="F64" t="n">
-        <v>755</v>
+        <v>722</v>
       </c>
       <c r="G64" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="H64" t="n">
         <v>5</v>
@@ -6250,10 +6250,10 @@
         <v>689</v>
       </c>
       <c r="K64" t="n">
-        <v>755</v>
+        <v>722</v>
       </c>
       <c r="L64" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="M64" t="n">
         <v>5</v>
@@ -6324,10 +6324,10 @@
         <v>974</v>
       </c>
       <c r="F65" t="n">
-        <v>762</v>
+        <v>602</v>
       </c>
       <c r="G65" t="n">
-        <v>0.74</v>
+        <v>0.59</v>
       </c>
       <c r="H65" t="n">
         <v>5</v>
@@ -6341,10 +6341,10 @@
         <v>974</v>
       </c>
       <c r="K65" t="n">
-        <v>762</v>
+        <v>602</v>
       </c>
       <c r="L65" t="n">
-        <v>0.74</v>
+        <v>0.59</v>
       </c>
       <c r="M65" t="n">
         <v>5</v>
@@ -7143,7 +7143,7 @@
         <v>80</v>
       </c>
       <c r="F74" t="n">
-        <v>751</v>
+        <v>717</v>
       </c>
       <c r="G74" t="n">
         <v>0.06</v>
@@ -7160,7 +7160,7 @@
         <v>80</v>
       </c>
       <c r="K74" t="n">
-        <v>751</v>
+        <v>717</v>
       </c>
       <c r="L74" t="n">
         <v>0.06</v>
@@ -7234,7 +7234,7 @@
         <v>80</v>
       </c>
       <c r="F75" t="n">
-        <v>638</v>
+        <v>597</v>
       </c>
       <c r="G75" t="n">
         <v>0.05</v>
@@ -7251,7 +7251,7 @@
         <v>80</v>
       </c>
       <c r="K75" t="n">
-        <v>638</v>
+        <v>597</v>
       </c>
       <c r="L75" t="n">
         <v>0.05</v>

</xml_diff>

<commit_message>
Cajonera 450 y módulo tacho 322 (B3/B4); 108/108; paquete regenerado
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4LkomGUWbJQWvHEkfxx2P
</commit_message>
<xml_diff>
--- a/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
+++ b/fusion/EXPORT_COCINA-01/salida/lista_corte.xlsx
@@ -2305,12 +2305,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Lateral der</t>
+          <t>COCINA-01_B3 Cajonera 450_Lateral der</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Lateral der</t>
+          <t>COCINA-01_B3 Cajonera 450_Lateral der</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -2381,7 +2381,7 @@
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Lateral der</t>
+          <t>COCINA-01_B3 Cajonera 450_Lateral der</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Lateral izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Lateral izq</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Lateral izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Lateral izq</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -2472,7 +2472,7 @@
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Lateral izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Lateral izq</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -2487,12 +2487,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Piso</t>
+          <t>COCINA-01_B3 Cajonera 450_Piso</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Piso</t>
+          <t>COCINA-01_B3 Cajonera 450_Piso</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2502,10 +2502,10 @@
         <v>580</v>
       </c>
       <c r="F23" t="n">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="G23" t="n">
-        <v>0.16</v>
+        <v>0.24</v>
       </c>
       <c r="H23" t="n">
         <v>18</v>
@@ -2519,10 +2519,10 @@
         <v>579</v>
       </c>
       <c r="K23" t="n">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="L23" t="n">
-        <v>0.16</v>
+        <v>0.24</v>
       </c>
       <c r="M23" t="n">
         <v>18</v>
@@ -2563,7 +2563,7 @@
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Piso</t>
+          <t>COCINA-01_B3 Cajonera 450_Piso</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Travesano delantero</t>
+          <t>COCINA-01_B3 Cajonera 450_Travesano delantero</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Travesano delantero</t>
+          <t>COCINA-01_B3 Cajonera 450_Travesano delantero</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2593,10 +2593,10 @@
         <v>100</v>
       </c>
       <c r="F24" t="n">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="G24" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="H24" t="n">
         <v>18</v>
@@ -2610,10 +2610,10 @@
         <v>99</v>
       </c>
       <c r="K24" t="n">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="L24" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="M24" t="n">
         <v>18</v>
@@ -2654,7 +2654,7 @@
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Travesano delantero</t>
+          <t>COCINA-01_B3 Cajonera 450_Travesano delantero</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Travesano trasero</t>
+          <t>COCINA-01_B3 Cajonera 450_Travesano trasero</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Travesano trasero</t>
+          <t>COCINA-01_B3 Cajonera 450_Travesano trasero</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -2684,10 +2684,10 @@
         <v>100</v>
       </c>
       <c r="F25" t="n">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="G25" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="H25" t="n">
         <v>18</v>
@@ -2701,10 +2701,10 @@
         <v>100</v>
       </c>
       <c r="K25" t="n">
-        <v>284</v>
+        <v>414</v>
       </c>
       <c r="L25" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="M25" t="n">
         <v>18</v>
@@ -2745,7 +2745,7 @@
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Travesano trasero</t>
+          <t>COCINA-01_B3 Cajonera 450_Travesano trasero</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -2760,12 +2760,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Fondo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Fondo</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2775,10 +2775,10 @@
         <v>746</v>
       </c>
       <c r="F26" t="n">
-        <v>294</v>
+        <v>424</v>
       </c>
       <c r="G26" t="n">
-        <v>0.22</v>
+        <v>0.32</v>
       </c>
       <c r="H26" t="n">
         <v>5</v>
@@ -2792,10 +2792,10 @@
         <v>746</v>
       </c>
       <c r="K26" t="n">
-        <v>294</v>
+        <v>424</v>
       </c>
       <c r="L26" t="n">
-        <v>0.22</v>
+        <v>0.32</v>
       </c>
       <c r="M26" t="n">
         <v>5</v>
@@ -2836,7 +2836,7 @@
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Fondo</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -2851,12 +2851,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 1</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 1</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 1</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -2866,10 +2866,10 @@
         <v>187</v>
       </c>
       <c r="F27" t="n">
-        <v>317</v>
+        <v>447</v>
       </c>
       <c r="G27" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="H27" t="n">
         <v>18</v>
@@ -2883,10 +2883,10 @@
         <v>185</v>
       </c>
       <c r="K27" t="n">
-        <v>315</v>
+        <v>445</v>
       </c>
       <c r="L27" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="M27" t="n">
         <v>18</v>
@@ -2927,7 +2927,7 @@
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 1</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 1</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
@@ -2942,12 +2942,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 frente</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 frente</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2957,10 +2957,10 @@
         <v>120</v>
       </c>
       <c r="F28" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G28" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H28" t="n">
         <v>18</v>
@@ -2974,10 +2974,10 @@
         <v>119</v>
       </c>
       <c r="K28" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L28" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M28" t="n">
         <v>18</v>
@@ -3018,7 +3018,7 @@
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 frente</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
@@ -3033,12 +3033,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 contrafrente</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 contrafrente</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -3048,10 +3048,10 @@
         <v>120</v>
       </c>
       <c r="F29" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G29" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H29" t="n">
         <v>18</v>
@@ -3065,10 +3065,10 @@
         <v>119</v>
       </c>
       <c r="K29" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L29" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M29" t="n">
         <v>18</v>
@@ -3109,7 +3109,7 @@
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 contrafrente</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -3124,12 +3124,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 costado der</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 costado der</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -3200,7 +3200,7 @@
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 costado der</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -3215,12 +3215,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 costado izq</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 costado izq</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -3291,7 +3291,7 @@
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 costado izq</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -3306,12 +3306,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 fondo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 fondo</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3321,10 +3321,10 @@
         <v>423</v>
       </c>
       <c r="F32" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="G32" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H32" t="n">
         <v>5</v>
@@ -3338,10 +3338,10 @@
         <v>423</v>
       </c>
       <c r="K32" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="L32" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="M32" t="n">
         <v>5</v>
@@ -3382,7 +3382,7 @@
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 1 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 1 fondo</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
@@ -3397,12 +3397,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 2</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 2</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 2</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -3412,10 +3412,10 @@
         <v>187</v>
       </c>
       <c r="F33" t="n">
-        <v>317</v>
+        <v>447</v>
       </c>
       <c r="G33" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="H33" t="n">
         <v>18</v>
@@ -3429,10 +3429,10 @@
         <v>185</v>
       </c>
       <c r="K33" t="n">
-        <v>315</v>
+        <v>445</v>
       </c>
       <c r="L33" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="M33" t="n">
         <v>18</v>
@@ -3473,7 +3473,7 @@
       <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 2</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 2</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -3488,12 +3488,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 frente</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 frente</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -3503,10 +3503,10 @@
         <v>120</v>
       </c>
       <c r="F34" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G34" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H34" t="n">
         <v>18</v>
@@ -3520,10 +3520,10 @@
         <v>119</v>
       </c>
       <c r="K34" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L34" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M34" t="n">
         <v>18</v>
@@ -3564,7 +3564,7 @@
       <c r="W34" t="inlineStr"/>
       <c r="X34" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 frente</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -3579,12 +3579,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 contrafrente</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 contrafrente</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -3594,10 +3594,10 @@
         <v>120</v>
       </c>
       <c r="F35" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G35" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H35" t="n">
         <v>18</v>
@@ -3611,10 +3611,10 @@
         <v>119</v>
       </c>
       <c r="K35" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L35" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M35" t="n">
         <v>18</v>
@@ -3655,7 +3655,7 @@
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 contrafrente</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -3670,12 +3670,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 costado der</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 costado der</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -3746,7 +3746,7 @@
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 costado der</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -3761,12 +3761,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 costado izq</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 costado izq</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -3837,7 +3837,7 @@
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 costado izq</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -3852,12 +3852,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 fondo</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 fondo</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -3867,10 +3867,10 @@
         <v>423</v>
       </c>
       <c r="F38" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="G38" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H38" t="n">
         <v>5</v>
@@ -3884,10 +3884,10 @@
         <v>423</v>
       </c>
       <c r="K38" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="L38" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="M38" t="n">
         <v>5</v>
@@ -3928,7 +3928,7 @@
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 2 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 2 fondo</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -3943,12 +3943,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 3</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 3</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 3</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -3958,10 +3958,10 @@
         <v>187</v>
       </c>
       <c r="F39" t="n">
-        <v>317</v>
+        <v>447</v>
       </c>
       <c r="G39" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="H39" t="n">
         <v>18</v>
@@ -3975,10 +3975,10 @@
         <v>185</v>
       </c>
       <c r="K39" t="n">
-        <v>315</v>
+        <v>445</v>
       </c>
       <c r="L39" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="M39" t="n">
         <v>18</v>
@@ -4019,7 +4019,7 @@
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 3</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 3</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -4034,12 +4034,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 frente</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 frente</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -4049,10 +4049,10 @@
         <v>120</v>
       </c>
       <c r="F40" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G40" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H40" t="n">
         <v>18</v>
@@ -4066,10 +4066,10 @@
         <v>119</v>
       </c>
       <c r="K40" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L40" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M40" t="n">
         <v>18</v>
@@ -4110,7 +4110,7 @@
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 frente</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -4125,12 +4125,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 contrafrente</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 contrafrente</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -4140,10 +4140,10 @@
         <v>120</v>
       </c>
       <c r="F41" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G41" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H41" t="n">
         <v>18</v>
@@ -4157,10 +4157,10 @@
         <v>119</v>
       </c>
       <c r="K41" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L41" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M41" t="n">
         <v>18</v>
@@ -4201,7 +4201,7 @@
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 contrafrente</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4216,12 +4216,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 costado der</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 costado der</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -4292,7 +4292,7 @@
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 costado der</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
@@ -4307,12 +4307,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 costado izq</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 costado izq</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -4383,7 +4383,7 @@
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 costado izq</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
@@ -4398,12 +4398,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 fondo</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 fondo</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -4413,10 +4413,10 @@
         <v>423</v>
       </c>
       <c r="F44" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="G44" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H44" t="n">
         <v>5</v>
@@ -4430,10 +4430,10 @@
         <v>423</v>
       </c>
       <c r="K44" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="L44" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="M44" t="n">
         <v>5</v>
@@ -4474,7 +4474,7 @@
       <c r="W44" t="inlineStr"/>
       <c r="X44" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 3 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 3 fondo</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
@@ -4489,12 +4489,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 4</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 4</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 4</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 4</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -4504,10 +4504,10 @@
         <v>187</v>
       </c>
       <c r="F45" t="n">
-        <v>317</v>
+        <v>447</v>
       </c>
       <c r="G45" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="H45" t="n">
         <v>18</v>
@@ -4521,10 +4521,10 @@
         <v>185</v>
       </c>
       <c r="K45" t="n">
-        <v>315</v>
+        <v>445</v>
       </c>
       <c r="L45" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="M45" t="n">
         <v>18</v>
@@ -4565,7 +4565,7 @@
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Frente cajon 4</t>
+          <t>COCINA-01_B3 Cajonera 450_Frente cajon 4</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
@@ -4580,12 +4580,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 frente</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 frente</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -4595,10 +4595,10 @@
         <v>120</v>
       </c>
       <c r="F46" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G46" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H46" t="n">
         <v>18</v>
@@ -4612,10 +4612,10 @@
         <v>119</v>
       </c>
       <c r="K46" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L46" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M46" t="n">
         <v>18</v>
@@ -4656,7 +4656,7 @@
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 frente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 frente</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
@@ -4671,12 +4671,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 contrafrente</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 contrafrente</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -4686,10 +4686,10 @@
         <v>120</v>
       </c>
       <c r="F47" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="G47" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="H47" t="n">
         <v>18</v>
@@ -4703,10 +4703,10 @@
         <v>119</v>
       </c>
       <c r="K47" t="n">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="L47" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M47" t="n">
         <v>18</v>
@@ -4747,7 +4747,7 @@
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 contrafrente</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 contrafrente</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
@@ -4762,12 +4762,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 costado der</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 costado der</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -4838,7 +4838,7 @@
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 costado der</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 costado der</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr">
@@ -4853,12 +4853,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 costado izq</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 costado izq</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -4929,7 +4929,7 @@
       <c r="W49" t="inlineStr"/>
       <c r="X49" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 costado izq</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 costado izq</t>
         </is>
       </c>
       <c r="Y49" t="inlineStr">
@@ -4944,12 +4944,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 fondo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 fondo</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -4959,10 +4959,10 @@
         <v>423</v>
       </c>
       <c r="F50" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H50" t="n">
         <v>5</v>
@@ -4976,10 +4976,10 @@
         <v>423</v>
       </c>
       <c r="K50" t="n">
-        <v>231</v>
+        <v>361</v>
       </c>
       <c r="L50" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="M50" t="n">
         <v>5</v>
@@ -5020,7 +5020,7 @@
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr">
         <is>
-          <t>COCINA-01_B3 Cajonera 320_Cajon 4 fondo</t>
+          <t>COCINA-01_B3 Cajonera 450_Cajon 4 fondo</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Lateral der</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Lateral der</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Lateral der</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Lateral der</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -5111,7 +5111,7 @@
       <c r="W51" t="inlineStr"/>
       <c r="X51" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Lateral der</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Lateral der</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
@@ -5126,12 +5126,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Lateral izq</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Lateral izq</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Lateral izq</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Lateral izq</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -5202,7 +5202,7 @@
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Lateral izq</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Lateral izq</t>
         </is>
       </c>
       <c r="Y52" t="inlineStr">
@@ -5217,12 +5217,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Piso</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Piso</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Piso</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Piso</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -5232,10 +5232,10 @@
         <v>580</v>
       </c>
       <c r="F53" t="n">
-        <v>416</v>
+        <v>286</v>
       </c>
       <c r="G53" t="n">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="H53" t="n">
         <v>18</v>
@@ -5249,10 +5249,10 @@
         <v>579</v>
       </c>
       <c r="K53" t="n">
-        <v>416</v>
+        <v>286</v>
       </c>
       <c r="L53" t="n">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="M53" t="n">
         <v>18</v>
@@ -5293,7 +5293,7 @@
       <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Piso</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Piso</t>
         </is>
       </c>
       <c r="Y53" t="inlineStr">
@@ -5308,12 +5308,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Travesano delantero</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Travesano delantero</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Travesano delantero</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Travesano delantero</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -5323,10 +5323,10 @@
         <v>100</v>
       </c>
       <c r="F54" t="n">
-        <v>416</v>
+        <v>286</v>
       </c>
       <c r="G54" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="H54" t="n">
         <v>18</v>
@@ -5340,10 +5340,10 @@
         <v>99</v>
       </c>
       <c r="K54" t="n">
-        <v>416</v>
+        <v>286</v>
       </c>
       <c r="L54" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="M54" t="n">
         <v>18</v>
@@ -5384,7 +5384,7 @@
       <c r="W54" t="inlineStr"/>
       <c r="X54" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Travesano delantero</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Travesano delantero</t>
         </is>
       </c>
       <c r="Y54" t="inlineStr">
@@ -5399,12 +5399,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Travesano trasero</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Travesano trasero</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Travesano trasero</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Travesano trasero</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -5414,10 +5414,10 @@
         <v>100</v>
       </c>
       <c r="F55" t="n">
-        <v>416</v>
+        <v>286</v>
       </c>
       <c r="G55" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="H55" t="n">
         <v>18</v>
@@ -5431,10 +5431,10 @@
         <v>100</v>
       </c>
       <c r="K55" t="n">
-        <v>416</v>
+        <v>286</v>
       </c>
       <c r="L55" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="M55" t="n">
         <v>18</v>
@@ -5475,7 +5475,7 @@
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Travesano trasero</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Travesano trasero</t>
         </is>
       </c>
       <c r="Y55" t="inlineStr">
@@ -5490,12 +5490,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Fondo</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Fondo</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Fondo</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Fondo</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -5505,10 +5505,10 @@
         <v>746</v>
       </c>
       <c r="F56" t="n">
-        <v>426</v>
+        <v>296</v>
       </c>
       <c r="G56" t="n">
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="H56" t="n">
         <v>5</v>
@@ -5522,10 +5522,10 @@
         <v>746</v>
       </c>
       <c r="K56" t="n">
-        <v>426</v>
+        <v>296</v>
       </c>
       <c r="L56" t="n">
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="M56" t="n">
         <v>5</v>
@@ -5566,7 +5566,7 @@
       <c r="W56" t="inlineStr"/>
       <c r="X56" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Fondo</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Fondo</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr">
@@ -5581,12 +5581,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Puerta</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Puerta</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Puerta</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Puerta</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -5596,10 +5596,10 @@
         <v>757</v>
       </c>
       <c r="F57" t="n">
-        <v>449</v>
+        <v>319</v>
       </c>
       <c r="G57" t="n">
-        <v>0.34</v>
+        <v>0.24</v>
       </c>
       <c r="H57" t="n">
         <v>18</v>
@@ -5613,10 +5613,10 @@
         <v>755</v>
       </c>
       <c r="K57" t="n">
-        <v>447</v>
+        <v>317</v>
       </c>
       <c r="L57" t="n">
-        <v>0.34</v>
+        <v>0.24</v>
       </c>
       <c r="M57" t="n">
         <v>18</v>
@@ -5657,7 +5657,7 @@
       <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr">
         <is>
-          <t>COCINA-01_B4 Bajo puerta 452_Puerta</t>
+          <t>COCINA-01_B4 Bajo tacho 322_Puerta</t>
         </is>
       </c>
       <c r="Y57" t="inlineStr">

</xml_diff>